<commit_message>
Günlük kur verisi: 01.09.2026 11:21
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -5427,7 +5427,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -5449,7 +5449,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -5471,7 +5471,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -5493,7 +5493,7 @@
       <row>28</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -5515,7 +5515,7 @@
       <row>28</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="5" name="Chart 5"/>
@@ -5537,7 +5537,7 @@
       <row>28</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="6" name="Chart 6"/>
@@ -5559,7 +5559,7 @@
       <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="7" name="Chart 7"/>
@@ -5581,7 +5581,7 @@
       <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="8" name="Chart 8"/>
@@ -5603,7 +5603,7 @@
       <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="9" name="Chart 9"/>
@@ -5625,7 +5625,7 @@
       <row>80</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="10" name="Chart 10"/>
@@ -5647,7 +5647,7 @@
       <row>80</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="11" name="Chart 11"/>
@@ -5669,7 +5669,7 @@
       <row>80</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="12" name="Chart 12"/>
@@ -5691,7 +5691,7 @@
       <row>106</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="13" name="Chart 13"/>
@@ -5713,7 +5713,7 @@
       <row>106</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="14" name="Chart 14"/>
@@ -5735,7 +5735,7 @@
       <row>106</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="15" name="Chart 15"/>
@@ -5757,7 +5757,7 @@
       <row>132</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="16" name="Chart 16"/>
@@ -5779,7 +5779,7 @@
       <row>132</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="17" name="Chart 17"/>
@@ -5801,7 +5801,7 @@
       <row>132</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="2880000"/>
+    <ext cx="6840000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="18" name="Chart 18"/>

</xml_diff>

<commit_message>
Günlük kur verisi: 01.09.2026 11:24
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -5427,7 +5427,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -5449,7 +5449,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -5471,7 +5471,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -5493,7 +5493,7 @@
       <row>28</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -5515,7 +5515,7 @@
       <row>28</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="5" name="Chart 5"/>
@@ -5537,7 +5537,7 @@
       <row>28</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="6" name="Chart 6"/>
@@ -5559,7 +5559,7 @@
       <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="7" name="Chart 7"/>
@@ -5581,7 +5581,7 @@
       <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="8" name="Chart 8"/>
@@ -5603,7 +5603,7 @@
       <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="9" name="Chart 9"/>
@@ -5625,7 +5625,7 @@
       <row>80</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="10" name="Chart 10"/>
@@ -5647,7 +5647,7 @@
       <row>80</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="11" name="Chart 11"/>
@@ -5669,7 +5669,7 @@
       <row>80</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="12" name="Chart 12"/>
@@ -5691,7 +5691,7 @@
       <row>106</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="13" name="Chart 13"/>
@@ -5713,7 +5713,7 @@
       <row>106</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="14" name="Chart 14"/>
@@ -5735,7 +5735,7 @@
       <row>106</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="15" name="Chart 15"/>
@@ -5757,7 +5757,7 @@
       <row>132</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="16" name="Chart 16"/>
@@ -5779,7 +5779,7 @@
       <row>132</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="17" name="Chart 17"/>
@@ -5801,7 +5801,7 @@
       <row>132</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6840000" cy="3240000"/>
+    <ext cx="6840000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="18" name="Chart 18"/>

</xml_diff>

<commit_message>
Günlük kur verisi: 02.09.2026 11:05
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -7210,7 +7210,7 @@
         <v>46267</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
@@ -7230,28 +7230,28 @@
         <v>0.02842045430622513</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>54.9918</v>
+        <v>55.0015</v>
       </c>
       <c r="I2" s="10" t="n">
-        <v>56.5547</v>
+        <v>56.5696</v>
       </c>
       <c r="J2" s="10" t="n">
-        <v>1.5629</v>
+        <v>1.5681</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>0.02842060088958717</v>
+        <v>0.02851013154186704</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>6532.97</v>
+        <v>6536.54</v>
       </c>
       <c r="M2" s="12" t="n">
-        <v>6769.14</v>
+        <v>6772.6</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>236.17</v>
+        <v>236.06</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>0.03615047979709076</v>
+        <v>0.03611390735771524</v>
       </c>
     </row>
     <row r="3">
@@ -7259,7 +7259,7 @@
         <v>46267</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
@@ -7279,28 +7279,28 @@
         <v>0.01630582291166461</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>55.445</v>
+        <v>55.459</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>56.355</v>
+        <v>56.374</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.91</v>
+        <v>0.915</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>0.0164126611957796</v>
+        <v>0.01649867469662273</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>6607.29</v>
+        <v>6614.61</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>6743.19</v>
+        <v>6750.58</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>135.9</v>
+        <v>135.97</v>
       </c>
       <c r="O3" s="13" t="n">
-        <v>0.02056819058948525</v>
+        <v>0.02055601161670907</v>
       </c>
     </row>
     <row r="4">
@@ -7308,7 +7308,7 @@
         <v>46267</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -7316,40 +7316,40 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>48.079</v>
+        <v>48.083</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>48.375</v>
+        <v>48.373</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.296</v>
+        <v>0.29</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>0.006156534037729569</v>
+        <v>0.006031237651560843</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>55.49</v>
+        <v>55.501</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>56.006</v>
+        <v>56.009</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.516</v>
+        <v>0.508</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>0.009298972787889709</v>
+        <v>0.009152988234446227</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>6673.09</v>
+        <v>6675.22</v>
       </c>
       <c r="M4" s="12" t="n">
-        <v>6740.67</v>
+        <v>6742.94</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>67.58</v>
+        <v>67.72</v>
       </c>
       <c r="O4" s="13" t="n">
-        <v>0.01012724240194573</v>
+        <v>0.01014498398554654</v>
       </c>
     </row>
     <row r="5">
@@ -7357,7 +7357,7 @@
         <v>46267</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -7365,40 +7365,40 @@
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>48.122</v>
+        <v>48.13</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>48.352</v>
+        <v>48.34</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>0.004779518723245085</v>
+        <v>0.004363183045917307</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>55.594</v>
+        <v>55.625</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>55.972</v>
+        <v>55.98</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.378</v>
+        <v>0.355</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>0.006799294887937547</v>
+        <v>0.006382022471910113</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>6581.32</v>
+        <v>6588.87</v>
       </c>
       <c r="M5" s="12" t="n">
         <v>6775</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>193.68</v>
+        <v>186.13</v>
       </c>
       <c r="O5" s="13" t="n">
-        <v>0.02942874681674801</v>
+        <v>0.02824915349673009</v>
       </c>
     </row>
     <row r="6">
@@ -7406,7 +7406,7 @@
         <v>46267</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
@@ -7414,40 +7414,40 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>47.4529</v>
+        <v>47.4531</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>48.7293</v>
+        <v>48.7294</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>1.2764</v>
+        <v>1.2763</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.02689825068647016</v>
+        <v>0.02689602997485939</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>55.0337</v>
+        <v>55.0539</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>56.3992</v>
+        <v>56.4187</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>1.3655</v>
+        <v>1.3648</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0.0248120696954775</v>
+        <v>0.02479025100855707</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>6593.7</v>
+        <v>6601.93</v>
       </c>
       <c r="M6" s="12" t="n">
-        <v>6744.8</v>
+        <v>6752.76</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>151.1</v>
+        <v>150.83</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>0.02291581357962904</v>
+        <v>0.02284634947659245</v>
       </c>
     </row>
     <row r="7">
@@ -7455,7 +7455,7 @@
         <v>46267</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
@@ -7475,28 +7475,28 @@
         <v>0.04065367214916916</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>54.753</v>
+        <v>54.776</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>56.987</v>
+        <v>57.007</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>2.234</v>
+        <v>2.231</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>0.04080141727393933</v>
+        <v>0.0407295165766029</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>6591.68</v>
+        <v>6598.78</v>
       </c>
       <c r="M7" s="12" t="n">
-        <v>6785.81</v>
+        <v>6793</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>194.13</v>
+        <v>194.22</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>0.02945076217292102</v>
+        <v>0.02943271331973486</v>
       </c>
     </row>
     <row r="8">
@@ -7504,7 +7504,7 @@
         <v>46267</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
@@ -7512,40 +7512,40 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>47.555</v>
+        <v>47.5548</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>48.9551</v>
+        <v>48.9549</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>1.4001</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>0.02944169908526969</v>
+        <v>0.02944182290746675</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>55.049</v>
+        <v>55.068</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>56.6746</v>
+        <v>56.6893</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>1.6256</v>
+        <v>1.6213</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>0.02953005504187179</v>
+        <v>0.02944178107067625</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>6607.51</v>
+        <v>6612.92</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>6803.13</v>
+        <v>6808.61</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>195.62</v>
+        <v>195.69</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>0.02960570623426979</v>
+        <v>0.02959207127864846</v>
       </c>
     </row>
     <row r="9">
@@ -7553,7 +7553,7 @@
         <v>46267</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -7561,40 +7561,40 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>48.2244</v>
+        <v>48.2243</v>
       </c>
       <c r="E9" s="8" t="n">
         <v>48.2813</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.0569</v>
+        <v>0.057</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.001179900631215733</v>
+        <v>0.001181976721279521</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>55.8136</v>
+        <v>55.8328</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>55.8969</v>
+        <v>55.9159</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.0833</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>0.001492467785629309</v>
+        <v>0.001488372426244071</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6660.19</v>
+        <v>6666.72</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>6689.09</v>
+        <v>6695.46</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>28.9</v>
+        <v>28.74</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>0.00433921554790479</v>
+        <v>0.004310965512275901</v>
       </c>
     </row>
     <row r="10">
@@ -7602,7 +7602,7 @@
         <v>46267</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -7610,40 +7610,40 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>48.238</v>
+        <v>48.2379</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>48.2763</v>
+        <v>48.2761</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.0383</v>
+        <v>0.0382</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.0007939798499108587</v>
+        <v>0.0007919084371417495</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>55.7909</v>
+        <v>55.8102</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>55.9004</v>
+        <v>55.924</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.1095</v>
+        <v>0.1138</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>0.001962685670960676</v>
+        <v>0.002039053793034248</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>6656.67</v>
+        <v>6664.59</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>6688.4</v>
+        <v>6696.21</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>31.73</v>
+        <v>31.62</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>0.004766647588058293</v>
+        <v>0.004744477904867366</v>
       </c>
     </row>
     <row r="11">
@@ -7651,7 +7651,7 @@
         <v>46267</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
@@ -7662,37 +7662,37 @@
         <v>47.9241</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>49.1615</v>
+        <v>49.1617</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1.2374</v>
+        <v>1.2376</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.02581999453302201</v>
+        <v>0.02582416779866497</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>55.3834</v>
+        <v>55.3879</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>56.6615</v>
+        <v>56.6664</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>1.2781</v>
+        <v>1.2785</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>0.0230773119743461</v>
+        <v>0.02308265884787111</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6610.38</v>
+        <v>6612.91</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>6718.58</v>
+        <v>6721.13</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>108.2</v>
+        <v>108.22</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>0.01636819668460815</v>
+        <v>0.01636495884565191</v>
       </c>
     </row>
     <row r="12">
@@ -7700,7 +7700,7 @@
         <v>46267</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
@@ -7720,28 +7720,28 @@
         <v>0.01776477349913789</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>55.3004</v>
+        <v>55.3243</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>56.4617</v>
+        <v>56.4812</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>1.1613</v>
+        <v>1.1569</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>0.02099984810236454</v>
+        <v>0.02091124514905747</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>6605.45</v>
+        <v>6613.01</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>6759.84</v>
+        <v>6767.11</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>154.39</v>
+        <v>154.1</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>0.02337312370845287</v>
+        <v>0.02330255057832969</v>
       </c>
     </row>
     <row r="13">
@@ -7749,7 +7749,7 @@
         <v>46267</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
@@ -7757,40 +7757,40 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>47.998</v>
+        <v>47.9983</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>48.605</v>
+        <v>48.6051</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.607</v>
+        <v>0.6068</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.01264636026501104</v>
+        <v>0.01264211440821863</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>55.5757</v>
+        <v>55.595</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>56.2369</v>
+        <v>56.2555</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>0.6612</v>
+        <v>0.6605</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>0.01189728604408042</v>
+        <v>0.01188056479899271</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6677.86</v>
+        <v>6683.49</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>6732.18</v>
+        <v>6737.85</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>54.32</v>
+        <v>54.36</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>0.008134342439044843</v>
+        <v>0.008133475175394891</v>
       </c>
     </row>
     <row r="14">
@@ -7798,7 +7798,7 @@
         <v>46267</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
@@ -7818,28 +7818,28 @@
         <v>0.02844860285750411</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>54.938</v>
+        <v>54.947</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>56.501</v>
+        <v>56.51</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>1.563</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>0.0284502530124868</v>
+        <v>0.02844559302600688</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>6576.27</v>
+        <v>6577.51</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>6819.21</v>
+        <v>6820.5</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>242.94</v>
+        <v>242.99</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>0.03694191388127312</v>
+        <v>0.03694255120858805</v>
       </c>
     </row>
     <row r="15">
@@ -7847,7 +7847,7 @@
         <v>46267</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
@@ -7858,37 +7858,37 @@
         <v>47.9982</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>48.6056</v>
+        <v>48.6051</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.6074000000000001</v>
+        <v>0.6069</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>0.01265464121571226</v>
+        <v>0.01264422415840594</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>55.5771</v>
+        <v>55.5975</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>56.2382</v>
+        <v>56.258</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>0.6611</v>
+        <v>0.6605</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>0.01189518704646338</v>
+        <v>0.01188003057691443</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>6677.96</v>
+        <v>6685.81</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>6732.29</v>
+        <v>6740.05</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>54.33</v>
+        <v>54.24</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>0.008135718093549526</v>
+        <v>0.008112704369403258</v>
       </c>
     </row>
     <row r="16">
@@ -7896,7 +7896,7 @@
         <v>46267</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
@@ -7916,28 +7916,28 @@
         <v>0.02047330948958786</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>55.4159</v>
+        <v>55.4326</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>56.5504</v>
+        <v>56.5675</v>
       </c>
       <c r="J16" s="10" t="n">
-        <v>1.1345</v>
+        <v>1.1349</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>0.02047246367919676</v>
+        <v>0.02047351197670685</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>6612.09</v>
+        <v>6613.09</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>6815.15</v>
+        <v>6816.65</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>203.06</v>
+        <v>203.56</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>0.03071041077783273</v>
+        <v>0.03078137451630025</v>
       </c>
     </row>
     <row r="17">
@@ -7945,7 +7945,7 @@
         <v>46267</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
@@ -7953,40 +7953,40 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>48.162</v>
+        <v>48.16</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>48.243</v>
+        <v>48.245</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.081</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.001681823844524729</v>
+        <v>0.001764950166112957</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>55.594</v>
+        <v>55.614</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>55.804</v>
+        <v>55.822</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>0.21</v>
+        <v>0.208</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>0.003777386048854193</v>
+        <v>0.003740065451145395</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>6602.23</v>
+        <v>6610.34</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>6701.08</v>
+        <v>6708.05</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>98.84999999999999</v>
+        <v>97.70999999999999</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>0.01497221393377692</v>
+        <v>0.01478138794676219</v>
       </c>
     </row>
     <row r="18">
@@ -7994,7 +7994,7 @@
         <v>46267</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
@@ -8002,40 +8002,40 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>48.2184</v>
+        <v>48.2181</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>48.3646</v>
+        <v>48.3642</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>0.1462</v>
+        <v>0.1461</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.003032037562424303</v>
+        <v>0.00302998251693866</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>55.8018</v>
+        <v>55.8231</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>55.973</v>
+        <v>55.9942</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>0.1712</v>
+        <v>0.1711</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>0.003068001390636144</v>
+        <v>0.003065039383337722</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>6666.77</v>
+        <v>6672.61</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>6713.86</v>
+        <v>6719.79</v>
       </c>
       <c r="N18" s="12" t="n">
-        <v>47.09</v>
+        <v>47.18</v>
       </c>
       <c r="O18" s="13" t="n">
-        <v>0.007063390517446979</v>
+        <v>0.007070696474093346</v>
       </c>
     </row>
     <row r="19">
@@ -8043,7 +8043,7 @@
         <v>46267</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
@@ -8059,16 +8059,16 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="12" t="n">
-        <v>6682.86</v>
+        <v>6685.7</v>
       </c>
       <c r="M19" s="12" t="n">
-        <v>6878.68</v>
+        <v>6881.57</v>
       </c>
       <c r="N19" s="12" t="n">
-        <v>195.82</v>
+        <v>195.87</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>0.02930182586497397</v>
+        <v>0.02929685747191768</v>
       </c>
     </row>
     <row r="20">
@@ -8076,7 +8076,7 @@
         <v>46267</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C20" s="31" t="inlineStr">
         <is>
@@ -8084,40 +8084,40 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>47.8045</v>
+        <v>47.7241</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>48.6911</v>
+        <v>48.6807</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0.8866000000000001</v>
+        <v>0.9566</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>0.01854637115752701</v>
+        <v>0.02004438009307666</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>55.2457</v>
+        <v>55.265</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>56.3859</v>
+        <v>56.4052</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>1.1402</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>0.02063871034306743</v>
+        <v>0.02063150275943183</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>6610.02</v>
+        <v>6615.9</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>7055.57</v>
+        <v>7061.4</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>445.55</v>
+        <v>445.5</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>0.06740524234419866</v>
+        <v>0.06733777717317371</v>
       </c>
     </row>
     <row r="21">
@@ -8125,7 +8125,7 @@
         <v>46267</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
@@ -8133,40 +8133,40 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>47.7513</v>
+        <v>47.7514</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>48.7549</v>
+        <v>48.7548</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.0036</v>
+        <v>1.0034</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.02101722885031403</v>
+        <v>0.02101299647759019</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>55.3574</v>
+        <v>55.3736</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>56.3663</v>
+        <v>56.3809</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>1.0089</v>
+        <v>1.0073</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>0.01822520566356079</v>
+        <v>0.01819097909473106</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>6576.42</v>
+        <v>6580.09</v>
       </c>
       <c r="M21" s="12" t="n">
-        <v>6828.38</v>
+        <v>6832</v>
       </c>
       <c r="N21" s="12" t="n">
-        <v>251.96</v>
+        <v>251.91</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>0.03831263818308441</v>
+        <v>0.03828367089203947</v>
       </c>
     </row>
     <row r="22">
@@ -8174,7 +8174,7 @@
         <v>46267</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -8182,40 +8182,40 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>47.6786</v>
+        <v>47.6784</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>48.8338</v>
+        <v>48.8334</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.1552</v>
+        <v>1.155</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>0.02422889933848728</v>
+        <v>0.02422480620155039</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>55.188</v>
+        <v>55.2069</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>56.5349</v>
+        <v>56.549</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>1.3469</v>
+        <v>1.3421</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>0.02440566789881858</v>
+        <v>0.02431036700122629</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>6600.05</v>
+        <v>6602.95</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>6781.04</v>
+        <v>6784.64</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>180.99</v>
+        <v>181.69</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>0.02742251952636722</v>
+        <v>0.02751648884210845</v>
       </c>
     </row>
     <row r="23">
@@ -8223,7 +8223,7 @@
         <v>46267</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C23" s="34" t="inlineStr">
         <is>
@@ -8272,7 +8272,7 @@
         <v>46267</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
@@ -8283,37 +8283,37 @@
         <v>47.6128</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>48.5991</v>
+        <v>48.5988</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>0.9863</v>
+        <v>0.986</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.02071501781033672</v>
+        <v>0.02070871698366826</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>55.2029</v>
+        <v>55.1375</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>56.3452</v>
+        <v>56.2799</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>1.1423</v>
+        <v>1.1424</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>0.02069275346041603</v>
+        <v>0.02071911131262752</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>6558.81</v>
+        <v>6561.59</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>6732.89</v>
+        <v>6735.59</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>174.08</v>
+        <v>174</v>
       </c>
       <c r="O24" s="13" t="n">
-        <v>0.02654140004055613</v>
+        <v>0.02651796287180394</v>
       </c>
     </row>
     <row r="25">
@@ -8321,7 +8321,7 @@
         <v>46267</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
@@ -8362,7 +8362,7 @@
         <v>46267</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
@@ -8370,40 +8370,40 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>48.2272</v>
+        <v>48.227</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>48.2801</v>
+        <v>48.28</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>0.0529</v>
+        <v>0.053</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>0.001096891380797558</v>
+        <v>0.001098969456943206</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>55.8142</v>
+        <v>55.8335</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>55.8918</v>
+        <v>55.9105</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>0.0776</v>
+        <v>0.077</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>0.001390327192721565</v>
+        <v>0.001379100360894445</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>6655.48</v>
+        <v>6661.11</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>6684.33</v>
+        <v>6689.87</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>28.85</v>
+        <v>28.76</v>
       </c>
       <c r="O26" s="13" t="n">
-        <v>0.004334773750353092</v>
+        <v>0.004317598718531896</v>
       </c>
     </row>
     <row r="27">
@@ -8411,7 +8411,7 @@
         <v>46267</v>
       </c>
       <c r="B27" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C27" s="38" t="inlineStr">
         <is>
@@ -8419,40 +8419,40 @@
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>48.163</v>
+        <v>48.162</v>
       </c>
       <c r="E27" s="8" t="n">
         <v>48.275</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.112</v>
+        <v>0.113</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>0.00232543653842161</v>
+        <v>0.002346248079398696</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>55.613</v>
+        <v>55.639</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>55.86</v>
+        <v>55.885</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>0.247</v>
+        <v>0.246</v>
       </c>
       <c r="K27" s="11" t="n">
-        <v>0.004441407584557567</v>
+        <v>0.004421359118603857</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>6614</v>
+        <v>6622</v>
       </c>
       <c r="M27" s="12" t="n">
-        <v>6690</v>
+        <v>6689</v>
       </c>
       <c r="N27" s="12" t="n">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>0.01149077713940127</v>
+        <v>0.01011778918755663</v>
       </c>
     </row>
     <row r="28">
@@ -8460,7 +8460,7 @@
         <v>46267</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -8468,40 +8468,40 @@
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>47.7615</v>
+        <v>47.761</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>48.7615</v>
+        <v>48.761</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>0.02093736586999989</v>
+        <v>0.0209375850589393</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>55.323</v>
+        <v>55.337</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>56.413</v>
+        <v>56.427</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>1.09</v>
       </c>
       <c r="K28" s="11" t="n">
-        <v>0.01970247455850189</v>
+        <v>0.01969748992536639</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>6662.49</v>
+        <v>6658.82</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>6762.49</v>
+        <v>6758.82</v>
       </c>
       <c r="N28" s="12" t="n">
         <v>100</v>
       </c>
       <c r="O28" s="13" t="n">
-        <v>0.0150094033912246</v>
+        <v>0.0150176758044218</v>
       </c>
     </row>
     <row r="29">
@@ -8509,7 +8509,7 @@
         <v>46267</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
@@ -8525,16 +8525,16 @@
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="12" t="n">
-        <v>6682.33</v>
+        <v>6684.14</v>
       </c>
       <c r="M29" s="12" t="n">
-        <v>6864.41</v>
+        <v>6866.24</v>
       </c>
       <c r="N29" s="12" t="n">
-        <v>182.08</v>
+        <v>182.1</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>0.0272479808689484</v>
+        <v>0.02724359453871403</v>
       </c>
     </row>
     <row r="30">
@@ -8542,7 +8542,7 @@
         <v>46267</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C30" s="41" t="inlineStr">
         <is>
@@ -8562,28 +8562,28 @@
         <v>0.02558322411533421</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>55.0871</v>
+        <v>55.1061</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>56.7391</v>
+        <v>56.7636</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>1.652</v>
+        <v>1.6575</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>0.02998887216789412</v>
+        <v>0.03007833978452476</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>6579.39</v>
+        <v>6585.25</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>6776.91</v>
+        <v>6783.56</v>
       </c>
       <c r="N30" s="12" t="n">
-        <v>197.52</v>
+        <v>198.31</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>0.0300210201857619</v>
+        <v>0.03011427052883337</v>
       </c>
     </row>
     <row r="31">
@@ -8591,7 +8591,7 @@
         <v>46267</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -8599,40 +8599,40 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>48.1513</v>
+        <v>48.2974</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>48.3928</v>
+        <v>48.2974</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>0.2415</v>
+        <v>0</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>0.005015440912291049</v>
+        <v>0</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>55.6838</v>
+        <v>55.9313</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>56.0193</v>
+        <v>55.9313</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>0.3355</v>
+        <v>0</v>
       </c>
       <c r="K31" s="11" t="n">
-        <v>0.006025091678369652</v>
+        <v>0</v>
       </c>
       <c r="L31" s="12" t="n">
-        <v>6591.43</v>
+        <v>6681.5</v>
       </c>
       <c r="M31" s="12" t="n">
-        <v>6724.93</v>
+        <v>6681.5</v>
       </c>
       <c r="N31" s="12" t="n">
-        <v>133.5</v>
+        <v>0</v>
       </c>
       <c r="O31" s="13" t="n">
-        <v>0.02025357168323111</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -8640,7 +8640,7 @@
         <v>46267</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C32" s="43" t="inlineStr">
         <is>
@@ -8660,28 +8660,28 @@
         <v>0.01676213483686123</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>55.4313</v>
+        <v>55.4468</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>56.282</v>
+        <v>56.2975</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>0.8507</v>
       </c>
       <c r="K32" s="11" t="n">
-        <v>0.01534692493230359</v>
+        <v>0.01534263474177049</v>
       </c>
       <c r="L32" s="12" t="n">
-        <v>6608.49</v>
+        <v>6610.55</v>
       </c>
       <c r="M32" s="12" t="n">
-        <v>6804.84</v>
+        <v>6806.97</v>
       </c>
       <c r="N32" s="12" t="n">
-        <v>196.35</v>
+        <v>196.42</v>
       </c>
       <c r="O32" s="13" t="n">
-        <v>0.02971177984683339</v>
+        <v>0.02971311010430297</v>
       </c>
     </row>
     <row r="33">
@@ -8689,7 +8689,7 @@
         <v>46267</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
@@ -8697,40 +8697,40 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>48.1538</v>
+        <v>48.1537</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>48.3569</v>
+        <v>48.3568</v>
       </c>
       <c r="F33" s="8" t="n">
         <v>0.2031</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>0.004217735671951123</v>
+        <v>0.004217744430853704</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>55.7318</v>
+        <v>55.7532</v>
       </c>
       <c r="I33" s="10" t="n">
-        <v>55.9564</v>
+        <v>55.9778</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>0.2246</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>0.004030015179843464</v>
+        <v>0.004028468321100851</v>
       </c>
       <c r="L33" s="12" t="n">
-        <v>6645.43</v>
+        <v>6651.71</v>
       </c>
       <c r="M33" s="12" t="n">
-        <v>6698.81</v>
+        <v>6705.14</v>
       </c>
       <c r="N33" s="12" t="n">
-        <v>53.38</v>
+        <v>53.43</v>
       </c>
       <c r="O33" s="13" t="n">
-        <v>0.008032587808463861</v>
+        <v>0.0080325209607755</v>
       </c>
     </row>
     <row r="34">
@@ -8738,7 +8738,7 @@
         <v>46267</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C34" s="45" t="inlineStr">
         <is>
@@ -8758,28 +8758,28 @@
         <v>0.02006493438703818</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>55.4714</v>
+        <v>55.4695</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>56.5735</v>
+        <v>56.5715</v>
       </c>
       <c r="J34" s="10" t="n">
-        <v>1.1021</v>
+        <v>1.102</v>
       </c>
       <c r="K34" s="11" t="n">
-        <v>0.01986789588869219</v>
+        <v>0.01986677363235652</v>
       </c>
       <c r="L34" s="12" t="n">
-        <v>6614.34</v>
+        <v>6611.87</v>
       </c>
       <c r="M34" s="12" t="n">
-        <v>6758.94</v>
+        <v>6756.47</v>
       </c>
       <c r="N34" s="12" t="n">
         <v>144.6</v>
       </c>
       <c r="O34" s="13" t="n">
-        <v>0.02186159163272526</v>
+        <v>0.02186975847982492</v>
       </c>
     </row>
     <row r="35">
@@ -8787,7 +8787,7 @@
         <v>46267</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C35" s="46" t="inlineStr">
         <is>
@@ -8798,25 +8798,25 @@
         <v>48.186</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>48.24</v>
+        <v>48.239</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.054</v>
+        <v>0.053</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>0.001120657452372058</v>
+        <v>0.00109990453658739</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>55.64</v>
+        <v>55.655</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>55.785</v>
+        <v>55.803</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>0.145</v>
+        <v>0.148</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>0.002606038820992092</v>
+        <v>0.002659239960470757</v>
       </c>
       <c r="L35" s="12" t="n"/>
       <c r="M35" s="12" t="n"/>
@@ -8828,7 +8828,7 @@
         <v>46267</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C36" s="47" t="inlineStr">
         <is>
@@ -8848,28 +8848,28 @@
         <v>0.02098635886673662</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>55.17</v>
+        <v>55.19</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>56.31</v>
+        <v>56.32</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="K36" s="11" t="n">
-        <v>0.02066340402392605</v>
+        <v>0.02047472368182642</v>
       </c>
       <c r="L36" s="12" t="n">
-        <v>6581.19</v>
+        <v>6582.59</v>
       </c>
       <c r="M36" s="12" t="n">
-        <v>6783.18</v>
+        <v>6784.52</v>
       </c>
       <c r="N36" s="12" t="n">
-        <v>201.99</v>
+        <v>201.93</v>
       </c>
       <c r="O36" s="13" t="n">
-        <v>0.03069201770500472</v>
+        <v>0.03067637510463207</v>
       </c>
     </row>
     <row r="37">
@@ -8877,7 +8877,7 @@
         <v>46267</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C37" s="48" t="inlineStr">
         <is>
@@ -8897,28 +8897,28 @@
         <v>0.02022948183877804</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>55.4352</v>
+        <v>55.4359</v>
       </c>
       <c r="I37" s="10" t="n">
-        <v>56.5567</v>
+        <v>56.5574</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>1.1215</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>0.02023082806592201</v>
+        <v>0.02023057260728156</v>
       </c>
       <c r="L37" s="12" t="n">
-        <v>6647.74</v>
+        <v>6649.04</v>
       </c>
       <c r="M37" s="12" t="n">
-        <v>6781.97</v>
+        <v>6783.29</v>
       </c>
       <c r="N37" s="12" t="n">
-        <v>134.23</v>
+        <v>134.25</v>
       </c>
       <c r="O37" s="13" t="n">
-        <v>0.02019182459001104</v>
+        <v>0.02019088469914454</v>
       </c>
     </row>
     <row r="38">
@@ -8926,7 +8926,7 @@
         <v>46267</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
@@ -8946,28 +8946,28 @@
         <v>0.01360495969827946</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>55.4338</v>
+        <v>55.4499</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>56.2441</v>
+        <v>56.2606</v>
       </c>
       <c r="J38" s="10" t="n">
-        <v>0.8103</v>
+        <v>0.8107</v>
       </c>
       <c r="K38" s="11" t="n">
-        <v>0.01461743557179915</v>
+        <v>0.0146204050863933</v>
       </c>
       <c r="L38" s="12" t="n">
-        <v>6614.38</v>
+        <v>6619.46</v>
       </c>
       <c r="M38" s="12" t="n">
-        <v>6747.93</v>
+        <v>6753.11</v>
       </c>
       <c r="N38" s="12" t="n">
-        <v>133.55</v>
+        <v>133.65</v>
       </c>
       <c r="O38" s="13" t="n">
-        <v>0.02019085689059292</v>
+        <v>0.02019046870892792</v>
       </c>
     </row>
     <row r="39">
@@ -8975,7 +8975,7 @@
         <v>46267</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="C39" s="50" t="inlineStr">
         <is>
@@ -8986,37 +8986,37 @@
         <v>47.7684</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>48.7652</v>
+        <v>48.7651</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.9968</v>
+        <v>0.9967</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>0.02086735163832157</v>
+        <v>0.02086525820416845</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>55.2611</v>
+        <v>55.2759</v>
       </c>
       <c r="I39" s="10" t="n">
-        <v>56.4695</v>
+        <v>56.485</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1.2084</v>
+        <v>1.2091</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>0.02186710000343823</v>
+        <v>0.02187390888253289</v>
       </c>
       <c r="L39" s="12" t="n">
-        <v>6632.7</v>
+        <v>6637.93</v>
       </c>
       <c r="M39" s="12" t="n">
-        <v>6843.25</v>
+        <v>6848.63</v>
       </c>
       <c r="N39" s="12" t="n">
-        <v>210.55</v>
+        <v>210.7</v>
       </c>
       <c r="O39" s="13" t="n">
-        <v>0.03174423688693895</v>
+        <v>0.03174182312859582</v>
       </c>
     </row>
   </sheetData>
@@ -42318,7 +42318,7 @@
       </c>
       <c r="B5" s="62" t="n"/>
       <c r="C5" s="64" t="n">
-        <v>0.4528240740740741</v>
+        <v>0.4614699074074074</v>
       </c>
       <c r="D5" s="62" t="n"/>
       <c r="F5" s="62" t="inlineStr">
@@ -42402,7 +42402,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="70" t="n">
-        <v>0.02023082806592201</v>
+        <v>0.02023057260728156</v>
       </c>
       <c r="O6" s="71" t="inlineStr">
         <is>
@@ -42410,10 +42410,10 @@
         </is>
       </c>
       <c r="P6" s="72" t="n">
-        <v>55.4352</v>
+        <v>55.4359</v>
       </c>
       <c r="Q6" s="72" t="n">
-        <v>56.5567</v>
+        <v>56.5574</v>
       </c>
     </row>
     <row r="7">
@@ -42455,7 +42455,7 @@
         <v>5</v>
       </c>
       <c r="N7" s="70" t="n">
-        <v>0.02019182459001104</v>
+        <v>0.02019088469914454</v>
       </c>
       <c r="O7" s="71" t="inlineStr">
         <is>
@@ -42463,10 +42463,10 @@
         </is>
       </c>
       <c r="P7" s="72" t="n">
-        <v>6647.74</v>
+        <v>6649.04</v>
       </c>
       <c r="Q7" s="72" t="n">
-        <v>6781.97</v>
+        <v>6783.29</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Günlük kur verisi: 02.09.2026 11:29
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -1007,24 +1007,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -1033,6 +1037,7 @@
           <max val="0.06809845902702412"/>
           <min val="0.01398473878667442"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -1050,9 +1055,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -1178,6 +1197,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -1186,24 +1213,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -1212,6 +1243,7 @@
           <max val="0.06361034633532447"/>
           <min val="0.02255547230137524"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -1229,9 +1261,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -1369,6 +1415,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -1377,24 +1431,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -1403,6 +1461,7 @@
           <max val="0.06393703694203891"/>
           <min val="0.02251604918664015"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -1420,9 +1479,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -1560,6 +1633,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -1568,24 +1649,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -1594,6 +1679,7 @@
           <max val="0.09492887751151027"/>
           <min val="0.02634377435370254"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -1611,9 +1697,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -1751,6 +1851,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -1759,24 +1867,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -1785,6 +1897,7 @@
           <max val="0.06300273000209422"/>
           <min val="0.01394771487950567"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -1802,9 +1915,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -1942,6 +2069,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -1950,24 +2085,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -1976,6 +2115,7 @@
           <max val="0.05612935000212975"/>
           <min val="0.01451066469310389"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -1993,9 +2133,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -2133,6 +2287,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -2141,24 +2303,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -2167,6 +2333,7 @@
           <max val="0.08822748202703072"/>
           <min val="0.0196170269615309"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -2184,9 +2351,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -2324,6 +2505,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -2332,24 +2521,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -2358,6 +2551,7 @@
           <max val="0.07017975595934527"/>
           <min val="0.01190344185435327"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -2375,9 +2569,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -2515,6 +2723,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -2523,24 +2739,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -2549,6 +2769,7 @@
           <max val="0.07017999927062174"/>
           <min val="0.01190503299558375"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -2566,9 +2787,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -2706,6 +2941,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -2714,24 +2957,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -2740,6 +2987,7 @@
           <max val="0.1709612332154084"/>
           <min val="0"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -2757,9 +3005,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -2897,6 +3159,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -2905,24 +3175,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -2931,6 +3205,7 @@
           <max val="0.06165859703981922"/>
           <min val="0.01797489899804002"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -2948,9 +3223,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -3464,24 +3753,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -3490,6 +3783,7 @@
           <max val="0.06809875047508467"/>
           <min val="0.01398628179112082"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -3507,9 +3801,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -3635,6 +3943,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -3643,24 +3959,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -3669,6 +3989,7 @@
           <max val="0.06209535841468713"/>
           <min val="0.01791241253707181"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -3686,9 +4007,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -3826,6 +4161,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -3834,24 +4177,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -3860,6 +4207,7 @@
           <max val="0.1462720659556508"/>
           <min val="0.007620168856054751"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -3877,9 +4225,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -4393,24 +4755,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -4419,6 +4785,7 @@
           <max val="0.1646791482454227"/>
           <min val="0.001344939025793405"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -4436,9 +4803,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -4820,24 +5201,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -4846,6 +5231,7 @@
           <max val="0.05171408776103012"/>
           <min val="0.0161237184650772"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -4863,9 +5249,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -5247,24 +5647,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -5273,6 +5677,7 @@
           <max val="0.05613143775214488"/>
           <min val="0.01554823152705276"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -5290,9 +5695,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -5674,24 +6093,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -5700,6 +6123,7 @@
           <max val="0.113954760403876"/>
           <min val="0.007962009561212546"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -5717,9 +6141,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -5845,6 +6283,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -5853,24 +6299,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -5879,6 +6329,7 @@
           <max val="0.04535890324268219"/>
           <min val="0.02563021945997443"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -5896,9 +6347,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -6036,6 +6501,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -6044,24 +6517,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -6070,6 +6547,7 @@
           <max val="0.04536575081521625"/>
           <min val="0.02562858686951813"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -6087,9 +6565,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -6227,6 +6719,14 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <dLbls>
+          <numFmt formatCode="0.00%"/>
+          <dLblPos val="t"/>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -6235,24 +6735,28 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="650"/>
+              <a:defRPr sz="700"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="650"/>
+            <a:endParaRPr sz="700"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="1"/>
+        <tickMarkSkip val="1"/>
       </catAx>
       <valAx>
         <axId val="100"/>
@@ -6261,6 +6765,7 @@
           <max val="0.07745416653140928"/>
           <min val="0.03018959592357282"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -6278,9 +6783,23 @@
           </tx>
         </title>
         <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
+        <majorTickMark val="out"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="700"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+            <a:endParaRPr sz="700"/>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -7210,7 +7729,7 @@
         <v>46267</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
@@ -7230,28 +7749,28 @@
         <v>0.02842045430622513</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>55.0015</v>
+        <v>55.006</v>
       </c>
       <c r="I2" s="10" t="n">
-        <v>56.5696</v>
+        <v>56.5693</v>
       </c>
       <c r="J2" s="10" t="n">
-        <v>1.5681</v>
+        <v>1.5633</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>0.02851013154186704</v>
+        <v>0.02842053594153365</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>6536.54</v>
+        <v>6539.92</v>
       </c>
       <c r="M2" s="12" t="n">
-        <v>6772.6</v>
+        <v>6776.25</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>236.06</v>
+        <v>236.33</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>0.03611390735771524</v>
+        <v>0.03613652766394695</v>
       </c>
     </row>
     <row r="3">
@@ -7259,7 +7778,7 @@
         <v>46267</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
@@ -7279,28 +7798,28 @@
         <v>0.01630582291166461</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>55.459</v>
+        <v>55.464</v>
       </c>
       <c r="I3" s="10" t="n">
         <v>56.374</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.915</v>
+        <v>0.91</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>0.01649867469662273</v>
+        <v>0.01640703879994231</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>6614.61</v>
+        <v>6613.3</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>6750.58</v>
+        <v>6749.32</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>135.97</v>
+        <v>136.02</v>
       </c>
       <c r="O3" s="13" t="n">
-        <v>0.02055601161670907</v>
+        <v>0.02056764399014108</v>
       </c>
     </row>
     <row r="4">
@@ -7308,7 +7827,7 @@
         <v>46267</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -7316,40 +7835,40 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>48.083</v>
+        <v>48.079</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>48.373</v>
+        <v>48.376</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.29</v>
+        <v>0.297</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>0.006031237651560843</v>
+        <v>0.006177333139208386</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>55.501</v>
+        <v>55.504</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>56.009</v>
+        <v>56.022</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.508</v>
+        <v>0.518</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>0.009152988234446227</v>
+        <v>0.009332660709138079</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>6675.22</v>
+        <v>6674.93</v>
       </c>
       <c r="M4" s="12" t="n">
-        <v>6742.94</v>
+        <v>6742.97</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>67.72</v>
+        <v>68.04000000000001</v>
       </c>
       <c r="O4" s="13" t="n">
-        <v>0.01014498398554654</v>
+        <v>0.0101933653236813</v>
       </c>
     </row>
     <row r="5">
@@ -7357,7 +7876,7 @@
         <v>46267</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -7377,28 +7896,28 @@
         <v>0.004363183045917307</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>55.625</v>
+        <v>55.621</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>55.98</v>
+        <v>55.976</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>0.355</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>0.006382022471910113</v>
+        <v>0.00638248143686737</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>6588.87</v>
+        <v>6583.96</v>
       </c>
       <c r="M5" s="12" t="n">
         <v>6775</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>186.13</v>
+        <v>191.04</v>
       </c>
       <c r="O5" s="13" t="n">
-        <v>0.02824915349673009</v>
+        <v>0.02901597215049909</v>
       </c>
     </row>
     <row r="6">
@@ -7406,7 +7925,7 @@
         <v>46267</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
@@ -7414,40 +7933,40 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>47.4531</v>
+        <v>47.4528</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>48.7294</v>
+        <v>48.7293</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>1.2763</v>
+        <v>1.2765</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.02689602997485939</v>
+        <v>0.02690041472789804</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>55.0539</v>
+        <v>55.0511</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>56.4187</v>
+        <v>56.4161</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>1.3648</v>
+        <v>1.365</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0.02479025100855707</v>
+        <v>0.02479514487448934</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>6601.93</v>
+        <v>6596.32</v>
       </c>
       <c r="M6" s="12" t="n">
-        <v>6752.76</v>
+        <v>6747.3</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>150.83</v>
+        <v>150.98</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>0.02284634947659245</v>
+        <v>0.02288851965944648</v>
       </c>
     </row>
     <row r="7">
@@ -7455,7 +7974,7 @@
         <v>46267</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
@@ -7475,28 +7994,28 @@
         <v>0.04065367214916916</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>54.776</v>
+        <v>54.772</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>57.007</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>2.231</v>
+        <v>2.235</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>0.0407295165766029</v>
+        <v>0.04080552106915943</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>6598.78</v>
+        <v>6593.35</v>
       </c>
       <c r="M7" s="12" t="n">
-        <v>6793</v>
+        <v>6787.56</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>194.22</v>
+        <v>194.21</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>0.02943271331973486</v>
+        <v>0.02945543615916037</v>
       </c>
     </row>
     <row r="8">
@@ -7504,7 +8023,7 @@
         <v>46267</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
@@ -7536,16 +8055,16 @@
         <v>0.02944178107067625</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>6612.92</v>
+        <v>6610.78</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>6808.61</v>
+        <v>6806.45</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>195.69</v>
+        <v>195.67</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>0.02959207127864846</v>
+        <v>0.02959862527568608</v>
       </c>
     </row>
     <row r="9">
@@ -7553,7 +8072,7 @@
         <v>46267</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -7561,40 +8080,40 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>48.2243</v>
+        <v>48.2242</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>48.2813</v>
+        <v>48.2817</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.057</v>
+        <v>0.0575</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.001181976721279521</v>
+        <v>0.001192347410636154</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>55.8328</v>
+        <v>55.8326</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>55.9159</v>
+        <v>55.9161</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.08309999999999999</v>
+        <v>0.0835</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>0.001488372426244071</v>
+        <v>0.00149554203099981</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6666.72</v>
+        <v>6662.85</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>6695.46</v>
+        <v>6691.74</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>28.74</v>
+        <v>28.89</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>0.004310965512275901</v>
+        <v>0.004335982349895314</v>
       </c>
     </row>
     <row r="10">
@@ -7602,7 +8121,7 @@
         <v>46267</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -7610,40 +8129,40 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>48.2379</v>
+        <v>48.2377</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>48.2761</v>
+        <v>48.2759</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>0.0382</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.0007919084371417495</v>
+        <v>0.0007919117205007701</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>55.8102</v>
+        <v>55.8099</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>55.924</v>
+        <v>55.919</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.1138</v>
+        <v>0.1091</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>0.002039053793034248</v>
+        <v>0.001954850304336686</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>6664.59</v>
+        <v>6659.12</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>6696.21</v>
+        <v>6690.78</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>31.62</v>
+        <v>31.66</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>0.004744477904867366</v>
+        <v>0.00475438196037915</v>
       </c>
     </row>
     <row r="11">
@@ -7651,7 +8170,7 @@
         <v>46267</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
@@ -7659,40 +8178,40 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>47.9241</v>
+        <v>47.9239</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>49.1617</v>
+        <v>49.1614</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1.2376</v>
+        <v>1.2375</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.02582416779866497</v>
+        <v>0.02582218892869738</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>55.3879</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>56.6664</v>
+        <v>56.6663</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>1.2785</v>
+        <v>1.2784</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>0.02308265884787111</v>
+        <v>0.02308085339938867</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6612.91</v>
+        <v>6614.87</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>6721.13</v>
+        <v>6723.1</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>108.22</v>
+        <v>108.23</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>0.01636495884565191</v>
+        <v>0.01636162161917014</v>
       </c>
     </row>
     <row r="12">
@@ -7700,7 +8219,7 @@
         <v>46267</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
@@ -7720,28 +8239,28 @@
         <v>0.01776477349913789</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>55.3243</v>
+        <v>55.3195</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>56.4812</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>1.1569</v>
+        <v>1.1617</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>0.02091124514905747</v>
+        <v>0.02099982827032059</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>6613.01</v>
+        <v>6607.97</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>6767.11</v>
+        <v>6762.41</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>154.1</v>
+        <v>154.44</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>0.02330255057832969</v>
+        <v>0.02337177680891408</v>
       </c>
     </row>
     <row r="13">
@@ -7749,7 +8268,7 @@
         <v>46267</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
@@ -7757,40 +8276,40 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>47.9983</v>
+        <v>47.9981</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>48.6051</v>
+        <v>48.6053</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.6068</v>
+        <v>0.6072</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.01264211440821863</v>
+        <v>0.01265050074898798</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>55.595</v>
+        <v>55.5975</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>56.2555</v>
+        <v>56.2586</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>0.6605</v>
+        <v>0.6611</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>0.01188056479899271</v>
+        <v>0.01189082242906605</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6683.49</v>
+        <v>6683.82</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>6737.85</v>
+        <v>6738.14</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>54.36</v>
+        <v>54.32</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>0.008133475175394891</v>
+        <v>0.008127089000002993</v>
       </c>
     </row>
     <row r="14">
@@ -7798,7 +8317,7 @@
         <v>46267</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
@@ -7818,28 +8337,28 @@
         <v>0.02844860285750411</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>54.947</v>
+        <v>54.952</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>56.51</v>
+        <v>56.515</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>1.563</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>0.02844559302600688</v>
+        <v>0.02844300480419275</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>6577.51</v>
+        <v>6577.16</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>6820.5</v>
+        <v>6820.13</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>242.99</v>
+        <v>242.97</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>0.03694255120858805</v>
+        <v>0.03694147626027039</v>
       </c>
     </row>
     <row r="15">
@@ -7847,7 +8366,7 @@
         <v>46267</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
@@ -7855,40 +8374,40 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>47.9982</v>
+        <v>47.998</v>
       </c>
       <c r="E15" s="8" t="n">
         <v>48.6051</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.6069</v>
+        <v>0.6071</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>0.01264422415840594</v>
+        <v>0.01264844368515355</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>55.5975</v>
+        <v>55.5959</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>56.258</v>
+        <v>56.2564</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>0.6605</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>0.01188003057691443</v>
+        <v>0.01188037247350974</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>6685.81</v>
+        <v>6680.4</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>6740.05</v>
+        <v>6734.79</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>54.24</v>
+        <v>54.39</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>0.008112704369403258</v>
+        <v>0.008141728040237111</v>
       </c>
     </row>
     <row r="16">
@@ -7896,7 +8415,7 @@
         <v>46267</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
@@ -7916,28 +8435,28 @@
         <v>0.02047330948958786</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>55.4326</v>
+        <v>55.4302</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>56.5675</v>
+        <v>56.5651</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>1.1349</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>0.02047351197670685</v>
+        <v>0.02047439843262337</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>6613.09</v>
+        <v>6613.91</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>6816.65</v>
+        <v>6817.49</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>203.56</v>
+        <v>203.58</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>0.03078137451630025</v>
+        <v>0.03078058213673908</v>
       </c>
     </row>
     <row r="17">
@@ -7945,7 +8464,7 @@
         <v>46267</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
@@ -7953,40 +8472,40 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>48.16</v>
+        <v>48.183</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>48.245</v>
+        <v>48.242</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.059</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.001764950166112957</v>
+        <v>0.001224498267023639</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>55.614</v>
+        <v>55.643</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>55.822</v>
+        <v>55.811</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>0.208</v>
+        <v>0.168</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>0.003740065451145395</v>
+        <v>0.003019247704113725</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>6610.34</v>
+        <v>6610.07</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>6708.05</v>
+        <v>6705</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>97.70999999999999</v>
+        <v>94.93000000000001</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>0.01478138794676219</v>
+        <v>0.01436142128600756</v>
       </c>
     </row>
     <row r="18">
@@ -7994,7 +8513,7 @@
         <v>46267</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
@@ -8005,37 +8524,37 @@
         <v>48.2181</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>48.3642</v>
+        <v>48.3643</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>0.1461</v>
+        <v>0.1462</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.00302998251693866</v>
+        <v>0.003032056426943409</v>
       </c>
       <c r="H18" s="10" t="n">
         <v>55.8231</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>55.9942</v>
+        <v>55.9943</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>0.1711</v>
+        <v>0.1712</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>0.003065039383337722</v>
+        <v>0.003066830756443121</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>6672.61</v>
+        <v>6669.56</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>6719.79</v>
+        <v>6716.68</v>
       </c>
       <c r="N18" s="12" t="n">
-        <v>47.18</v>
+        <v>47.12</v>
       </c>
       <c r="O18" s="13" t="n">
-        <v>0.007070696474093346</v>
+        <v>0.007064933818722674</v>
       </c>
     </row>
     <row r="19">
@@ -8043,7 +8562,7 @@
         <v>46267</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
@@ -8059,16 +8578,16 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="12" t="n">
-        <v>6685.7</v>
+        <v>6685.53</v>
       </c>
       <c r="M19" s="12" t="n">
-        <v>6881.57</v>
+        <v>6881.39</v>
       </c>
       <c r="N19" s="12" t="n">
-        <v>195.87</v>
+        <v>195.86</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>0.02929685747191768</v>
+        <v>0.02929610666618802</v>
       </c>
     </row>
     <row r="20">
@@ -8076,7 +8595,7 @@
         <v>46267</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C20" s="31" t="inlineStr">
         <is>
@@ -8084,40 +8603,40 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>47.7241</v>
+        <v>47.8071</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>48.6807</v>
+        <v>48.6877</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0.9566</v>
+        <v>0.8806</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>0.02004438009307666</v>
+        <v>0.01841985813822633</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>55.265</v>
+        <v>55.3609</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>56.4052</v>
+        <v>56.4133</v>
       </c>
       <c r="J20" s="10" t="n">
-        <v>1.1402</v>
+        <v>1.0524</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>0.02063150275943183</v>
+        <v>0.01900980656022572</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>6615.9</v>
+        <v>6613.08</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>7061.4</v>
+        <v>7057.74</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>445.5</v>
+        <v>444.66</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>0.06733777717317371</v>
+        <v>0.06723947086682756</v>
       </c>
     </row>
     <row r="21">
@@ -8125,7 +8644,7 @@
         <v>46267</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
@@ -8136,37 +8655,37 @@
         <v>47.7514</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>48.7548</v>
+        <v>48.7543</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.0034</v>
+        <v>1.0029</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.02101299647759019</v>
+        <v>0.02100252558040183</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>55.3736</v>
+        <v>55.3718</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>56.3809</v>
+        <v>56.3808</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>1.0073</v>
+        <v>1.009</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>0.01819097909473106</v>
+        <v>0.01822227198682362</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>6580.09</v>
+        <v>6581.47</v>
       </c>
       <c r="M21" s="12" t="n">
-        <v>6832</v>
+        <v>6833.43</v>
       </c>
       <c r="N21" s="12" t="n">
-        <v>251.91</v>
+        <v>251.96</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>0.03828367089203947</v>
+        <v>0.03828324067419588</v>
       </c>
     </row>
     <row r="22">
@@ -8174,7 +8693,7 @@
         <v>46267</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -8182,40 +8701,40 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>47.6784</v>
+        <v>47.6783</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>48.8334</v>
+        <v>48.8332</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.155</v>
+        <v>1.1549</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>0.02422480620155039</v>
+        <v>0.02422275962020458</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>55.2069</v>
+        <v>55.202</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>56.549</v>
+        <v>56.5488</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>1.3421</v>
+        <v>1.3468</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>0.02431036700122629</v>
+        <v>0.02439766675120467</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>6602.95</v>
+        <v>6604.18</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>6784.64</v>
+        <v>6785.28</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>181.69</v>
+        <v>181.1</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>0.02751648884210845</v>
+        <v>0.02742202665584524</v>
       </c>
     </row>
     <row r="23">
@@ -8223,7 +8742,7 @@
         <v>46267</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C23" s="34" t="inlineStr">
         <is>
@@ -8231,28 +8750,28 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>48.17</v>
+        <v>48.22</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>48.18</v>
+        <v>48.23</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>0.01</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>0.0002075980900975711</v>
+        <v>0.0002073828287017835</v>
       </c>
       <c r="H23" s="10" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="I23" s="10" t="n">
         <v>55.75</v>
-      </c>
-      <c r="I23" s="10" t="n">
-        <v>55.8</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>0.05</v>
       </c>
       <c r="K23" s="11" t="n">
-        <v>0.0008968609865470851</v>
+        <v>0.0008976660682226212</v>
       </c>
       <c r="L23" s="12" t="n">
         <v>6722.02</v>
@@ -8272,7 +8791,7 @@
         <v>46267</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
@@ -8280,40 +8799,40 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>47.6128</v>
+        <v>47.6129</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>48.5988</v>
+        <v>48.5986</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>0.986</v>
+        <v>0.9857</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.02070871698366826</v>
+        <v>0.02070237267631251</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>55.1375</v>
+        <v>55.1334</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>56.2799</v>
+        <v>56.2772</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>1.1424</v>
+        <v>1.1438</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>0.02071911131262752</v>
+        <v>0.02074604504710393</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>6561.59</v>
+        <v>6561.48</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>6735.59</v>
+        <v>6735.43</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>174</v>
+        <v>173.95</v>
       </c>
       <c r="O24" s="13" t="n">
-        <v>0.02651796287180394</v>
+        <v>0.02651078720044868</v>
       </c>
     </row>
     <row r="25">
@@ -8321,7 +8840,7 @@
         <v>46267</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
@@ -8362,7 +8881,7 @@
         <v>46267</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
@@ -8373,37 +8892,37 @@
         <v>48.227</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>48.28</v>
+        <v>48.2796</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>0.053</v>
+        <v>0.0526</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>0.001098969456943206</v>
+        <v>0.001090675347834201</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>55.8335</v>
+        <v>55.8305</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>55.9105</v>
+        <v>55.9073</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>0.077</v>
+        <v>0.07679999999999999</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>0.001379100360894445</v>
+        <v>0.001375592194230752</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>6661.11</v>
+        <v>6658.35</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>6689.87</v>
+        <v>6687.13</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>28.76</v>
+        <v>28.78</v>
       </c>
       <c r="O26" s="13" t="n">
-        <v>0.004317598718531896</v>
+        <v>0.004322392184249852</v>
       </c>
     </row>
     <row r="27">
@@ -8411,7 +8930,7 @@
         <v>46267</v>
       </c>
       <c r="B27" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C27" s="38" t="inlineStr">
         <is>
@@ -8419,40 +8938,40 @@
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>48.162</v>
+        <v>48.182</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>48.275</v>
+        <v>48.285</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.113</v>
+        <v>0.103</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>0.002346248079398696</v>
+        <v>0.002137727782159313</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>55.639</v>
+        <v>55.652</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>55.885</v>
+        <v>55.883</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>0.246</v>
+        <v>0.231</v>
       </c>
       <c r="K27" s="11" t="n">
-        <v>0.004421359118603857</v>
+        <v>0.004150794221231942</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>6622</v>
+        <v>6623</v>
       </c>
       <c r="M27" s="12" t="n">
-        <v>6689</v>
+        <v>6683</v>
       </c>
       <c r="N27" s="12" t="n">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>0.01011778918755663</v>
+        <v>0.009059338668277217</v>
       </c>
     </row>
     <row r="28">
@@ -8460,7 +8979,7 @@
         <v>46267</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -8492,16 +9011,16 @@
         <v>0.01969748992536639</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>6658.82</v>
+        <v>6662.57</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>6758.82</v>
+        <v>6762.57</v>
       </c>
       <c r="N28" s="12" t="n">
         <v>100</v>
       </c>
       <c r="O28" s="13" t="n">
-        <v>0.0150176758044218</v>
+        <v>0.01500922316763651</v>
       </c>
     </row>
     <row r="29">
@@ -8509,7 +9028,7 @@
         <v>46267</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
@@ -8525,16 +9044,16 @@
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="12" t="n">
-        <v>6684.14</v>
+        <v>6686.42</v>
       </c>
       <c r="M29" s="12" t="n">
-        <v>6866.24</v>
+        <v>6868.55</v>
       </c>
       <c r="N29" s="12" t="n">
-        <v>182.1</v>
+        <v>182.13</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>0.02724359453871403</v>
+        <v>0.02723879146090135</v>
       </c>
     </row>
     <row r="30">
@@ -8542,7 +9061,7 @@
         <v>46267</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C30" s="41" t="inlineStr">
         <is>
@@ -8562,28 +9081,28 @@
         <v>0.02558322411533421</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>55.1061</v>
+        <v>55.1014</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>56.7636</v>
+        <v>56.7587</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>1.6575</v>
+        <v>1.6573</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>0.03007833978452476</v>
+        <v>0.03007727571350274</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>6585.25</v>
+        <v>6581.7</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>6783.56</v>
+        <v>6779.29</v>
       </c>
       <c r="N30" s="12" t="n">
-        <v>198.31</v>
+        <v>197.59</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>0.03011427052883337</v>
+        <v>0.03002111916374189</v>
       </c>
     </row>
     <row r="31">
@@ -8591,7 +9110,7 @@
         <v>46267</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -8599,10 +9118,10 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>48.2974</v>
+        <v>48.2768</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>48.2974</v>
+        <v>48.2768</v>
       </c>
       <c r="F31" s="8" t="n">
         <v>0</v>
@@ -8611,10 +9130,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>55.9313</v>
+        <v>55.9056</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>55.9313</v>
+        <v>55.9056</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>0</v>
@@ -8623,10 +9142,10 @@
         <v>0</v>
       </c>
       <c r="L31" s="12" t="n">
-        <v>6681.5</v>
+        <v>6677.96</v>
       </c>
       <c r="M31" s="12" t="n">
-        <v>6681.5</v>
+        <v>6677.96</v>
       </c>
       <c r="N31" s="12" t="n">
         <v>0</v>
@@ -8640,7 +9159,7 @@
         <v>46267</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C32" s="43" t="inlineStr">
         <is>
@@ -8651,37 +9170,37 @@
         <v>47.8519</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>48.654</v>
+        <v>48.6538</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.8021</v>
+        <v>0.8018999999999999</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>0.01676213483686123</v>
+        <v>0.01675795527450321</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>55.4468</v>
+        <v>55.4453</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>56.2975</v>
+        <v>56.2957</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>0.8507</v>
+        <v>0.8504</v>
       </c>
       <c r="K32" s="11" t="n">
-        <v>0.01534263474177049</v>
+        <v>0.01533763907851522</v>
       </c>
       <c r="L32" s="12" t="n">
-        <v>6610.55</v>
+        <v>6610.7</v>
       </c>
       <c r="M32" s="12" t="n">
-        <v>6806.97</v>
+        <v>6807.01</v>
       </c>
       <c r="N32" s="12" t="n">
-        <v>196.42</v>
+        <v>196.31</v>
       </c>
       <c r="O32" s="13" t="n">
-        <v>0.02971311010430297</v>
+        <v>0.02969579620917603</v>
       </c>
     </row>
     <row r="33">
@@ -8689,7 +9208,7 @@
         <v>46267</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
@@ -8697,40 +9216,40 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>48.1537</v>
+        <v>48.1536</v>
       </c>
       <c r="E33" s="8" t="n">
         <v>48.3568</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>0.2031</v>
+        <v>0.2032</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>0.004217744430853704</v>
+        <v>0.004219829877724615</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>55.7532</v>
+        <v>55.7495</v>
       </c>
       <c r="I33" s="10" t="n">
-        <v>55.9778</v>
+        <v>55.9741</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>0.2246</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>0.004028468321100851</v>
+        <v>0.004028735683728105</v>
       </c>
       <c r="L33" s="12" t="n">
-        <v>6651.71</v>
+        <v>6650.95</v>
       </c>
       <c r="M33" s="12" t="n">
-        <v>6705.14</v>
+        <v>6704.37</v>
       </c>
       <c r="N33" s="12" t="n">
-        <v>53.43</v>
+        <v>53.42</v>
       </c>
       <c r="O33" s="13" t="n">
-        <v>0.0080325209607755</v>
+        <v>0.00803193528744014</v>
       </c>
     </row>
     <row r="34">
@@ -8738,7 +9257,7 @@
         <v>46267</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C34" s="45" t="inlineStr">
         <is>
@@ -8746,40 +9265,40 @@
         </is>
       </c>
       <c r="D34" s="8" t="n">
-        <v>47.8945</v>
+        <v>47.8944</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>48.8555</v>
+        <v>48.8554</v>
       </c>
       <c r="F34" s="8" t="n">
         <v>0.961</v>
       </c>
       <c r="G34" s="9" t="n">
-        <v>0.02006493438703818</v>
+        <v>0.02006497628115187</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>55.4695</v>
+        <v>55.4805</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>56.5715</v>
+        <v>56.5825</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>1.102</v>
       </c>
       <c r="K34" s="11" t="n">
-        <v>0.01986677363235652</v>
+        <v>0.01986283468966574</v>
       </c>
       <c r="L34" s="12" t="n">
-        <v>6611.87</v>
+        <v>6616.12</v>
       </c>
       <c r="M34" s="12" t="n">
-        <v>6756.47</v>
+        <v>6760.72</v>
       </c>
       <c r="N34" s="12" t="n">
         <v>144.6</v>
       </c>
       <c r="O34" s="13" t="n">
-        <v>0.02186975847982492</v>
+        <v>0.0218557099931682</v>
       </c>
     </row>
     <row r="35">
@@ -8787,7 +9306,7 @@
         <v>46267</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C35" s="46" t="inlineStr">
         <is>
@@ -8795,28 +9314,28 @@
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>48.186</v>
+        <v>48.194</v>
       </c>
       <c r="E35" s="8" t="n">
         <v>48.239</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.053</v>
+        <v>0.045</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>0.00109990453658739</v>
+        <v>0.0009337261899821554</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>55.655</v>
+        <v>55.664</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>55.803</v>
+        <v>55.798</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>0.148</v>
+        <v>0.134</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>0.002659239960470757</v>
+        <v>0.002407300948548434</v>
       </c>
       <c r="L35" s="12" t="n"/>
       <c r="M35" s="12" t="n"/>
@@ -8828,7 +9347,7 @@
         <v>46267</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C36" s="47" t="inlineStr">
         <is>
@@ -8860,16 +9379,16 @@
         <v>0.02047472368182642</v>
       </c>
       <c r="L36" s="12" t="n">
-        <v>6582.59</v>
+        <v>6585.46</v>
       </c>
       <c r="M36" s="12" t="n">
-        <v>6784.52</v>
+        <v>6787.98</v>
       </c>
       <c r="N36" s="12" t="n">
-        <v>201.93</v>
+        <v>202.52</v>
       </c>
       <c r="O36" s="13" t="n">
-        <v>0.03067637510463207</v>
+        <v>0.03075259738879289</v>
       </c>
     </row>
     <row r="37">
@@ -8877,7 +9396,7 @@
         <v>46267</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C37" s="48" t="inlineStr">
         <is>
@@ -8897,28 +9416,28 @@
         <v>0.02022948183877804</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>55.4359</v>
+        <v>55.4491</v>
       </c>
       <c r="I37" s="10" t="n">
-        <v>56.5574</v>
+        <v>56.5709</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1.1215</v>
+        <v>1.1218</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>0.02023057260728156</v>
+        <v>0.02023116696213284</v>
       </c>
       <c r="L37" s="12" t="n">
-        <v>6649.04</v>
+        <v>6652.77</v>
       </c>
       <c r="M37" s="12" t="n">
-        <v>6783.29</v>
+        <v>6787.1</v>
       </c>
       <c r="N37" s="12" t="n">
-        <v>134.25</v>
+        <v>134.33</v>
       </c>
       <c r="O37" s="13" t="n">
-        <v>0.02019088469914454</v>
+        <v>0.02019158936803768</v>
       </c>
     </row>
     <row r="38">
@@ -8926,7 +9445,7 @@
         <v>46267</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
@@ -8946,28 +9465,28 @@
         <v>0.01360495969827946</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>55.4499</v>
+        <v>55.4475</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>56.2606</v>
+        <v>56.2582</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>0.8107</v>
       </c>
       <c r="K38" s="11" t="n">
-        <v>0.0146204050863933</v>
+        <v>0.01462103791875197</v>
       </c>
       <c r="L38" s="12" t="n">
-        <v>6619.46</v>
+        <v>6616.73</v>
       </c>
       <c r="M38" s="12" t="n">
-        <v>6753.11</v>
+        <v>6750.33</v>
       </c>
       <c r="N38" s="12" t="n">
-        <v>133.65</v>
+        <v>133.6</v>
       </c>
       <c r="O38" s="13" t="n">
-        <v>0.02019046870892792</v>
+        <v>0.02019124250196094</v>
       </c>
     </row>
     <row r="39">
@@ -8975,7 +9494,7 @@
         <v>46267</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="C39" s="50" t="inlineStr">
         <is>
@@ -8983,40 +9502,40 @@
         </is>
       </c>
       <c r="D39" s="8" t="n">
-        <v>47.7684</v>
+        <v>47.7683</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>48.7651</v>
+        <v>48.7652</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.9967</v>
+        <v>0.9969</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>0.02086525820416845</v>
+        <v>0.02086948876137522</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>55.2759</v>
+        <v>55.2729</v>
       </c>
       <c r="I39" s="10" t="n">
-        <v>56.485</v>
+        <v>56.4822</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1.2091</v>
+        <v>1.2093</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>0.02187390888253289</v>
+        <v>0.02187871452375396</v>
       </c>
       <c r="L39" s="12" t="n">
-        <v>6637.93</v>
+        <v>6638.17</v>
       </c>
       <c r="M39" s="12" t="n">
-        <v>6848.63</v>
+        <v>6848.85</v>
       </c>
       <c r="N39" s="12" t="n">
-        <v>210.7</v>
+        <v>210.68</v>
       </c>
       <c r="O39" s="13" t="n">
-        <v>0.03174182312859582</v>
+        <v>0.03173766263895019</v>
       </c>
     </row>
   </sheetData>
@@ -42318,7 +42837,7 @@
       </c>
       <c r="B5" s="62" t="n"/>
       <c r="C5" s="64" t="n">
-        <v>0.4614699074074074</v>
+        <v>0.4783564814814815</v>
       </c>
       <c r="D5" s="62" t="n"/>
       <c r="F5" s="62" t="inlineStr">
@@ -42402,7 +42921,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="70" t="n">
-        <v>0.02023057260728156</v>
+        <v>0.02023116696213284</v>
       </c>
       <c r="O6" s="71" t="inlineStr">
         <is>
@@ -42410,10 +42929,10 @@
         </is>
       </c>
       <c r="P6" s="72" t="n">
-        <v>55.4359</v>
+        <v>55.4491</v>
       </c>
       <c r="Q6" s="72" t="n">
-        <v>56.5574</v>
+        <v>56.5709</v>
       </c>
     </row>
     <row r="7">
@@ -42455,7 +42974,7 @@
         <v>5</v>
       </c>
       <c r="N7" s="70" t="n">
-        <v>0.02019088469914454</v>
+        <v>0.02019158936803768</v>
       </c>
       <c r="O7" s="71" t="inlineStr">
         <is>
@@ -42463,10 +42982,10 @@
         </is>
       </c>
       <c r="P7" s="72" t="n">
-        <v>6649.04</v>
+        <v>6652.77</v>
       </c>
       <c r="Q7" s="72" t="n">
-        <v>6783.29</v>
+        <v>6787.1</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Günlük kur verisi: 02.09.2026 11:42
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -1009,23 +1009,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -1037,41 +1036,11 @@
           <max val="0.06809845902702412"/>
           <min val="0.01398473878667442"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -1215,23 +1184,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -1243,41 +1211,11 @@
           <max val="0.06361034633532447"/>
           <min val="0.02255547230137524"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -1433,23 +1371,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -1461,41 +1398,11 @@
           <max val="0.06393703694203891"/>
           <min val="0.02251604918664015"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -1651,23 +1558,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -1679,41 +1585,11 @@
           <max val="0.09492887751151027"/>
           <min val="0.02634377435370254"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -1869,23 +1745,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -1897,41 +1772,11 @@
           <max val="0.06300273000209422"/>
           <min val="0.01394771487950567"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -2087,23 +1932,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -2115,41 +1959,11 @@
           <max val="0.05612935000212975"/>
           <min val="0.01451066469310389"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -2305,23 +2119,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -2333,41 +2146,11 @@
           <max val="0.08822748202703072"/>
           <min val="0.0196170269615309"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -2523,23 +2306,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -2551,41 +2333,11 @@
           <max val="0.07017975595934527"/>
           <min val="0.01190344185435327"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -2741,23 +2493,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -2769,41 +2520,11 @@
           <max val="0.07017999927062174"/>
           <min val="0.01190503299558375"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -2959,23 +2680,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -2987,41 +2707,11 @@
           <max val="0.1709612332154084"/>
           <min val="0"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -3177,23 +2867,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -3205,41 +2894,11 @@
           <max val="0.06165859703981922"/>
           <min val="0.01797489899804002"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -3755,23 +3414,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -3783,41 +3441,11 @@
           <max val="0.06809875047508467"/>
           <min val="0.01398628179112082"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -3961,23 +3589,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -3989,41 +3616,11 @@
           <max val="0.06209535841468713"/>
           <min val="0.01791241253707181"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -4179,23 +3776,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -4207,41 +3803,11 @@
           <max val="0.1462720659556508"/>
           <min val="0.007620168856054751"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -4757,23 +4323,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -4785,41 +4350,11 @@
           <max val="0.1646791482454227"/>
           <min val="0.001344939025793405"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -5203,23 +4738,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -5231,41 +4765,11 @@
           <max val="0.05171408776103012"/>
           <min val="0.0161237184650772"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -5649,23 +5153,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -5677,41 +5180,11 @@
           <max val="0.05613143775214488"/>
           <min val="0.01554823152705276"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -6095,23 +5568,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -6123,41 +5595,11 @@
           <max val="0.113954760403876"/>
           <min val="0.007962009561212546"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <legend>
@@ -6301,23 +5743,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -6329,41 +5770,11 @@
           <max val="0.04535890324268219"/>
           <min val="0.02563021945997443"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -6519,23 +5930,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -6547,41 +5957,11 @@
           <max val="0.04536575081521625"/>
           <min val="0.02562858686951813"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -6737,23 +6117,22 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
           <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="700"/>
+              <a:defRPr sz="700" b="1"/>
             </a:pPr>
             <a:r>
               <a:t/>
             </a:r>
-            <a:endParaRPr sz="700"/>
+            <a:endParaRPr sz="700" b="1"/>
           </a:p>
         </txPr>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
         <tickLblSkip val="1"/>
         <tickMarkSkip val="1"/>
@@ -6765,41 +6144,11 @@
           <max val="0.07745416653140928"/>
           <min val="0.03018959592357282"/>
         </scaling>
-        <delete val="0"/>
+        <delete val="1"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Makas %</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="out"/>
+        <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="700"/>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-            <a:endParaRPr sz="700"/>
-          </a:p>
-        </txPr>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
       <spPr>
         <a:solidFill>
@@ -7729,7 +7078,7 @@
         <v>46267</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
@@ -7749,28 +7098,28 @@
         <v>0.02842045430622513</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>55.006</v>
+        <v>55.0059</v>
       </c>
       <c r="I2" s="10" t="n">
-        <v>56.5693</v>
+        <v>56.5692</v>
       </c>
       <c r="J2" s="10" t="n">
         <v>1.5633</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>0.02842053594153365</v>
+        <v>0.02842058760969278</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>6539.92</v>
+        <v>6536.37</v>
       </c>
       <c r="M2" s="12" t="n">
-        <v>6776.25</v>
+        <v>6772.41</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>236.33</v>
+        <v>236.04</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>0.03613652766394695</v>
+        <v>0.03611178681745372</v>
       </c>
     </row>
     <row r="3">
@@ -7778,7 +7127,7 @@
         <v>46267</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
@@ -7798,28 +7147,28 @@
         <v>0.01630582291166461</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>55.464</v>
+        <v>55.469</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>56.374</v>
+        <v>56.384</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.91</v>
+        <v>0.915</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>0.01640703879994231</v>
+        <v>0.01649570030106906</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>6613.3</v>
+        <v>6614.98</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>6749.32</v>
+        <v>6751.04</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>136.02</v>
+        <v>136.06</v>
       </c>
       <c r="O3" s="13" t="n">
-        <v>0.02056764399014108</v>
+        <v>0.02056846732718769</v>
       </c>
     </row>
     <row r="4">
@@ -7827,7 +7176,7 @@
         <v>46267</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -7835,40 +7184,40 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>48.079</v>
+        <v>48.078</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>48.376</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.297</v>
+        <v>0.298</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>0.006177333139208386</v>
+        <v>0.006198261158950039</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>55.504</v>
+        <v>55.509</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>56.022</v>
+        <v>56.023</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.518</v>
+        <v>0.514</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>0.009332660709138079</v>
+        <v>0.009259759678610676</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>6674.93</v>
+        <v>6673.88</v>
       </c>
       <c r="M4" s="12" t="n">
-        <v>6742.97</v>
+        <v>6741.22</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>68.04000000000001</v>
+        <v>67.34</v>
       </c>
       <c r="O4" s="13" t="n">
-        <v>0.0101933653236813</v>
+        <v>0.01009008253070178</v>
       </c>
     </row>
     <row r="5">
@@ -7876,7 +7225,7 @@
         <v>46267</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -7896,28 +7245,28 @@
         <v>0.004363183045917307</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>55.621</v>
+        <v>55.63</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>55.976</v>
+        <v>55.984</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.355</v>
+        <v>0.354</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>0.00638248143686737</v>
+        <v>0.006363472946252022</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>6583.96</v>
+        <v>6588.32</v>
       </c>
       <c r="M5" s="12" t="n">
         <v>6775</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>191.04</v>
+        <v>186.68</v>
       </c>
       <c r="O5" s="13" t="n">
-        <v>0.02901597215049909</v>
+        <v>0.0283349928358064</v>
       </c>
     </row>
     <row r="6">
@@ -7925,7 +7274,7 @@
         <v>46267</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
@@ -7936,37 +7285,37 @@
         <v>47.4528</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>48.7293</v>
+        <v>48.729</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>1.2765</v>
+        <v>1.2762</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.02690041472789804</v>
+        <v>0.02689409265628161</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>55.0511</v>
+        <v>55.0575</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>56.4161</v>
+        <v>56.422</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>1.365</v>
+        <v>1.3645</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0.02479514487448934</v>
+        <v>0.02478318121963402</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>6596.32</v>
+        <v>6598.14</v>
       </c>
       <c r="M6" s="12" t="n">
-        <v>6747.3</v>
+        <v>6749.04</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>150.98</v>
+        <v>150.9</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>0.02288851965944648</v>
+        <v>0.02287008156844201</v>
       </c>
     </row>
     <row r="7">
@@ -7974,7 +7323,7 @@
         <v>46267</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
@@ -7994,28 +7343,28 @@
         <v>0.04065367214916916</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>54.772</v>
+        <v>54.781</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>57.007</v>
+        <v>57.012</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>2.235</v>
+        <v>2.231</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>0.04080552106915943</v>
+        <v>0.04072579909092568</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>6593.35</v>
+        <v>6594.98</v>
       </c>
       <c r="M7" s="12" t="n">
-        <v>6787.56</v>
+        <v>6789.19</v>
       </c>
       <c r="N7" s="12" t="n">
         <v>194.21</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>0.02945543615916037</v>
+        <v>0.02944815602170135</v>
       </c>
     </row>
     <row r="8">
@@ -8023,7 +7372,7 @@
         <v>46267</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
@@ -8043,28 +7392,28 @@
         <v>0.02944182290746675</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>55.068</v>
+        <v>55.0775</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>56.6893</v>
+        <v>56.6991</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>1.6213</v>
+        <v>1.6216</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>0.02944178107067625</v>
+        <v>0.0294421496981526</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>6610.78</v>
+        <v>6611.71</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>6806.45</v>
+        <v>6807.36</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>195.67</v>
+        <v>195.65</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>0.02959862527568608</v>
+        <v>0.02959143701100018</v>
       </c>
     </row>
     <row r="9">
@@ -8072,7 +7421,7 @@
         <v>46267</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -8080,40 +7429,40 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>48.2242</v>
+        <v>48.2241</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>48.2817</v>
+        <v>48.281</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.0575</v>
+        <v>0.0569</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.001192347410636154</v>
+        <v>0.001179907971325541</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>55.8326</v>
+        <v>55.8376</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>55.9161</v>
+        <v>55.9206</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.0835</v>
+        <v>0.083</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>0.00149554203099981</v>
+        <v>0.001486453572503116</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6662.85</v>
+        <v>6665.67</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>6691.74</v>
+        <v>6694.52</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>28.89</v>
+        <v>28.85</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>0.004335982349895314</v>
+        <v>0.004328147057985169</v>
       </c>
     </row>
     <row r="10">
@@ -8121,7 +7470,7 @@
         <v>46267</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -8129,40 +7478,40 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>48.2377</v>
+        <v>48.2378</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>48.2759</v>
+        <v>48.2758</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.0382</v>
+        <v>0.038</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.0007919117205007701</v>
+        <v>0.0007877639527507474</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>55.8099</v>
+        <v>55.815</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>55.919</v>
+        <v>55.9286</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.1091</v>
+        <v>0.1136</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>0.001954850304336686</v>
+        <v>0.002035295171548867</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>6659.12</v>
+        <v>6661.29</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>6690.78</v>
+        <v>6692.94</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>31.66</v>
+        <v>31.65</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>0.00475438196037915</v>
+        <v>0.004751331949217044</v>
       </c>
     </row>
     <row r="11">
@@ -8170,7 +7519,7 @@
         <v>46267</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
@@ -8178,40 +7527,40 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>47.9239</v>
+        <v>47.924</v>
       </c>
       <c r="E11" s="8" t="n">
         <v>49.1614</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1.2375</v>
+        <v>1.2374</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.02582218892869738</v>
+        <v>0.02582004840998247</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>55.3879</v>
+        <v>55.4024</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>56.6663</v>
+        <v>56.681</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>1.2784</v>
+        <v>1.2786</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>0.02308085339938867</v>
+        <v>0.02307842259541103</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6614.87</v>
+        <v>6614.85</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>6723.1</v>
+        <v>6723.08</v>
       </c>
       <c r="N11" s="12" t="n">
         <v>108.23</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>0.01636162161917014</v>
+        <v>0.01636167108853564</v>
       </c>
     </row>
     <row r="12">
@@ -8219,7 +7568,7 @@
         <v>46267</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
@@ -8242,25 +7591,25 @@
         <v>55.3195</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>56.4812</v>
+        <v>56.4909</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>1.1617</v>
+        <v>1.1714</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>0.02099982827032059</v>
+        <v>0.02117517331140014</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>6607.97</v>
+        <v>6609.94</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>6762.41</v>
+        <v>6764.43</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>154.44</v>
+        <v>154.49</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>0.02337177680891408</v>
+        <v>0.02337237554349964</v>
       </c>
     </row>
     <row r="13">
@@ -8268,7 +7617,7 @@
         <v>46267</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
@@ -8276,40 +7625,40 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>47.9981</v>
+        <v>47.9979</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>48.6053</v>
+        <v>48.6049</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.6072</v>
+        <v>0.607</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.01265050074898798</v>
+        <v>0.01264638661274764</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>55.5975</v>
+        <v>55.5966</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>56.2586</v>
+        <v>56.2577</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>0.6611</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>0.01189082242906605</v>
+        <v>0.01189101491817845</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6683.82</v>
+        <v>6678.06</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>6738.14</v>
+        <v>6732.35</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>54.32</v>
+        <v>54.29</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>0.008127089000002993</v>
+        <v>0.008129606502487249</v>
       </c>
     </row>
     <row r="14">
@@ -8317,7 +7666,7 @@
         <v>46267</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
@@ -8349,16 +7698,16 @@
         <v>0.02844300480419275</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>6577.16</v>
+        <v>6573.4</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>6820.13</v>
+        <v>6816.24</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>242.97</v>
+        <v>242.84</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>0.03694147626027039</v>
+        <v>0.03694283019441993</v>
       </c>
     </row>
     <row r="15">
@@ -8366,7 +7715,7 @@
         <v>46267</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
@@ -8374,40 +7723,40 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>47.998</v>
+        <v>47.9979</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>48.6051</v>
+        <v>48.6049</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.6071</v>
+        <v>0.607</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>0.01264844368515355</v>
+        <v>0.01264638661274764</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>55.5959</v>
+        <v>55.6023</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>56.2564</v>
+        <v>56.2623</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>0.6605</v>
+        <v>0.66</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>0.01188037247350974</v>
+        <v>0.01187001257142241</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>6680.4</v>
+        <v>6681.92</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>6734.79</v>
+        <v>6736.04</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>54.39</v>
+        <v>54.12</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>0.008141728040237111</v>
+        <v>0.008099468416263588</v>
       </c>
     </row>
     <row r="16">
@@ -8415,7 +7764,7 @@
         <v>46267</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
@@ -8435,28 +7784,28 @@
         <v>0.02047330948958786</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>55.4302</v>
+        <v>55.4422</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>56.5651</v>
+        <v>56.5773</v>
       </c>
       <c r="J16" s="10" t="n">
-        <v>1.1349</v>
+        <v>1.1351</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>0.02047439843262337</v>
+        <v>0.02047357428096288</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>6613.91</v>
+        <v>6614.91</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>6817.49</v>
+        <v>6818.07</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>203.58</v>
+        <v>203.16</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>0.03078058213673908</v>
+        <v>0.03071243599686163</v>
       </c>
     </row>
     <row r="17">
@@ -8464,7 +7813,7 @@
         <v>46267</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
@@ -8472,40 +7821,40 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>48.183</v>
+        <v>48.1928</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>48.242</v>
+        <v>48.2518</v>
       </c>
       <c r="F17" s="8" t="n">
         <v>0.059</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.001224498267023639</v>
+        <v>0.001224249265450441</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>55.643</v>
+        <v>55.672</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>55.811</v>
+        <v>55.839</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>0.168</v>
+        <v>0.167</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>0.003019247704113725</v>
+        <v>0.002999712602385401</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>6610.07</v>
+        <v>6611.85</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>6705</v>
+        <v>6706.82</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>94.93000000000001</v>
+        <v>94.97</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>0.01436142128600756</v>
+        <v>0.01436360473997444</v>
       </c>
     </row>
     <row r="18">
@@ -8513,7 +7862,7 @@
         <v>46267</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
@@ -8521,40 +7870,40 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>48.2181</v>
+        <v>48.2178</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>48.3643</v>
+        <v>48.364</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>0.1462</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.003032056426943409</v>
+        <v>0.003032075291697257</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>55.8231</v>
+        <v>55.828</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>55.9943</v>
+        <v>55.999</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>0.1712</v>
+        <v>0.171</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>0.003066830756443121</v>
+        <v>0.003062979150247187</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>6669.56</v>
+        <v>6672.81</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>6716.68</v>
+        <v>6719.89</v>
       </c>
       <c r="N18" s="12" t="n">
-        <v>47.12</v>
+        <v>47.08</v>
       </c>
       <c r="O18" s="13" t="n">
-        <v>0.007064933818722674</v>
+        <v>0.007055498358262861</v>
       </c>
     </row>
     <row r="19">
@@ -8562,7 +7911,7 @@
         <v>46267</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
@@ -8578,16 +7927,16 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="12" t="n">
-        <v>6685.53</v>
+        <v>6684.59</v>
       </c>
       <c r="M19" s="12" t="n">
-        <v>6881.39</v>
+        <v>6880.44</v>
       </c>
       <c r="N19" s="12" t="n">
-        <v>195.86</v>
+        <v>195.85</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>0.02929610666618802</v>
+        <v>0.02929873036341795</v>
       </c>
     </row>
     <row r="20">
@@ -8595,7 +7944,7 @@
         <v>46267</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C20" s="31" t="inlineStr">
         <is>
@@ -8603,40 +7952,40 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>47.8071</v>
+        <v>47.8064</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>48.6877</v>
+        <v>48.6889</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0.8806</v>
+        <v>0.8825</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>0.01841985813822633</v>
+        <v>0.01845987148164262</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>55.3609</v>
+        <v>55.3698</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>56.4133</v>
+        <v>56.4197</v>
       </c>
       <c r="J20" s="10" t="n">
-        <v>1.0524</v>
+        <v>1.0499</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>0.01900980656022572</v>
+        <v>0.01896160000577932</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>6613.08</v>
+        <v>6614.8</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>7057.74</v>
+        <v>7060.2</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>444.66</v>
+        <v>445.4</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>0.06723947086682756</v>
+        <v>0.0673338574106549</v>
       </c>
     </row>
     <row r="21">
@@ -8644,7 +7993,7 @@
         <v>46267</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
@@ -8652,40 +8001,40 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>47.7514</v>
+        <v>47.7513</v>
       </c>
       <c r="E21" s="8" t="n">
         <v>48.7543</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.0029</v>
+        <v>1.003</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.02100252558040183</v>
+        <v>0.02100466374737442</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>55.3718</v>
+        <v>55.3789</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>56.3808</v>
+        <v>56.3854</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>1.009</v>
+        <v>1.0065</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>0.01822227198682362</v>
+        <v>0.01817479220425108</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>6581.47</v>
+        <v>6582.5</v>
       </c>
       <c r="M21" s="12" t="n">
-        <v>6833.43</v>
+        <v>6834.42</v>
       </c>
       <c r="N21" s="12" t="n">
-        <v>251.96</v>
+        <v>251.92</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>0.03828324067419588</v>
+        <v>0.03827117356627421</v>
       </c>
     </row>
     <row r="22">
@@ -8693,7 +8042,7 @@
         <v>46267</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -8713,28 +8062,28 @@
         <v>0.02422275962020458</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>55.202</v>
+        <v>55.2115</v>
       </c>
       <c r="I22" s="10" t="n">
         <v>56.5488</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>1.3468</v>
+        <v>1.3373</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>0.02439766675120467</v>
+        <v>0.02422140314970613</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>6604.18</v>
+        <v>6601.95</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>6785.28</v>
+        <v>6783.02</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>181.1</v>
+        <v>181.07</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>0.02742202665584524</v>
+        <v>0.0274267451283333</v>
       </c>
     </row>
     <row r="23">
@@ -8742,7 +8091,7 @@
         <v>46267</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C23" s="34" t="inlineStr">
         <is>
@@ -8791,7 +8140,7 @@
         <v>46267</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
@@ -8799,40 +8148,40 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>47.6129</v>
+        <v>47.6865</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>48.5986</v>
+        <v>48.6724</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>0.9857</v>
+        <v>0.9859</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.02070237267631251</v>
+        <v>0.02067461440869009</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>55.1334</v>
+        <v>55.1413</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>56.2772</v>
+        <v>56.2835</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>1.1438</v>
+        <v>1.1422</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>0.02074604504710393</v>
+        <v>0.0207140564331998</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>6561.48</v>
+        <v>6563.64</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>6735.43</v>
+        <v>6737.46</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>173.95</v>
+        <v>173.82</v>
       </c>
       <c r="O24" s="13" t="n">
-        <v>0.02651078720044868</v>
+        <v>0.02648225679653363</v>
       </c>
     </row>
     <row r="25">
@@ -8840,7 +8189,7 @@
         <v>46267</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
@@ -8881,7 +8230,7 @@
         <v>46267</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
@@ -8889,40 +8238,40 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>48.227</v>
+        <v>48.2269</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>48.2796</v>
+        <v>48.2797</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>0.0526</v>
+        <v>0.0528</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>0.001090675347834201</v>
+        <v>0.001094824672537526</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>55.8305</v>
+        <v>55.8388</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>55.9073</v>
+        <v>55.9157</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>0.07679999999999999</v>
+        <v>0.0769</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>0.001375592194230752</v>
+        <v>0.001377178592663166</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>6658.35</v>
+        <v>6661.79</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>6687.13</v>
+        <v>6690.54</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>28.78</v>
+        <v>28.75</v>
       </c>
       <c r="O26" s="13" t="n">
-        <v>0.004322392184249852</v>
+        <v>0.004315656903024562</v>
       </c>
     </row>
     <row r="27">
@@ -8930,7 +8279,7 @@
         <v>46267</v>
       </c>
       <c r="B27" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C27" s="38" t="inlineStr">
         <is>
@@ -8938,40 +8287,40 @@
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>48.182</v>
+        <v>48.192</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>48.285</v>
+        <v>48.291</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.103</v>
+        <v>0.099</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>0.002137727782159313</v>
+        <v>0.002054282868525896</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>55.652</v>
+        <v>55.665</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>55.883</v>
+        <v>55.904</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>0.231</v>
+        <v>0.239</v>
       </c>
       <c r="K27" s="11" t="n">
-        <v>0.004150794221231942</v>
+        <v>0.004293541722806072</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>6623</v>
+        <v>6624</v>
       </c>
       <c r="M27" s="12" t="n">
-        <v>6683</v>
+        <v>6686</v>
       </c>
       <c r="N27" s="12" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>0.009059338668277217</v>
+        <v>0.009359903381642512</v>
       </c>
     </row>
     <row r="28">
@@ -8979,7 +8328,7 @@
         <v>46267</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -8999,28 +8348,28 @@
         <v>0.0209375850589393</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>55.337</v>
+        <v>55.344</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>56.427</v>
+        <v>56.434</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>1.09</v>
       </c>
       <c r="K28" s="11" t="n">
-        <v>0.01969748992536639</v>
+        <v>0.01969499855449552</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>6662.57</v>
+        <v>6655.57</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>6762.57</v>
+        <v>6755.57</v>
       </c>
       <c r="N28" s="12" t="n">
         <v>100</v>
       </c>
       <c r="O28" s="13" t="n">
-        <v>0.01500922316763651</v>
+        <v>0.01502500912769305</v>
       </c>
     </row>
     <row r="29">
@@ -9028,7 +8377,7 @@
         <v>46267</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
@@ -9044,16 +8393,16 @@
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="12" t="n">
-        <v>6686.42</v>
+        <v>6684.49</v>
       </c>
       <c r="M29" s="12" t="n">
-        <v>6868.55</v>
+        <v>6866.61</v>
       </c>
       <c r="N29" s="12" t="n">
-        <v>182.13</v>
+        <v>182.12</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>0.02723879146090135</v>
+        <v>0.02724516006456738</v>
       </c>
     </row>
     <row r="30">
@@ -9061,7 +8410,7 @@
         <v>46267</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C30" s="41" t="inlineStr">
         <is>
@@ -9081,28 +8430,28 @@
         <v>0.02558322411533421</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>55.1014</v>
+        <v>55.1109</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>56.7587</v>
+        <v>56.7636</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>1.6573</v>
+        <v>1.6527</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>0.03007727571350274</v>
+        <v>0.02998862294028949</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>6581.7</v>
+        <v>6584.82</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>6779.29</v>
+        <v>6782.96</v>
       </c>
       <c r="N30" s="12" t="n">
-        <v>197.59</v>
+        <v>198.14</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>0.03002111916374189</v>
+        <v>0.03009042008741317</v>
       </c>
     </row>
     <row r="31">
@@ -9110,7 +8459,7 @@
         <v>46267</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -9118,10 +8467,10 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>48.2768</v>
+        <v>48.297</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>48.2768</v>
+        <v>48.297</v>
       </c>
       <c r="F31" s="8" t="n">
         <v>0</v>
@@ -9130,10 +8479,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>55.9056</v>
+        <v>55.9351</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>55.9056</v>
+        <v>55.9351</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>0</v>
@@ -9142,10 +8491,10 @@
         <v>0</v>
       </c>
       <c r="L31" s="12" t="n">
-        <v>6677.96</v>
+        <v>6682.99</v>
       </c>
       <c r="M31" s="12" t="n">
-        <v>6677.96</v>
+        <v>6682.99</v>
       </c>
       <c r="N31" s="12" t="n">
         <v>0</v>
@@ -9159,7 +8508,7 @@
         <v>46267</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C32" s="43" t="inlineStr">
         <is>
@@ -9170,37 +8519,37 @@
         <v>47.8519</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>48.6538</v>
+        <v>48.6536</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.8018999999999999</v>
+        <v>0.8017</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>0.01675795527450321</v>
+        <v>0.01675377571214518</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>55.4453</v>
+        <v>55.4553</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>56.2957</v>
+        <v>56.3054</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>0.8504</v>
+        <v>0.8501</v>
       </c>
       <c r="K32" s="11" t="n">
-        <v>0.01533763907851522</v>
+        <v>0.01532946354992219</v>
       </c>
       <c r="L32" s="12" t="n">
-        <v>6610.7</v>
+        <v>6614.04</v>
       </c>
       <c r="M32" s="12" t="n">
-        <v>6807.01</v>
+        <v>6810.1</v>
       </c>
       <c r="N32" s="12" t="n">
-        <v>196.31</v>
+        <v>196.06</v>
       </c>
       <c r="O32" s="13" t="n">
-        <v>0.02969579620917603</v>
+        <v>0.02964300185665645</v>
       </c>
     </row>
     <row r="33">
@@ -9208,7 +8557,7 @@
         <v>46267</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
@@ -9228,28 +8577,28 @@
         <v>0.004219829877724615</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>55.7495</v>
+        <v>55.759</v>
       </c>
       <c r="I33" s="10" t="n">
-        <v>55.9741</v>
+        <v>55.9836</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>0.2246</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>0.004028735683728105</v>
+        <v>0.004028049283523735</v>
       </c>
       <c r="L33" s="12" t="n">
-        <v>6650.95</v>
+        <v>6649.89</v>
       </c>
       <c r="M33" s="12" t="n">
-        <v>6704.37</v>
+        <v>6703.31</v>
       </c>
       <c r="N33" s="12" t="n">
         <v>53.42</v>
       </c>
       <c r="O33" s="13" t="n">
-        <v>0.00803193528744014</v>
+        <v>0.008033215587024748</v>
       </c>
     </row>
     <row r="34">
@@ -9257,7 +8606,7 @@
         <v>46267</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C34" s="45" t="inlineStr">
         <is>
@@ -9265,40 +8614,40 @@
         </is>
       </c>
       <c r="D34" s="8" t="n">
-        <v>47.8944</v>
+        <v>47.8942</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>48.8554</v>
+        <v>48.8552</v>
       </c>
       <c r="F34" s="8" t="n">
         <v>0.961</v>
       </c>
       <c r="G34" s="9" t="n">
-        <v>0.02006497628115187</v>
+        <v>0.02006506006990408</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>55.4805</v>
+        <v>55.4892</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>56.5825</v>
+        <v>56.5913</v>
       </c>
       <c r="J34" s="10" t="n">
-        <v>1.102</v>
+        <v>1.1021</v>
       </c>
       <c r="K34" s="11" t="n">
-        <v>0.01986283468966574</v>
+        <v>0.01986152260259654</v>
       </c>
       <c r="L34" s="12" t="n">
-        <v>6616.12</v>
+        <v>6615.97</v>
       </c>
       <c r="M34" s="12" t="n">
-        <v>6760.72</v>
+        <v>6760.57</v>
       </c>
       <c r="N34" s="12" t="n">
         <v>144.6</v>
       </c>
       <c r="O34" s="13" t="n">
-        <v>0.0218557099931682</v>
+        <v>0.02185620551483758</v>
       </c>
     </row>
     <row r="35">
@@ -9306,7 +8655,7 @@
         <v>46267</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C35" s="46" t="inlineStr">
         <is>
@@ -9314,28 +8663,28 @@
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>48.194</v>
+        <v>48.199</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>48.239</v>
+        <v>48.25</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.045</v>
+        <v>0.051</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>0.0009337261899821554</v>
+        <v>0.001058113238863877</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>55.664</v>
+        <v>55.69</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>55.798</v>
+        <v>55.819</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>0.134</v>
+        <v>0.129</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>0.002407300948548434</v>
+        <v>0.002316394325731729</v>
       </c>
       <c r="L35" s="12" t="n"/>
       <c r="M35" s="12" t="n"/>
@@ -9347,7 +8696,7 @@
         <v>46267</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C36" s="47" t="inlineStr">
         <is>
@@ -9370,25 +8719,25 @@
         <v>55.19</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>56.32</v>
+        <v>56.33</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="K36" s="11" t="n">
-        <v>0.02047472368182642</v>
+        <v>0.02065591592679833</v>
       </c>
       <c r="L36" s="12" t="n">
-        <v>6585.46</v>
+        <v>6584.14</v>
       </c>
       <c r="M36" s="12" t="n">
-        <v>6787.98</v>
+        <v>6786.1</v>
       </c>
       <c r="N36" s="12" t="n">
-        <v>202.52</v>
+        <v>201.96</v>
       </c>
       <c r="O36" s="13" t="n">
-        <v>0.03075259738879289</v>
+        <v>0.03067370985428621</v>
       </c>
     </row>
     <row r="37">
@@ -9396,7 +8745,7 @@
         <v>46267</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C37" s="48" t="inlineStr">
         <is>
@@ -9416,28 +8765,28 @@
         <v>0.02022948183877804</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>55.4491</v>
+        <v>55.4447</v>
       </c>
       <c r="I37" s="10" t="n">
-        <v>56.5709</v>
+        <v>56.5664</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1.1218</v>
+        <v>1.1217</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>0.02023116696213284</v>
+        <v>0.02023096887529376</v>
       </c>
       <c r="L37" s="12" t="n">
-        <v>6652.77</v>
+        <v>6646.78</v>
       </c>
       <c r="M37" s="12" t="n">
-        <v>6787.1</v>
+        <v>6780.98</v>
       </c>
       <c r="N37" s="12" t="n">
-        <v>134.33</v>
+        <v>134.2</v>
       </c>
       <c r="O37" s="13" t="n">
-        <v>0.02019158936803768</v>
+        <v>0.02019022744847881</v>
       </c>
     </row>
     <row r="38">
@@ -9445,7 +8794,7 @@
         <v>46267</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
@@ -9465,28 +8814,28 @@
         <v>0.01360495969827946</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>55.4475</v>
+        <v>55.4571</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>56.2582</v>
+        <v>56.2678</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>0.8107</v>
       </c>
       <c r="K38" s="11" t="n">
-        <v>0.01462103791875197</v>
+        <v>0.01461850691796001</v>
       </c>
       <c r="L38" s="12" t="n">
-        <v>6616.73</v>
+        <v>6618.5</v>
       </c>
       <c r="M38" s="12" t="n">
-        <v>6750.33</v>
+        <v>6752.13</v>
       </c>
       <c r="N38" s="12" t="n">
-        <v>133.6</v>
+        <v>133.63</v>
       </c>
       <c r="O38" s="13" t="n">
-        <v>0.02019124250196094</v>
+        <v>0.02019037546271814</v>
       </c>
     </row>
     <row r="39">
@@ -9494,7 +8843,7 @@
         <v>46267</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="C39" s="50" t="inlineStr">
         <is>
@@ -9505,37 +8854,37 @@
         <v>47.7683</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>48.7652</v>
+        <v>48.7651</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.9969</v>
+        <v>0.9968</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>0.02086948876137522</v>
+        <v>0.02086739532283962</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>55.2729</v>
+        <v>55.2806</v>
       </c>
       <c r="I39" s="10" t="n">
-        <v>56.4822</v>
+        <v>56.4894</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1.2093</v>
+        <v>1.2088</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>0.02187871452375396</v>
+        <v>0.02186662228702293</v>
       </c>
       <c r="L39" s="12" t="n">
-        <v>6638.17</v>
+        <v>6639.21</v>
       </c>
       <c r="M39" s="12" t="n">
-        <v>6848.85</v>
+        <v>6850.01</v>
       </c>
       <c r="N39" s="12" t="n">
-        <v>210.68</v>
+        <v>210.8</v>
       </c>
       <c r="O39" s="13" t="n">
-        <v>0.03173766263895019</v>
+        <v>0.03175076552782635</v>
       </c>
     </row>
   </sheetData>
@@ -42837,7 +42186,7 @@
       </c>
       <c r="B5" s="62" t="n"/>
       <c r="C5" s="64" t="n">
-        <v>0.4783564814814815</v>
+        <v>0.4871875</v>
       </c>
       <c r="D5" s="62" t="n"/>
       <c r="F5" s="62" t="inlineStr">
@@ -42921,7 +42270,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="70" t="n">
-        <v>0.02023116696213284</v>
+        <v>0.02023096887529376</v>
       </c>
       <c r="O6" s="71" t="inlineStr">
         <is>
@@ -42929,10 +42278,10 @@
         </is>
       </c>
       <c r="P6" s="72" t="n">
-        <v>55.4491</v>
+        <v>55.4447</v>
       </c>
       <c r="Q6" s="72" t="n">
-        <v>56.5709</v>
+        <v>56.5664</v>
       </c>
     </row>
     <row r="7">
@@ -42974,7 +42323,7 @@
         <v>5</v>
       </c>
       <c r="N7" s="70" t="n">
-        <v>0.02019158936803768</v>
+        <v>0.02019022744847881</v>
       </c>
       <c r="O7" s="71" t="inlineStr">
         <is>
@@ -42982,10 +42331,10 @@
         </is>
       </c>
       <c r="P7" s="72" t="n">
-        <v>6652.77</v>
+        <v>6646.78</v>
       </c>
       <c r="Q7" s="72" t="n">
-        <v>6787.1</v>
+        <v>6780.98</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Günlük kur verisi: 02.09.2026 12:00
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -585,10 +585,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -677,10 +677,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -769,10 +769,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -861,10 +861,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -953,10 +953,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -1120,10 +1120,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -1307,10 +1307,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -1494,10 +1494,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -1681,10 +1681,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -1868,10 +1868,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -2055,10 +2055,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -2242,10 +2242,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -2429,10 +2429,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -2616,10 +2616,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -2803,10 +2803,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -2990,10 +2990,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -3082,10 +3082,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -3174,10 +3174,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -3266,10 +3266,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -3358,10 +3358,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -3525,10 +3525,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -3712,10 +3712,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -3899,10 +3899,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -3991,10 +3991,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -4083,10 +4083,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -4175,10 +4175,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -4267,10 +4267,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -5679,10 +5679,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -5866,10 +5866,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -6053,10 +6053,10 @@
                   <v>28.08</v>
                 </pt>
                 <pt idx="1">
-                  <v>29.08 Cmt</v>
+                  <v>🔵 29.08 Cmt</v>
                 </pt>
                 <pt idx="2">
-                  <v>30.08 Paz</v>
+                  <v>🔴 30.08 Paz</v>
                 </pt>
                 <pt idx="3">
                   <v>31.08</v>
@@ -7078,7 +7078,7 @@
         <v>46267</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
@@ -7098,28 +7098,28 @@
         <v>0.02842045430622513</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>55.0059</v>
+        <v>54.9729</v>
       </c>
       <c r="I2" s="10" t="n">
-        <v>56.5692</v>
+        <v>56.5401</v>
       </c>
       <c r="J2" s="10" t="n">
-        <v>1.5633</v>
+        <v>1.5672</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>0.02842058760969278</v>
+        <v>0.02850859241553565</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>6536.37</v>
+        <v>6523.14</v>
       </c>
       <c r="M2" s="12" t="n">
-        <v>6772.41</v>
+        <v>6758.76</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>236.04</v>
+        <v>235.62</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>0.03611178681745372</v>
+        <v>0.03612064128625171</v>
       </c>
     </row>
     <row r="3">
@@ -7127,7 +7127,7 @@
         <v>46267</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
@@ -7147,28 +7147,28 @@
         <v>0.01630582291166461</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>55.469</v>
+        <v>55.426</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>56.384</v>
+        <v>56.34</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.915</v>
+        <v>0.914</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>0.01649570030106906</v>
+        <v>0.01649045574279219</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>6614.98</v>
+        <v>6598.1</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>6751.04</v>
+        <v>6733.81</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>136.06</v>
+        <v>135.71</v>
       </c>
       <c r="O3" s="13" t="n">
-        <v>0.02056846732718769</v>
+        <v>0.02056804231521196</v>
       </c>
     </row>
     <row r="4">
@@ -7176,7 +7176,7 @@
         <v>46267</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -7184,40 +7184,40 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>48.078</v>
+        <v>48.081</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>48.376</v>
+        <v>48.374</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.298</v>
+        <v>0.293</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>0.006198261158950039</v>
+        <v>0.006093883238701359</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>55.509</v>
+        <v>55.476</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>56.023</v>
+        <v>55.988</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.514</v>
+        <v>0.512</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>0.009259759678610676</v>
+        <v>0.009229216237652318</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>6673.88</v>
+        <v>6663.21</v>
       </c>
       <c r="M4" s="12" t="n">
-        <v>6741.22</v>
+        <v>6729.36</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>67.34</v>
+        <v>66.15000000000001</v>
       </c>
       <c r="O4" s="13" t="n">
-        <v>0.01009008253070178</v>
+        <v>0.009927647485221087</v>
       </c>
     </row>
     <row r="5">
@@ -7225,7 +7225,7 @@
         <v>46267</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -7236,37 +7236,37 @@
         <v>48.13</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>48.34</v>
+        <v>48.33</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>0.004363183045917307</v>
+        <v>0.00415541242468315</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>55.63</v>
+        <v>55.594</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>55.984</v>
+        <v>55.938</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.354</v>
+        <v>0.344</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>0.006363472946252022</v>
+        <v>0.00618771809907544</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>6588.32</v>
+        <v>6572.1</v>
       </c>
       <c r="M5" s="12" t="n">
-        <v>6775</v>
+        <v>6755</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>186.68</v>
+        <v>182.9</v>
       </c>
       <c r="O5" s="13" t="n">
-        <v>0.0283349928358064</v>
+        <v>0.0278297652196406</v>
       </c>
     </row>
     <row r="6">
@@ -7274,7 +7274,7 @@
         <v>46267</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
@@ -7282,40 +7282,40 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>47.4528</v>
+        <v>47.4534</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>48.729</v>
+        <v>48.7297</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>1.2762</v>
+        <v>1.2763</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.02689409265628161</v>
+        <v>0.02689585993838166</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>55.0575</v>
+        <v>55.0203</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>56.422</v>
+        <v>56.3848</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>1.3645</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0.02478318121963402</v>
+        <v>0.02479993747762189</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>6598.14</v>
+        <v>6581.24</v>
       </c>
       <c r="M6" s="12" t="n">
-        <v>6749.04</v>
+        <v>6732.31</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>150.9</v>
+        <v>151.07</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>0.02287008156844201</v>
+        <v>0.02295464076678559</v>
       </c>
     </row>
     <row r="7">
@@ -7323,7 +7323,7 @@
         <v>46267</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
@@ -7343,28 +7343,28 @@
         <v>0.04065367214916916</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>54.781</v>
+        <v>54.743</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>57.012</v>
+        <v>56.973</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>2.231</v>
+        <v>2.23</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>0.04072579909092568</v>
+        <v>0.04073580183767787</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>6594.98</v>
+        <v>6578.25</v>
       </c>
       <c r="M7" s="12" t="n">
-        <v>6789.19</v>
+        <v>6772.46</v>
       </c>
       <c r="N7" s="12" t="n">
         <v>194.21</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>0.02944815602170135</v>
+        <v>0.02952304944324098</v>
       </c>
     </row>
     <row r="8">
@@ -7372,7 +7372,7 @@
         <v>46267</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
@@ -7380,40 +7380,40 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>47.5548</v>
+        <v>47.5551</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>48.9549</v>
+        <v>48.9552</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>1.4001</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>0.02944182290746675</v>
+        <v>0.02944163717456172</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>55.0775</v>
+        <v>55.0398</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>56.6991</v>
+        <v>56.6603</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>1.6216</v>
+        <v>1.6205</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>0.0294421496981526</v>
+        <v>0.02944233082242305</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>6611.71</v>
+        <v>6595.09</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>6807.36</v>
+        <v>6790.33</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>195.65</v>
+        <v>195.24</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>0.02959143701100018</v>
+        <v>0.02960384164583046</v>
       </c>
     </row>
     <row r="9">
@@ -7421,7 +7421,7 @@
         <v>46267</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -7429,40 +7429,40 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>48.2241</v>
+        <v>48.2247</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>48.281</v>
+        <v>48.2816</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>0.0569</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.001179907971325541</v>
+        <v>0.001179893291197249</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>55.8376</v>
+        <v>55.7992</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>55.9206</v>
+        <v>55.8824</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.083</v>
+        <v>0.0832</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>0.001486453572503116</v>
+        <v>0.001491060803739122</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6665.67</v>
+        <v>6648.06</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>6694.52</v>
+        <v>6676.93</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>28.85</v>
+        <v>28.87</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>0.004328147057985169</v>
+        <v>0.004342620253126477</v>
       </c>
     </row>
     <row r="10">
@@ -7470,7 +7470,7 @@
         <v>46267</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -7478,40 +7478,40 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>48.2378</v>
+        <v>48.2382</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>48.2758</v>
+        <v>48.2764</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.038</v>
+        <v>0.0382</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.0007877639527507474</v>
+        <v>0.0007919035121542678</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>55.815</v>
+        <v>55.7767</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>55.9286</v>
+        <v>55.8904</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.1136</v>
+        <v>0.1137</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>0.002035295171548867</v>
+        <v>0.002038485604203906</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>6661.29</v>
+        <v>6644.07</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>6692.94</v>
+        <v>6675.7</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>31.65</v>
+        <v>31.63</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>0.004751331949217044</v>
+        <v>0.004760636176319635</v>
       </c>
     </row>
     <row r="11">
@@ -7519,7 +7519,7 @@
         <v>46267</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
@@ -7527,40 +7527,40 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>47.924</v>
+        <v>47.9238</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>49.1614</v>
+        <v>49.162</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1.2374</v>
+        <v>1.2382</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.02582004840998247</v>
+        <v>0.02583684933164733</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>55.4024</v>
+        <v>55.3929</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>56.681</v>
+        <v>56.6712</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>1.2786</v>
+        <v>1.2783</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>0.02307842259541103</v>
+        <v>0.02307696473735804</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6614.85</v>
+        <v>6603.89</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>6723.08</v>
+        <v>6712.04</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>108.23</v>
+        <v>108.15</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>0.01636167108853564</v>
+        <v>0.01637671130197505</v>
       </c>
     </row>
     <row r="12">
@@ -7568,7 +7568,7 @@
         <v>46267</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
@@ -7588,28 +7588,28 @@
         <v>0.01776477349913789</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>55.3195</v>
+        <v>55.2908</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>56.4909</v>
+        <v>56.447</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>1.1714</v>
+        <v>1.1562</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>0.02117517331140014</v>
+        <v>0.02091125467528052</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>6609.94</v>
+        <v>6593.27</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>6764.43</v>
+        <v>6747.42</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>154.49</v>
+        <v>154.15</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>0.02337237554349964</v>
+        <v>0.0233799010202828</v>
       </c>
     </row>
     <row r="13">
@@ -7617,7 +7617,7 @@
         <v>46267</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
@@ -7625,40 +7625,40 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>47.9979</v>
+        <v>47.9984</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>48.6049</v>
+        <v>48.6053</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.607</v>
+        <v>0.6069</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.01264638661274764</v>
+        <v>0.01264417147238241</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>55.5966</v>
+        <v>55.563</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>56.2577</v>
+        <v>56.223</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>0.6611</v>
+        <v>0.66</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>0.01189101491817845</v>
+        <v>0.0118784082932887</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6678.06</v>
+        <v>6667.55</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>6732.35</v>
+        <v>6721.57</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>54.29</v>
+        <v>54.02</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>0.008129606502487249</v>
+        <v>0.008101926494739446</v>
       </c>
     </row>
     <row r="14">
@@ -7666,7 +7666,7 @@
         <v>46267</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
@@ -7686,28 +7686,28 @@
         <v>0.02844860285750411</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>54.952</v>
+        <v>54.928</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>56.515</v>
+        <v>56.491</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>1.563</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>0.02844300480419275</v>
+        <v>0.02845543256626857</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>6573.4</v>
+        <v>6565.63</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>6816.24</v>
+        <v>6808.18</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>242.84</v>
+        <v>242.55</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>0.03694283019441993</v>
+        <v>0.03694238024378468</v>
       </c>
     </row>
     <row r="15">
@@ -7715,7 +7715,7 @@
         <v>46267</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
@@ -7723,40 +7723,40 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>47.9979</v>
+        <v>47.9984</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>48.6049</v>
+        <v>48.6054</v>
       </c>
       <c r="F15" s="8" t="n">
         <v>0.607</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>0.01264638661274764</v>
+        <v>0.01264625487516251</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>55.6023</v>
+        <v>55.5645</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>56.2623</v>
+        <v>56.2243</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>0.66</v>
+        <v>0.6598000000000001</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>0.01187001257142241</v>
+        <v>0.01187448820739861</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>6681.92</v>
+        <v>6665.24</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>6736.04</v>
+        <v>6719.66</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>54.12</v>
+        <v>54.42</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>0.008099468416263588</v>
+        <v>0.008164747255912765</v>
       </c>
     </row>
     <row r="16">
@@ -7764,7 +7764,7 @@
         <v>46267</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
@@ -7784,28 +7784,28 @@
         <v>0.02047330948958786</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>55.4422</v>
+        <v>55.4063</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>56.5773</v>
+        <v>56.5406</v>
       </c>
       <c r="J16" s="10" t="n">
-        <v>1.1351</v>
+        <v>1.1343</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>0.02047357428096288</v>
+        <v>0.02047240115293748</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>6614.91</v>
+        <v>6600.43</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>6818.07</v>
+        <v>6803.15</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>203.16</v>
+        <v>202.72</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>0.03071243599686163</v>
+        <v>0.03071315050686092</v>
       </c>
     </row>
     <row r="17">
@@ -7813,7 +7813,7 @@
         <v>46267</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
@@ -7821,40 +7821,40 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>48.1928</v>
+        <v>48.2001</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>48.2518</v>
+        <v>48.262</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.059</v>
+        <v>0.0619</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.001224249265450441</v>
+        <v>0.001284229700768256</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>55.672</v>
+        <v>55.648</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>55.839</v>
+        <v>55.819</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>0.167</v>
+        <v>0.171</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>0.002999712602385401</v>
+        <v>0.003072886716503738</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>6611.85</v>
+        <v>6596.45</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>6706.82</v>
+        <v>6691.71</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>94.97</v>
+        <v>95.26000000000001</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>0.01436360473997444</v>
+        <v>0.01444110089517847</v>
       </c>
     </row>
     <row r="18">
@@ -7862,7 +7862,7 @@
         <v>46267</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
@@ -7870,40 +7870,40 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>48.2178</v>
+        <v>48.2184</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>48.364</v>
+        <v>48.3646</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>0.1462</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.003032075291697257</v>
+        <v>0.003032037562424303</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>55.828</v>
+        <v>55.7922</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>55.999</v>
+        <v>55.9632</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>0.171</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>0.003062979150247187</v>
+        <v>0.003064944562143096</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>6672.81</v>
+        <v>6654.79</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>6719.89</v>
+        <v>6701.75</v>
       </c>
       <c r="N18" s="12" t="n">
-        <v>47.08</v>
+        <v>46.96</v>
       </c>
       <c r="O18" s="13" t="n">
-        <v>0.007055498358262861</v>
+        <v>0.007056571281738418</v>
       </c>
     </row>
     <row r="19">
@@ -7911,7 +7911,7 @@
         <v>46267</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
@@ -7927,16 +7927,16 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="12" t="n">
-        <v>6684.59</v>
+        <v>6672.01</v>
       </c>
       <c r="M19" s="12" t="n">
-        <v>6880.44</v>
+        <v>6867.62</v>
       </c>
       <c r="N19" s="12" t="n">
-        <v>195.85</v>
+        <v>195.61</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>0.02929873036341795</v>
+        <v>0.02931800162170021</v>
       </c>
     </row>
     <row r="20">
@@ -7944,7 +7944,7 @@
         <v>46267</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C20" s="31" t="inlineStr">
         <is>
@@ -7952,40 +7952,40 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>47.8064</v>
+        <v>47.7241</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>48.6889</v>
+        <v>48.6807</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0.8825</v>
+        <v>0.9566</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>0.01845987148164262</v>
+        <v>0.02004438009307666</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>55.3698</v>
+        <v>55.2361</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>56.4197</v>
+        <v>56.3714</v>
       </c>
       <c r="J20" s="10" t="n">
-        <v>1.0499</v>
+        <v>1.1353</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>0.01896160000577932</v>
+        <v>0.02055358723733211</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>6614.8</v>
+        <v>6597.45</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>7060.2</v>
+        <v>7042.64</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>445.4</v>
+        <v>445.19</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>0.0673338574106549</v>
+        <v>0.06747910177417032</v>
       </c>
     </row>
     <row r="21">
@@ -7993,7 +7993,7 @@
         <v>46267</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
@@ -8001,40 +8001,40 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>47.7513</v>
+        <v>47.7516</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>48.7543</v>
+        <v>48.7545</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.003</v>
+        <v>1.0029</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.02100466374737442</v>
+        <v>0.02100243761465584</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>55.3789</v>
+        <v>55.3406</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>56.3854</v>
+        <v>56.347</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>1.0065</v>
+        <v>1.0064</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>0.01817479220425108</v>
+        <v>0.01818556358261385</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>6582.5</v>
+        <v>6566.33</v>
       </c>
       <c r="M21" s="12" t="n">
-        <v>6834.42</v>
+        <v>6818.24</v>
       </c>
       <c r="N21" s="12" t="n">
-        <v>251.92</v>
+        <v>251.91</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>0.03827117356627421</v>
+        <v>0.03836389581394782</v>
       </c>
     </row>
     <row r="22">
@@ -8042,7 +8042,7 @@
         <v>46267</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -8050,40 +8050,40 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>47.6783</v>
+        <v>47.6787</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>48.8332</v>
+        <v>48.8337</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.1549</v>
+        <v>1.155</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>0.02422275962020458</v>
+        <v>0.02422465377621454</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>55.2115</v>
+        <v>55.1737</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>56.5488</v>
+        <v>56.5151</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>1.3373</v>
+        <v>1.3414</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>0.02422140314970613</v>
+        <v>0.02431230821931464</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>6601.95</v>
+        <v>6592.4</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>6783.02</v>
+        <v>6774.4</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>181.07</v>
+        <v>182</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>0.0274267451283333</v>
+        <v>0.02760754808567441</v>
       </c>
     </row>
     <row r="23">
@@ -8091,7 +8091,7 @@
         <v>46267</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C23" s="34" t="inlineStr">
         <is>
@@ -8099,16 +8099,16 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>48.22</v>
+        <v>48.24</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>48.23</v>
+        <v>48.25</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>0.01</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>0.0002073828287017835</v>
+        <v>0.0002072968490878939</v>
       </c>
       <c r="H23" s="10" t="n">
         <v>55.7</v>
@@ -8140,7 +8140,7 @@
         <v>46267</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
@@ -8148,40 +8148,40 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>47.6865</v>
+        <v>47.6131</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>48.6724</v>
+        <v>48.5992</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>0.9859</v>
+        <v>0.9861</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.02067461440869009</v>
+        <v>0.02071068676477692</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>55.1413</v>
+        <v>55.105</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>56.2835</v>
+        <v>56.2468</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>1.1422</v>
+        <v>1.1418</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>0.0207140564331998</v>
+        <v>0.02072044279103529</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>6563.64</v>
+        <v>6547.71</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>6737.46</v>
+        <v>6721.33</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>173.82</v>
+        <v>173.62</v>
       </c>
       <c r="O24" s="13" t="n">
-        <v>0.02648225679653363</v>
+        <v>0.02651614075760838</v>
       </c>
     </row>
     <row r="25">
@@ -8189,7 +8189,7 @@
         <v>46267</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
@@ -8230,7 +8230,7 @@
         <v>46267</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
@@ -8238,40 +8238,40 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>48.2269</v>
+        <v>48.2272</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>48.2797</v>
+        <v>48.2802</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>0.0528</v>
+        <v>0.053</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>0.001094824672537526</v>
+        <v>0.001098964899475814</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>55.8388</v>
+        <v>55.8012</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>55.9157</v>
+        <v>55.8776</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>0.0769</v>
+        <v>0.0764</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>0.001377178592663166</v>
+        <v>0.001369146183236203</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>6661.79</v>
+        <v>6643.48</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>6690.54</v>
+        <v>6672.33</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>28.75</v>
+        <v>28.85</v>
       </c>
       <c r="O26" s="13" t="n">
-        <v>0.004315656903024562</v>
+        <v>0.004342603575234667</v>
       </c>
     </row>
     <row r="27">
@@ -8279,7 +8279,7 @@
         <v>46267</v>
       </c>
       <c r="B27" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C27" s="38" t="inlineStr">
         <is>
@@ -8287,40 +8287,40 @@
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>48.192</v>
+        <v>48.194</v>
       </c>
       <c r="E27" s="8" t="n">
         <v>48.291</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.099</v>
+        <v>0.097</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>0.002054282868525896</v>
+        <v>0.002012698676183757</v>
       </c>
       <c r="H27" s="10" t="n">
         <v>55.665</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>55.904</v>
+        <v>55.866</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>0.239</v>
+        <v>0.201</v>
       </c>
       <c r="K27" s="11" t="n">
-        <v>0.004293541722806072</v>
+        <v>0.003610886553489625</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>6624</v>
+        <v>6620</v>
       </c>
       <c r="M27" s="12" t="n">
-        <v>6686</v>
+        <v>6668</v>
       </c>
       <c r="N27" s="12" t="n">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>0.009359903381642512</v>
+        <v>0.007250755287009063</v>
       </c>
     </row>
     <row r="28">
@@ -8328,7 +8328,7 @@
         <v>46267</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -8336,40 +8336,40 @@
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>47.761</v>
+        <v>47.7615</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>48.761</v>
+        <v>48.7615</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>0.0209375850589393</v>
+        <v>0.02093736586999989</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>55.344</v>
+        <v>55.31</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>56.434</v>
+        <v>56.4</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>1.09</v>
       </c>
       <c r="K28" s="11" t="n">
-        <v>0.01969499855449552</v>
+        <v>0.01970710540589405</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>6655.57</v>
+        <v>6646.28</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>6755.57</v>
+        <v>6746.28</v>
       </c>
       <c r="N28" s="12" t="n">
         <v>100</v>
       </c>
       <c r="O28" s="13" t="n">
-        <v>0.01502500912769305</v>
+        <v>0.01504601070072281</v>
       </c>
     </row>
     <row r="29">
@@ -8377,7 +8377,7 @@
         <v>46267</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
@@ -8393,16 +8393,16 @@
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="12" t="n">
-        <v>6684.49</v>
+        <v>6672.01</v>
       </c>
       <c r="M29" s="12" t="n">
-        <v>6866.61</v>
+        <v>6853.91</v>
       </c>
       <c r="N29" s="12" t="n">
-        <v>182.12</v>
+        <v>181.9</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>0.02724516006456738</v>
+        <v>0.02726314858640799</v>
       </c>
     </row>
     <row r="30">
@@ -8410,7 +8410,7 @@
         <v>46267</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C30" s="41" t="inlineStr">
         <is>
@@ -8430,28 +8430,28 @@
         <v>0.02558322411533421</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>55.1109</v>
+        <v>55.0776</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>56.7636</v>
+        <v>56.7293</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>1.6527</v>
+        <v>1.6517</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>0.02998862294028949</v>
+        <v>0.0299885979055006</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>6584.82</v>
+        <v>6567.5</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>6782.96</v>
+        <v>6765.12</v>
       </c>
       <c r="N30" s="12" t="n">
-        <v>198.14</v>
+        <v>197.62</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>0.03009042008741317</v>
+        <v>0.03009059763989341</v>
       </c>
     </row>
     <row r="31">
@@ -8459,7 +8459,7 @@
         <v>46267</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -8467,10 +8467,10 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>48.297</v>
+        <v>48.2964</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>48.297</v>
+        <v>48.2964</v>
       </c>
       <c r="F31" s="8" t="n">
         <v>0</v>
@@ -8479,10 +8479,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>55.9351</v>
+        <v>55.8988</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>55.9351</v>
+        <v>55.8988</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>0</v>
@@ -8491,10 +8491,10 @@
         <v>0</v>
       </c>
       <c r="L31" s="12" t="n">
-        <v>6682.99</v>
+        <v>6664.82</v>
       </c>
       <c r="M31" s="12" t="n">
-        <v>6682.99</v>
+        <v>6664.82</v>
       </c>
       <c r="N31" s="12" t="n">
         <v>0</v>
@@ -8508,7 +8508,7 @@
         <v>46267</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C32" s="43" t="inlineStr">
         <is>
@@ -8519,37 +8519,37 @@
         <v>47.8519</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>48.6536</v>
+        <v>48.6539</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.8017</v>
+        <v>0.802</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>0.01675377571214518</v>
+        <v>0.01676004505568222</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>55.4553</v>
+        <v>55.4265</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>56.3054</v>
+        <v>56.277</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>0.8501</v>
+        <v>0.8505</v>
       </c>
       <c r="K32" s="11" t="n">
-        <v>0.01532946354992219</v>
+        <v>0.01534464561175611</v>
       </c>
       <c r="L32" s="12" t="n">
-        <v>6614.04</v>
+        <v>6599.48</v>
       </c>
       <c r="M32" s="12" t="n">
-        <v>6810.1</v>
+        <v>6795.93</v>
       </c>
       <c r="N32" s="12" t="n">
-        <v>196.06</v>
+        <v>196.45</v>
       </c>
       <c r="O32" s="13" t="n">
-        <v>0.02964300185665645</v>
+        <v>0.02976749683308382</v>
       </c>
     </row>
     <row r="33">
@@ -8557,7 +8557,7 @@
         <v>46267</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
@@ -8565,40 +8565,40 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>48.1536</v>
+        <v>48.1539</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>48.3568</v>
+        <v>48.3571</v>
       </c>
       <c r="F33" s="8" t="n">
         <v>0.2032</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>0.004219829877724615</v>
+        <v>0.004219803588079054</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>55.759</v>
+        <v>55.7173</v>
       </c>
       <c r="I33" s="10" t="n">
-        <v>55.9836</v>
+        <v>55.9418</v>
       </c>
       <c r="J33" s="10" t="n">
-        <v>0.2246</v>
+        <v>0.2245</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>0.004028049283523735</v>
+        <v>0.004029269185692774</v>
       </c>
       <c r="L33" s="12" t="n">
-        <v>6649.89</v>
+        <v>6632.87</v>
       </c>
       <c r="M33" s="12" t="n">
-        <v>6703.31</v>
+        <v>6686.15</v>
       </c>
       <c r="N33" s="12" t="n">
-        <v>53.42</v>
+        <v>53.28</v>
       </c>
       <c r="O33" s="13" t="n">
-        <v>0.008033215587024748</v>
+        <v>0.008032721883588854</v>
       </c>
     </row>
     <row r="34">
@@ -8606,7 +8606,7 @@
         <v>46267</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C34" s="45" t="inlineStr">
         <is>
@@ -8614,40 +8614,40 @@
         </is>
       </c>
       <c r="D34" s="8" t="n">
-        <v>47.8942</v>
+        <v>47.8943</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>48.8552</v>
+        <v>48.8553</v>
       </c>
       <c r="F34" s="8" t="n">
         <v>0.961</v>
       </c>
       <c r="G34" s="9" t="n">
-        <v>0.02006506006990408</v>
+        <v>0.0200650181754405</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>55.4892</v>
+        <v>55.4732</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>56.5913</v>
+        <v>56.5752</v>
       </c>
       <c r="J34" s="10" t="n">
-        <v>1.1021</v>
+        <v>1.102</v>
       </c>
       <c r="K34" s="11" t="n">
-        <v>0.01986152260259654</v>
+        <v>0.01986544854091706</v>
       </c>
       <c r="L34" s="12" t="n">
-        <v>6615.97</v>
+        <v>6600.33</v>
       </c>
       <c r="M34" s="12" t="n">
-        <v>6760.57</v>
+        <v>6744.93</v>
       </c>
       <c r="N34" s="12" t="n">
         <v>144.6</v>
       </c>
       <c r="O34" s="13" t="n">
-        <v>0.02185620551483758</v>
+        <v>0.02190799550931545</v>
       </c>
     </row>
     <row r="35">
@@ -8655,7 +8655,7 @@
         <v>46267</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C35" s="46" t="inlineStr">
         <is>
@@ -8663,28 +8663,28 @@
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>48.199</v>
+        <v>48.224</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>48.25</v>
+        <v>48.265</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.051</v>
+        <v>0.041</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>0.001058113238863877</v>
+        <v>0.0008501990710019908</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>55.69</v>
+        <v>55.689</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>55.819</v>
+        <v>55.799</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>0.129</v>
+        <v>0.11</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>0.002316394325731729</v>
+        <v>0.001975255436441667</v>
       </c>
       <c r="L35" s="12" t="n"/>
       <c r="M35" s="12" t="n"/>
@@ -8696,7 +8696,7 @@
         <v>46267</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C36" s="47" t="inlineStr">
         <is>
@@ -8716,28 +8716,28 @@
         <v>0.02098635886673662</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>55.19</v>
+        <v>55.16</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>56.33</v>
+        <v>56.29</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="K36" s="11" t="n">
-        <v>0.02065591592679833</v>
+        <v>0.02048585931834663</v>
       </c>
       <c r="L36" s="12" t="n">
-        <v>6584.14</v>
+        <v>6570.03</v>
       </c>
       <c r="M36" s="12" t="n">
-        <v>6786.1</v>
+        <v>6772.25</v>
       </c>
       <c r="N36" s="12" t="n">
-        <v>201.96</v>
+        <v>202.22</v>
       </c>
       <c r="O36" s="13" t="n">
-        <v>0.03067370985428621</v>
+        <v>0.03077915930368659</v>
       </c>
     </row>
     <row r="37">
@@ -8745,7 +8745,7 @@
         <v>46267</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C37" s="48" t="inlineStr">
         <is>
@@ -8765,28 +8765,28 @@
         <v>0.02022948183877804</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>55.4447</v>
+        <v>55.4349</v>
       </c>
       <c r="I37" s="10" t="n">
-        <v>56.5664</v>
+        <v>56.5564</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1.1217</v>
+        <v>1.1215</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>0.02023096887529376</v>
+        <v>0.02023093755017146</v>
       </c>
       <c r="L37" s="12" t="n">
-        <v>6646.78</v>
+        <v>6647.04</v>
       </c>
       <c r="M37" s="12" t="n">
-        <v>6780.98</v>
+        <v>6781.26</v>
       </c>
       <c r="N37" s="12" t="n">
-        <v>134.2</v>
+        <v>134.22</v>
       </c>
       <c r="O37" s="13" t="n">
-        <v>0.02019022744847881</v>
+        <v>0.02019244656268053</v>
       </c>
     </row>
     <row r="38">
@@ -8794,7 +8794,7 @@
         <v>46267</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
@@ -8814,28 +8814,28 @@
         <v>0.01360495969827946</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>55.4571</v>
+        <v>55.4161</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>56.2678</v>
+        <v>56.2262</v>
       </c>
       <c r="J38" s="10" t="n">
-        <v>0.8107</v>
+        <v>0.8101</v>
       </c>
       <c r="K38" s="11" t="n">
-        <v>0.01461850691796001</v>
+        <v>0.01461849534702009</v>
       </c>
       <c r="L38" s="12" t="n">
-        <v>6618.5</v>
+        <v>6601.38</v>
       </c>
       <c r="M38" s="12" t="n">
-        <v>6752.13</v>
+        <v>6734.67</v>
       </c>
       <c r="N38" s="12" t="n">
-        <v>133.63</v>
+        <v>133.29</v>
       </c>
       <c r="O38" s="13" t="n">
-        <v>0.02019037546271814</v>
+        <v>0.0201912327422448</v>
       </c>
     </row>
     <row r="39">
@@ -8843,7 +8843,7 @@
         <v>46267</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="C39" s="50" t="inlineStr">
         <is>
@@ -8851,40 +8851,40 @@
         </is>
       </c>
       <c r="D39" s="8" t="n">
-        <v>47.7683</v>
+        <v>47.7687</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>48.7651</v>
+        <v>48.7655</v>
       </c>
       <c r="F39" s="8" t="n">
         <v>0.9968</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>0.02086739532283962</v>
+        <v>0.0208672205858648</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>55.2806</v>
+        <v>55.2409</v>
       </c>
       <c r="I39" s="10" t="n">
-        <v>56.4894</v>
+        <v>56.4493</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1.2088</v>
+        <v>1.2084</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>0.02186662228702293</v>
+        <v>0.02187509616968587</v>
       </c>
       <c r="L39" s="12" t="n">
-        <v>6639.21</v>
+        <v>6621.58</v>
       </c>
       <c r="M39" s="12" t="n">
-        <v>6850.01</v>
+        <v>6831.73</v>
       </c>
       <c r="N39" s="12" t="n">
-        <v>210.8</v>
+        <v>210.15</v>
       </c>
       <c r="O39" s="13" t="n">
-        <v>0.03175076552782635</v>
+        <v>0.03173713826609359</v>
       </c>
     </row>
   </sheetData>
@@ -42186,7 +42186,7 @@
       </c>
       <c r="B5" s="62" t="n"/>
       <c r="C5" s="64" t="n">
-        <v>0.4871875</v>
+        <v>0.4999768518518519</v>
       </c>
       <c r="D5" s="62" t="n"/>
       <c r="F5" s="62" t="inlineStr">
@@ -42270,7 +42270,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="70" t="n">
-        <v>0.02023096887529376</v>
+        <v>0.02023093755017146</v>
       </c>
       <c r="O6" s="71" t="inlineStr">
         <is>
@@ -42278,10 +42278,10 @@
         </is>
       </c>
       <c r="P6" s="72" t="n">
-        <v>55.4447</v>
+        <v>55.4349</v>
       </c>
       <c r="Q6" s="72" t="n">
-        <v>56.5664</v>
+        <v>56.5564</v>
       </c>
     </row>
     <row r="7">
@@ -42323,7 +42323,7 @@
         <v>5</v>
       </c>
       <c r="N7" s="70" t="n">
-        <v>0.02019022744847881</v>
+        <v>0.02019244656268053</v>
       </c>
       <c r="O7" s="71" t="inlineStr">
         <is>
@@ -42331,10 +42331,10 @@
         </is>
       </c>
       <c r="P7" s="72" t="n">
-        <v>6646.78</v>
+        <v>6647.04</v>
       </c>
       <c r="Q7" s="72" t="n">
-        <v>6780.98</v>
+        <v>6781.26</v>
       </c>
     </row>
     <row r="8">
@@ -42376,7 +42376,7 @@
       </c>
       <c r="B9" s="62" t="n"/>
       <c r="C9" s="73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" s="62" t="n"/>
       <c r="F9" s="62" t="inlineStr">
@@ -42977,7 +42977,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>29.08 Cmt</t>
+          <t>🔵 29.08 Cmt</t>
         </is>
       </c>
       <c r="B3" s="55" t="n">
@@ -43079,7 +43079,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>30.08 Paz</t>
+          <t>🔴 30.08 Paz</t>
         </is>
       </c>
       <c r="B4" s="55" t="n">

</xml_diff>

<commit_message>
Günlük kur verisi: 02.09.2026 14:16
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -7078,7 +7078,7 @@
         <v>46267</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
@@ -7098,28 +7098,28 @@
         <v>0.02842045430622513</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>54.9729</v>
+        <v>54.9733</v>
       </c>
       <c r="I2" s="10" t="n">
-        <v>56.5401</v>
+        <v>56.5405</v>
       </c>
       <c r="J2" s="10" t="n">
         <v>1.5672</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>0.02850859241553565</v>
+        <v>0.02850838497961737</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>6523.14</v>
+        <v>6522.09</v>
       </c>
       <c r="M2" s="12" t="n">
-        <v>6758.76</v>
+        <v>6757.84</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>235.62</v>
+        <v>235.75</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>0.03612064128625171</v>
+        <v>0.03614638865762355</v>
       </c>
     </row>
     <row r="3">
@@ -7127,7 +7127,7 @@
         <v>46267</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
@@ -7159,16 +7159,16 @@
         <v>0.01649045574279219</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>6598.1</v>
+        <v>6599.06</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>6733.81</v>
+        <v>6734.34</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>135.71</v>
+        <v>135.28</v>
       </c>
       <c r="O3" s="13" t="n">
-        <v>0.02056804231521196</v>
+        <v>0.02049988937818416</v>
       </c>
     </row>
     <row r="4">
@@ -7176,7 +7176,7 @@
         <v>46267</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -7196,28 +7196,28 @@
         <v>0.006093883238701359</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>55.476</v>
+        <v>55.473</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>55.988</v>
+        <v>55.983</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.512</v>
+        <v>0.51</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>0.009229216237652318</v>
+        <v>0.00919366178140717</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>6663.21</v>
+        <v>6663.18</v>
       </c>
       <c r="M4" s="12" t="n">
-        <v>6729.36</v>
+        <v>6730.38</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>66.15000000000001</v>
+        <v>67.2</v>
       </c>
       <c r="O4" s="13" t="n">
-        <v>0.009927647485221087</v>
+        <v>0.01008527459861507</v>
       </c>
     </row>
     <row r="5">
@@ -7225,7 +7225,7 @@
         <v>46267</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -7233,40 +7233,40 @@
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>48.13</v>
+        <v>48.18</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>48.33</v>
+        <v>48.37</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>0.00415541242468315</v>
+        <v>0.00394354503943545</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>55.594</v>
+        <v>55.658</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>55.938</v>
+        <v>55.978</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.344</v>
+        <v>0.32</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>0.00618771809907544</v>
+        <v>0.005749398109885372</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>6572.1</v>
+        <v>6600.17</v>
       </c>
       <c r="M5" s="12" t="n">
-        <v>6755</v>
+        <v>6770</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>182.9</v>
+        <v>169.83</v>
       </c>
       <c r="O5" s="13" t="n">
-        <v>0.0278297652196406</v>
+        <v>0.02573115540963338</v>
       </c>
     </row>
     <row r="6">
@@ -7274,7 +7274,7 @@
         <v>46267</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
@@ -7282,40 +7282,40 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>47.4534</v>
+        <v>47.4536</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>48.7297</v>
+        <v>48.7303</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>1.2763</v>
+        <v>1.2767</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.02689585993838166</v>
+        <v>0.02690417586863799</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>55.0203</v>
+        <v>55.0165</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>56.3848</v>
+        <v>56.3818</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>1.3645</v>
+        <v>1.3653</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0.02479993747762189</v>
+        <v>0.02481619150618451</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>6581.24</v>
+        <v>6595.52</v>
       </c>
       <c r="M6" s="12" t="n">
-        <v>6732.31</v>
+        <v>6746.54</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>151.07</v>
+        <v>151.02</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>0.02295464076678559</v>
+        <v>0.02289736063267188</v>
       </c>
     </row>
     <row r="7">
@@ -7323,7 +7323,7 @@
         <v>46267</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
@@ -7334,37 +7334,37 @@
         <v>47.302</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>49.225</v>
+        <v>49.226</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>1.923</v>
+        <v>1.924</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>0.04065367214916916</v>
+        <v>0.04067481290431695</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>54.743</v>
+        <v>54.738</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>56.973</v>
+        <v>56.974</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>2.23</v>
+        <v>2.236</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>0.04073580183767787</v>
+        <v>0.040849135883664</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>6578.25</v>
+        <v>6589.45</v>
       </c>
       <c r="M7" s="12" t="n">
-        <v>6772.46</v>
+        <v>6783.97</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>194.21</v>
+        <v>194.52</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>0.02952304944324098</v>
+        <v>0.02951991440863805</v>
       </c>
     </row>
     <row r="8">
@@ -7372,7 +7372,7 @@
         <v>46267</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
@@ -7380,40 +7380,40 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>47.5551</v>
+        <v>47.555</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>48.9552</v>
+        <v>48.9551</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>1.4001</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>0.02944163717456172</v>
+        <v>0.02944169908526969</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>55.0398</v>
+        <v>55.0301</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>56.6603</v>
+        <v>56.6552</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>1.6205</v>
+        <v>1.6251</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>0.02944233082242305</v>
+        <v>0.02953111115553125</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>6595.09</v>
+        <v>6600.75</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>6790.33</v>
+        <v>6796.06</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>195.24</v>
+        <v>195.31</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>0.02960384164583046</v>
+        <v>0.02958906184903231</v>
       </c>
     </row>
     <row r="9">
@@ -7421,7 +7421,7 @@
         <v>46267</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -7429,40 +7429,40 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>48.2247</v>
+        <v>48.2245</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>48.2816</v>
+        <v>48.2821</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.0569</v>
+        <v>0.0576</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.001179893291197249</v>
+        <v>0.001194413627927713</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>55.7992</v>
+        <v>55.7996</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>55.8824</v>
+        <v>55.8827</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.0832</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>0.001491060803739122</v>
+        <v>0.001489257987512455</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6648.06</v>
+        <v>6659.64</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>6676.93</v>
+        <v>6688.18</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>28.87</v>
+        <v>28.54</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>0.004342620253126477</v>
+        <v>0.004285516934849331</v>
       </c>
     </row>
     <row r="10">
@@ -7470,7 +7470,7 @@
         <v>46267</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -7478,40 +7478,40 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>48.2382</v>
+        <v>48.2381</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>48.2764</v>
+        <v>48.2772</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.0382</v>
+        <v>0.0391</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.0007919035121542678</v>
+        <v>0.0008105626050777289</v>
       </c>
       <c r="H10" s="10" t="n">
         <v>55.7767</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>55.8904</v>
+        <v>55.8867</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.1137</v>
+        <v>0.11</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>0.002038485604203906</v>
+        <v>0.001972149661059188</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>6644.07</v>
+        <v>6655.84</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>6675.7</v>
+        <v>6687.65</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>31.63</v>
+        <v>31.81</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>0.004760636176319635</v>
+        <v>0.004779261520709632</v>
       </c>
     </row>
     <row r="11">
@@ -7519,7 +7519,7 @@
         <v>46267</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
@@ -7527,40 +7527,40 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>47.9238</v>
+        <v>47.9241</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>49.162</v>
+        <v>49.1615</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1.2382</v>
+        <v>1.2374</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.02583684933164733</v>
+        <v>0.02581999453302201</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>55.3929</v>
+        <v>55.3594</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>56.6712</v>
+        <v>56.6321</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>1.2783</v>
+        <v>1.2727</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>0.02307696473735804</v>
+        <v>0.02298977228799445</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6603.89</v>
+        <v>6601.47</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>6712.04</v>
+        <v>6709.49</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>108.15</v>
+        <v>108.02</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>0.01637671130197505</v>
+        <v>0.01636302217536397</v>
       </c>
     </row>
     <row r="12">
@@ -7568,7 +7568,7 @@
         <v>46267</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
@@ -7588,28 +7588,28 @@
         <v>0.01776477349913789</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>55.2908</v>
+        <v>55.2861</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>56.447</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>1.1562</v>
+        <v>1.1609</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>0.02091125467528052</v>
+        <v>0.02099804471648389</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>6593.27</v>
+        <v>6606.01</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>6747.42</v>
+        <v>6760.81</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>154.15</v>
+        <v>154.8</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>0.0233799010202828</v>
+        <v>0.02343320703420067</v>
       </c>
     </row>
     <row r="13">
@@ -7617,7 +7617,7 @@
         <v>46267</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
@@ -7625,40 +7625,40 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>47.9984</v>
+        <v>47.9985</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>48.6053</v>
+        <v>48.606</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.6069</v>
+        <v>0.6075</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.01264417147238241</v>
+        <v>0.01265664552017251</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>55.563</v>
+        <v>55.5613</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>56.223</v>
+        <v>56.2222</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>0.66</v>
+        <v>0.6609</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>0.0118784082932887</v>
+        <v>0.01189497006009579</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6667.55</v>
+        <v>6670.14</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>6721.57</v>
+        <v>6724.29</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>54.02</v>
+        <v>54.15</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>0.008101926494739446</v>
+        <v>0.008118270381131431</v>
       </c>
     </row>
     <row r="14">
@@ -7666,7 +7666,7 @@
         <v>46267</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
@@ -7674,40 +7674,40 @@
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>47.454</v>
+        <v>47.455</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>48.804</v>
+        <v>48.805</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>1.35</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>0.02844860285750411</v>
+        <v>0.02844800337161522</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>54.928</v>
+        <v>54.914</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>56.491</v>
+        <v>56.477</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>1.563</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>0.02845543256626857</v>
+        <v>0.028462687110755</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>6565.63</v>
+        <v>6562.01</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>6808.18</v>
+        <v>6804.43</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>242.55</v>
+        <v>242.42</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>0.03694238024378468</v>
+        <v>0.03694294888304041</v>
       </c>
     </row>
     <row r="15">
@@ -7715,7 +7715,7 @@
         <v>46267</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
@@ -7723,40 +7723,40 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>47.9984</v>
+        <v>47.9988</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>48.6054</v>
+        <v>48.6058</v>
       </c>
       <c r="F15" s="8" t="n">
         <v>0.607</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>0.01264625487516251</v>
+        <v>0.01264614948707051</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>55.5645</v>
+        <v>55.5608</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>56.2243</v>
+        <v>56.2216</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>0.6598000000000001</v>
+        <v>0.6608000000000001</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>0.01187448820739861</v>
+        <v>0.01189327727462528</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>6665.24</v>
+        <v>6679.6</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>6719.66</v>
+        <v>6734.63</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>54.42</v>
+        <v>55.03</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>0.008164747255912765</v>
+        <v>0.008238517276483621</v>
       </c>
     </row>
     <row r="16">
@@ -7764,7 +7764,7 @@
         <v>46267</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
@@ -7772,40 +7772,40 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>47.8672</v>
+        <v>47.8675</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>48.8472</v>
+        <v>48.8475</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>0.98</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>0.02047330948958786</v>
+        <v>0.02047318117720792</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>55.4063</v>
+        <v>55.3947</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>56.5406</v>
+        <v>56.5288</v>
       </c>
       <c r="J16" s="10" t="n">
-        <v>1.1343</v>
+        <v>1.1341</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>0.02047240115293748</v>
+        <v>0.02047307774931537</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>6600.43</v>
+        <v>6596.25</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>6803.15</v>
+        <v>6798.84</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>202.72</v>
+        <v>202.59</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>0.03071315050686092</v>
+        <v>0.03071290505969301</v>
       </c>
     </row>
     <row r="17">
@@ -7813,7 +7813,7 @@
         <v>46267</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
@@ -7821,40 +7821,40 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>48.2001</v>
+        <v>48.24</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>48.262</v>
+        <v>48.309</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.0619</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.001284229700768256</v>
+        <v>0.001430348258706468</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>55.648</v>
+        <v>55.682</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>55.819</v>
+        <v>55.86</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>0.171</v>
+        <v>0.178</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>0.003072886716503738</v>
+        <v>0.003196724255594268</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>6596.45</v>
+        <v>6616.79</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>6691.71</v>
+        <v>6705.79</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>95.26000000000001</v>
+        <v>89</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>0.01444110089517847</v>
+        <v>0.01345063089504125</v>
       </c>
     </row>
     <row r="18">
@@ -7862,7 +7862,7 @@
         <v>46267</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
@@ -7870,40 +7870,40 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>48.2184</v>
+        <v>48.2187</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>48.3646</v>
+        <v>48.3651</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>0.1462</v>
+        <v>0.1464</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.003032037562424303</v>
+        <v>0.003036166466536842</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>55.7922</v>
+        <v>55.7901</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>55.9632</v>
+        <v>55.9613</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>0.171</v>
+        <v>0.1712</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>0.003064944562143096</v>
+        <v>0.003068644795402769</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>6654.79</v>
+        <v>6666</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>6701.75</v>
+        <v>6713.15</v>
       </c>
       <c r="N18" s="12" t="n">
-        <v>46.96</v>
+        <v>47.15</v>
       </c>
       <c r="O18" s="13" t="n">
-        <v>0.007056571281738418</v>
+        <v>0.007073207320732073</v>
       </c>
     </row>
     <row r="19">
@@ -7911,7 +7911,7 @@
         <v>46267</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
@@ -7927,16 +7927,16 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="12" t="n">
-        <v>6672.01</v>
+        <v>6669.35</v>
       </c>
       <c r="M19" s="12" t="n">
-        <v>6867.62</v>
+        <v>6864.8</v>
       </c>
       <c r="N19" s="12" t="n">
-        <v>195.61</v>
+        <v>195.45</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>0.02931800162170021</v>
+        <v>0.02930570445395728</v>
       </c>
     </row>
     <row r="20">
@@ -7944,7 +7944,7 @@
         <v>46267</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C20" s="31" t="inlineStr">
         <is>
@@ -7952,40 +7952,40 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>47.7241</v>
+        <v>47.8049</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>48.6807</v>
+        <v>48.6915</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0.9566</v>
+        <v>0.8866000000000001</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>0.02004438009307666</v>
+        <v>0.01854621597367634</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>55.2361</v>
+        <v>55.3246</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>56.3714</v>
+        <v>56.3839</v>
       </c>
       <c r="J20" s="10" t="n">
-        <v>1.1353</v>
+        <v>1.0593</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>0.02055358723733211</v>
+        <v>0.0191469978996685</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>6597.45</v>
+        <v>6610.81</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>7042.64</v>
+        <v>7056.88</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>445.19</v>
+        <v>446.07</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>0.06747910177417032</v>
+        <v>0.06747584637888548</v>
       </c>
     </row>
     <row r="21">
@@ -7993,7 +7993,7 @@
         <v>46267</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
@@ -8001,40 +8001,40 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>47.7516</v>
+        <v>47.7518</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>48.7545</v>
+        <v>48.7551</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.0029</v>
+        <v>1.0033</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.02100243761465584</v>
+        <v>0.02101072629722859</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>55.3406</v>
+        <v>55.3409</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>56.347</v>
+        <v>56.3476</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>1.0064</v>
+        <v>1.0067</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>0.01818556358261385</v>
+        <v>0.01819088594511473</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>6566.33</v>
+        <v>6571.18</v>
       </c>
       <c r="M21" s="12" t="n">
-        <v>6818.24</v>
+        <v>6823.01</v>
       </c>
       <c r="N21" s="12" t="n">
-        <v>251.91</v>
+        <v>251.83</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>0.03836389581394782</v>
+        <v>0.03832340614623249</v>
       </c>
     </row>
     <row r="22">
@@ -8042,7 +8042,7 @@
         <v>46267</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -8050,40 +8050,40 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>47.6787</v>
+        <v>47.6776</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>48.8337</v>
+        <v>48.8354</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.155</v>
+        <v>1.1578</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>0.02422465377621454</v>
+        <v>0.02428394046680202</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>55.1737</v>
+        <v>55.1678</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>56.5151</v>
+        <v>56.5123</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>1.3414</v>
+        <v>1.3445</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>0.02431230821931464</v>
+        <v>0.0243711005332821</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>6592.4</v>
+        <v>6595.24</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>6774.4</v>
+        <v>6776.85</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>182</v>
+        <v>181.61</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>0.02760754808567441</v>
+        <v>0.02753652634324149</v>
       </c>
     </row>
     <row r="23">
@@ -8091,7 +8091,7 @@
         <v>46267</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C23" s="34" t="inlineStr">
         <is>
@@ -8099,40 +8099,40 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>48.24</v>
+        <v>48.28</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>48.25</v>
+        <v>48.29</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>0.01</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>0.0002072968490878939</v>
+        <v>0.0002071251035625518</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>55.7</v>
+        <v>55.75</v>
       </c>
       <c r="I23" s="10" t="n">
-        <v>55.75</v>
+        <v>55.8</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>0.05</v>
       </c>
       <c r="K23" s="11" t="n">
-        <v>0.0008976660682226212</v>
+        <v>0.0008968609865470851</v>
       </c>
       <c r="L23" s="12" t="n">
-        <v>6722.02</v>
+        <v>6669.43</v>
       </c>
       <c r="M23" s="12" t="n">
-        <v>6728.25</v>
+        <v>6675.67</v>
       </c>
       <c r="N23" s="12" t="n">
-        <v>6.23</v>
+        <v>6.24</v>
       </c>
       <c r="O23" s="13" t="n">
-        <v>0.0009268047402417725</v>
+        <v>0.0009356121887477641</v>
       </c>
     </row>
     <row r="24">
@@ -8140,7 +8140,7 @@
         <v>46267</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
@@ -8148,40 +8148,40 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>47.6131</v>
+        <v>47.6134</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>48.5992</v>
+        <v>48.5996</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>0.9861</v>
+        <v>0.9862</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.02071068676477692</v>
+        <v>0.0207126565210634</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>55.105</v>
+        <v>55.1015</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>56.2468</v>
+        <v>56.2432</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>1.1418</v>
+        <v>1.1417</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>0.02072044279103529</v>
+        <v>0.02071994410315509</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>6547.71</v>
+        <v>6557.78</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>6721.33</v>
+        <v>6731.8</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>173.62</v>
+        <v>174.02</v>
       </c>
       <c r="O24" s="13" t="n">
-        <v>0.02651614075760838</v>
+        <v>0.02653641933703174</v>
       </c>
     </row>
     <row r="25">
@@ -8189,7 +8189,7 @@
         <v>46267</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
@@ -8230,7 +8230,7 @@
         <v>46267</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
@@ -8238,40 +8238,40 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>48.2272</v>
+        <v>48.2274</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>48.2802</v>
+        <v>48.2805</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>0.053</v>
+        <v>0.0531</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>0.001098964899475814</v>
+        <v>0.001101033852125555</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>55.8012</v>
+        <v>55.798</v>
       </c>
       <c r="I26" s="10" t="n">
         <v>55.8776</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>0.0764</v>
+        <v>0.0796</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>0.001369146183236203</v>
+        <v>0.00142657442919101</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>6643.48</v>
+        <v>6658.48</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>6672.33</v>
+        <v>6686.88</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>28.85</v>
+        <v>28.4</v>
       </c>
       <c r="O26" s="13" t="n">
-        <v>0.004342603575234667</v>
+        <v>0.004265237711910226</v>
       </c>
     </row>
     <row r="27">
@@ -8279,7 +8279,7 @@
         <v>46267</v>
       </c>
       <c r="B27" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C27" s="38" t="inlineStr">
         <is>
@@ -8287,40 +8287,40 @@
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>48.194</v>
+        <v>48.256</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>48.291</v>
+        <v>48.355</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.097</v>
+        <v>0.099</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>0.002012698676183757</v>
+        <v>0.002051558355437666</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>55.665</v>
+        <v>55.697</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>55.866</v>
+        <v>55.918</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>0.201</v>
+        <v>0.221</v>
       </c>
       <c r="K27" s="11" t="n">
-        <v>0.003610886553489625</v>
+        <v>0.003967897732373377</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>6620</v>
+        <v>6636</v>
       </c>
       <c r="M27" s="12" t="n">
-        <v>6668</v>
+        <v>6687</v>
       </c>
       <c r="N27" s="12" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>0.007250755287009063</v>
+        <v>0.007685352622061483</v>
       </c>
     </row>
     <row r="28">
@@ -8328,7 +8328,7 @@
         <v>46267</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -8336,40 +8336,40 @@
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>47.7615</v>
+        <v>47.762</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>48.7615</v>
+        <v>48.762</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>0.02093736586999989</v>
+        <v>0.02093714668564968</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>55.31</v>
+        <v>55.301</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>56.4</v>
+        <v>56.391</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>1.09</v>
       </c>
       <c r="K28" s="11" t="n">
-        <v>0.01970710540589405</v>
+        <v>0.01971031265257409</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>6646.28</v>
+        <v>6644.9</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>6746.28</v>
+        <v>6744.9</v>
       </c>
       <c r="N28" s="12" t="n">
         <v>100</v>
       </c>
       <c r="O28" s="13" t="n">
-        <v>0.01504601070072281</v>
+        <v>0.01504913542716971</v>
       </c>
     </row>
     <row r="29">
@@ -8377,7 +8377,7 @@
         <v>46267</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
@@ -8393,16 +8393,16 @@
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="12" t="n">
-        <v>6672.01</v>
+        <v>6667.97</v>
       </c>
       <c r="M29" s="12" t="n">
-        <v>6853.91</v>
+        <v>6849.7</v>
       </c>
       <c r="N29" s="12" t="n">
-        <v>181.9</v>
+        <v>181.73</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>0.02726314858640799</v>
+        <v>0.02725417180941126</v>
       </c>
     </row>
     <row r="30">
@@ -8410,7 +8410,7 @@
         <v>46267</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C30" s="41" t="inlineStr">
         <is>
@@ -8430,28 +8430,28 @@
         <v>0.02558322411533421</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>55.0776</v>
+        <v>55.0681</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>56.7293</v>
+        <v>56.7244</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>1.6517</v>
+        <v>1.6563</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>0.0299885979055006</v>
+        <v>0.03007730428324202</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>6567.5</v>
+        <v>6578.08</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>6765.12</v>
+        <v>6776.19</v>
       </c>
       <c r="N30" s="12" t="n">
-        <v>197.62</v>
+        <v>198.11</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>0.03009059763989341</v>
+        <v>0.03011669058448666</v>
       </c>
     </row>
     <row r="31">
@@ -8459,7 +8459,7 @@
         <v>46267</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -8467,40 +8467,40 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>48.2964</v>
+        <v>48.153</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>48.2964</v>
+        <v>48.3944</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>0</v>
+        <v>0.2414</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>0</v>
+        <v>0.005013187132681245</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>55.8988</v>
+        <v>55.6683</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>55.8988</v>
+        <v>56.0036</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>0</v>
+        <v>0.3353</v>
       </c>
       <c r="K31" s="11" t="n">
-        <v>0</v>
+        <v>0.006023176565478019</v>
       </c>
       <c r="L31" s="12" t="n">
-        <v>6664.82</v>
+        <v>6593.08</v>
       </c>
       <c r="M31" s="12" t="n">
-        <v>6664.82</v>
+        <v>6726.61</v>
       </c>
       <c r="N31" s="12" t="n">
-        <v>0</v>
+        <v>133.53</v>
       </c>
       <c r="O31" s="13" t="n">
-        <v>0</v>
+        <v>0.02025305320123524</v>
       </c>
     </row>
     <row r="32">
@@ -8508,7 +8508,7 @@
         <v>46267</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C32" s="43" t="inlineStr">
         <is>
@@ -8516,40 +8516,40 @@
         </is>
       </c>
       <c r="D32" s="8" t="n">
-        <v>47.8519</v>
+        <v>47.8522</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>48.6539</v>
+        <v>48.6544</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.802</v>
+        <v>0.8022</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>0.01676004505568222</v>
+        <v>0.01676411951801589</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>55.4265</v>
+        <v>55.4133</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>56.277</v>
+        <v>56.2636</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>0.8505</v>
+        <v>0.8502999999999999</v>
       </c>
       <c r="K32" s="11" t="n">
-        <v>0.01534464561175611</v>
+        <v>0.0153446916173554</v>
       </c>
       <c r="L32" s="12" t="n">
-        <v>6599.48</v>
+        <v>6595.3</v>
       </c>
       <c r="M32" s="12" t="n">
-        <v>6795.93</v>
+        <v>6791.42</v>
       </c>
       <c r="N32" s="12" t="n">
-        <v>196.45</v>
+        <v>196.12</v>
       </c>
       <c r="O32" s="13" t="n">
-        <v>0.02976749683308382</v>
+        <v>0.02973632738465271</v>
       </c>
     </row>
     <row r="33">
@@ -8557,7 +8557,7 @@
         <v>46267</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
@@ -8565,40 +8565,40 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>48.1539</v>
+        <v>48.1543</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>48.3571</v>
+        <v>48.3575</v>
       </c>
       <c r="F33" s="8" t="n">
         <v>0.2032</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>0.004219803588079054</v>
+        <v>0.004219768535727858</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>55.7173</v>
+        <v>55.7174</v>
       </c>
       <c r="I33" s="10" t="n">
-        <v>55.9418</v>
+        <v>55.942</v>
       </c>
       <c r="J33" s="10" t="n">
-        <v>0.2245</v>
+        <v>0.2246</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>0.004029269185692774</v>
+        <v>0.004031056725547136</v>
       </c>
       <c r="L33" s="12" t="n">
-        <v>6632.87</v>
+        <v>6638.6</v>
       </c>
       <c r="M33" s="12" t="n">
-        <v>6686.15</v>
+        <v>6691.93</v>
       </c>
       <c r="N33" s="12" t="n">
-        <v>53.28</v>
+        <v>53.33</v>
       </c>
       <c r="O33" s="13" t="n">
-        <v>0.008032721883588854</v>
+        <v>0.008033320278371945</v>
       </c>
     </row>
     <row r="34">
@@ -8606,7 +8606,7 @@
         <v>46267</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C34" s="45" t="inlineStr">
         <is>
@@ -8614,40 +8614,40 @@
         </is>
       </c>
       <c r="D34" s="8" t="n">
-        <v>47.8943</v>
+        <v>47.8946</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>48.8553</v>
+        <v>48.8556</v>
       </c>
       <c r="F34" s="8" t="n">
         <v>0.961</v>
       </c>
       <c r="G34" s="9" t="n">
-        <v>0.0200650181754405</v>
+        <v>0.02006489249309943</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>55.4732</v>
+        <v>55.4497</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>56.5752</v>
+        <v>56.5517</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>1.102</v>
       </c>
       <c r="K34" s="11" t="n">
-        <v>0.01986544854091706</v>
+        <v>0.01987386766745357</v>
       </c>
       <c r="L34" s="12" t="n">
-        <v>6600.33</v>
+        <v>6594.99</v>
       </c>
       <c r="M34" s="12" t="n">
-        <v>6744.93</v>
+        <v>6739.59</v>
       </c>
       <c r="N34" s="12" t="n">
         <v>144.6</v>
       </c>
       <c r="O34" s="13" t="n">
-        <v>0.02190799550931545</v>
+        <v>0.02192573453485146</v>
       </c>
     </row>
     <row r="35">
@@ -8655,7 +8655,7 @@
         <v>46267</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C35" s="46" t="inlineStr">
         <is>
@@ -8663,28 +8663,28 @@
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>48.224</v>
+        <v>48.255</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>48.265</v>
+        <v>48.3</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.041</v>
+        <v>0.045</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>0.0008501990710019908</v>
+        <v>0.0009325458501709667</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>55.689</v>
+        <v>55.73</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>55.799</v>
+        <v>55.824</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>0.11</v>
+        <v>0.094</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>0.001975255436441667</v>
+        <v>0.001686703750224296</v>
       </c>
       <c r="L35" s="12" t="n"/>
       <c r="M35" s="12" t="n"/>
@@ -8696,7 +8696,7 @@
         <v>46267</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C36" s="47" t="inlineStr">
         <is>
@@ -8707,37 +8707,37 @@
         <v>47.65</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>48.65</v>
+        <v>48.66</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="G36" s="9" t="n">
-        <v>0.02098635886673662</v>
+        <v>0.02119622245540399</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>55.16</v>
+        <v>55.15</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>56.29</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="K36" s="11" t="n">
-        <v>0.02048585931834663</v>
+        <v>0.02067089755213055</v>
       </c>
       <c r="L36" s="12" t="n">
-        <v>6570.03</v>
+        <v>6569.54</v>
       </c>
       <c r="M36" s="12" t="n">
-        <v>6772.25</v>
+        <v>6771.48</v>
       </c>
       <c r="N36" s="12" t="n">
-        <v>202.22</v>
+        <v>201.94</v>
       </c>
       <c r="O36" s="13" t="n">
-        <v>0.03077915930368659</v>
+        <v>0.03073883407361855</v>
       </c>
     </row>
     <row r="37">
@@ -8745,7 +8745,7 @@
         <v>46267</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C37" s="48" t="inlineStr">
         <is>
@@ -8753,40 +8753,40 @@
         </is>
       </c>
       <c r="D37" s="8" t="n">
-        <v>47.8905</v>
+        <v>47.8908</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>48.8593</v>
+        <v>48.8596</v>
       </c>
       <c r="F37" s="8" t="n">
         <v>0.9688</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>0.02022948183877804</v>
+        <v>0.02022935511622274</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>55.4349</v>
+        <v>55.4124</v>
       </c>
       <c r="I37" s="10" t="n">
-        <v>56.5564</v>
+        <v>56.5334</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1.1215</v>
+        <v>1.121</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>0.02023093755017146</v>
+        <v>0.02023012899639792</v>
       </c>
       <c r="L37" s="12" t="n">
-        <v>6647.04</v>
+        <v>6629.01</v>
       </c>
       <c r="M37" s="12" t="n">
-        <v>6781.26</v>
+        <v>6762.86</v>
       </c>
       <c r="N37" s="12" t="n">
-        <v>134.22</v>
+        <v>133.85</v>
       </c>
       <c r="O37" s="13" t="n">
-        <v>0.02019244656268053</v>
+        <v>0.02019155198136675</v>
       </c>
     </row>
     <row r="38">
@@ -8794,7 +8794,7 @@
         <v>46267</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
@@ -8802,40 +8802,40 @@
         </is>
       </c>
       <c r="D38" s="8" t="n">
-        <v>47.9384</v>
+        <v>47.9387</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>48.5906</v>
+        <v>48.5909</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>0.6522</v>
       </c>
       <c r="G38" s="9" t="n">
-        <v>0.01360495969827946</v>
+        <v>0.01360487455855082</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>55.4161</v>
+        <v>55.4124</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>56.2262</v>
+        <v>56.2225</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>0.8101</v>
       </c>
       <c r="K38" s="11" t="n">
-        <v>0.01461849534702009</v>
+        <v>0.01461947145404278</v>
       </c>
       <c r="L38" s="12" t="n">
-        <v>6601.38</v>
+        <v>6607.06</v>
       </c>
       <c r="M38" s="12" t="n">
-        <v>6734.67</v>
+        <v>6740.46</v>
       </c>
       <c r="N38" s="12" t="n">
-        <v>133.29</v>
+        <v>133.4</v>
       </c>
       <c r="O38" s="13" t="n">
-        <v>0.0201912327422448</v>
+        <v>0.02019052347034838</v>
       </c>
     </row>
     <row r="39">
@@ -8843,7 +8843,7 @@
         <v>46267</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="C39" s="50" t="inlineStr">
         <is>
@@ -8851,40 +8851,40 @@
         </is>
       </c>
       <c r="D39" s="8" t="n">
-        <v>47.7687</v>
+        <v>47.769</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>48.7655</v>
+        <v>48.766</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.9968</v>
+        <v>0.997</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>0.0208672205858648</v>
+        <v>0.02087127635077142</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>55.2409</v>
+        <v>55.2408</v>
       </c>
       <c r="I39" s="10" t="n">
-        <v>56.4493</v>
+        <v>56.4494</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1.2084</v>
+        <v>1.2086</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>0.02187509616968587</v>
+        <v>0.02187875628158897</v>
       </c>
       <c r="L39" s="12" t="n">
-        <v>6621.58</v>
+        <v>6627.03</v>
       </c>
       <c r="M39" s="12" t="n">
-        <v>6831.73</v>
+        <v>6837.43</v>
       </c>
       <c r="N39" s="12" t="n">
-        <v>210.15</v>
+        <v>210.4</v>
       </c>
       <c r="O39" s="13" t="n">
-        <v>0.03173713826609359</v>
+        <v>0.03174876226605282</v>
       </c>
     </row>
   </sheetData>
@@ -42186,7 +42186,7 @@
       </c>
       <c r="B5" s="62" t="n"/>
       <c r="C5" s="64" t="n">
-        <v>0.4999768518518519</v>
+        <v>0.5944791666666667</v>
       </c>
       <c r="D5" s="62" t="n"/>
       <c r="F5" s="62" t="inlineStr">
@@ -42217,7 +42217,7 @@
         <v>5</v>
       </c>
       <c r="N5" s="70" t="n">
-        <v>0.02022948183877804</v>
+        <v>0.02022935511622274</v>
       </c>
       <c r="O5" s="71" t="inlineStr">
         <is>
@@ -42225,10 +42225,10 @@
         </is>
       </c>
       <c r="P5" s="72" t="n">
-        <v>47.8905</v>
+        <v>47.8908</v>
       </c>
       <c r="Q5" s="72" t="n">
-        <v>48.8593</v>
+        <v>48.8596</v>
       </c>
     </row>
     <row r="6">
@@ -42270,7 +42270,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="70" t="n">
-        <v>0.02023093755017146</v>
+        <v>0.02023012899639792</v>
       </c>
       <c r="O6" s="71" t="inlineStr">
         <is>
@@ -42278,10 +42278,10 @@
         </is>
       </c>
       <c r="P6" s="72" t="n">
-        <v>55.4349</v>
+        <v>55.4124</v>
       </c>
       <c r="Q6" s="72" t="n">
-        <v>56.5564</v>
+        <v>56.5334</v>
       </c>
     </row>
     <row r="7">
@@ -42323,7 +42323,7 @@
         <v>5</v>
       </c>
       <c r="N7" s="70" t="n">
-        <v>0.02019244656268053</v>
+        <v>0.02019155198136675</v>
       </c>
       <c r="O7" s="71" t="inlineStr">
         <is>
@@ -42331,10 +42331,10 @@
         </is>
       </c>
       <c r="P7" s="72" t="n">
-        <v>6647.04</v>
+        <v>6629.01</v>
       </c>
       <c r="Q7" s="72" t="n">
-        <v>6781.26</v>
+        <v>6762.86</v>
       </c>
     </row>
     <row r="8">
@@ -42376,7 +42376,7 @@
       </c>
       <c r="B9" s="62" t="n"/>
       <c r="C9" s="73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" s="62" t="n"/>
       <c r="F9" s="62" t="inlineStr">

</xml_diff>

<commit_message>
Günlük kur verisi: 02.09.2026 14:55
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -7078,7 +7078,7 @@
         <v>46267</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
@@ -7098,28 +7098,28 @@
         <v>0.02842045430622513</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>54.9733</v>
+        <v>54.9873</v>
       </c>
       <c r="I2" s="10" t="n">
-        <v>56.5405</v>
+        <v>56.5501</v>
       </c>
       <c r="J2" s="10" t="n">
-        <v>1.5672</v>
+        <v>1.5628</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>0.02850838497961737</v>
+        <v>0.02842110814679026</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>6522.09</v>
+        <v>6538.87</v>
       </c>
       <c r="M2" s="12" t="n">
-        <v>6757.84</v>
+        <v>6775.12</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>235.75</v>
+        <v>236.25</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>0.03614638865762355</v>
+        <v>0.0361300958728343</v>
       </c>
     </row>
     <row r="3">
@@ -7127,7 +7127,7 @@
         <v>46267</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
@@ -7147,28 +7147,28 @@
         <v>0.01630582291166461</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>55.426</v>
+        <v>55.44</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>56.34</v>
+        <v>56.355</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.914</v>
+        <v>0.915</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>0.01649045574279219</v>
+        <v>0.016504329004329</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>6599.06</v>
+        <v>6611.61</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>6734.34</v>
+        <v>6747.97</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>135.28</v>
+        <v>136.36</v>
       </c>
       <c r="O3" s="13" t="n">
-        <v>0.02049988937818416</v>
+        <v>0.02062432599623995</v>
       </c>
     </row>
     <row r="4">
@@ -7176,7 +7176,7 @@
         <v>46267</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -7184,40 +7184,40 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>48.081</v>
+        <v>48.085</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>48.374</v>
+        <v>48.37</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.293</v>
+        <v>0.285</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>0.006093883238701359</v>
+        <v>0.005927004263283769</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>55.473</v>
+        <v>55.498</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>55.983</v>
+        <v>56.001</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.51</v>
+        <v>0.503</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>0.00919366178140717</v>
+        <v>0.009063389671699881</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>6663.18</v>
+        <v>6677.77</v>
       </c>
       <c r="M4" s="12" t="n">
-        <v>6730.38</v>
+        <v>6744.08</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>67.2</v>
+        <v>66.31</v>
       </c>
       <c r="O4" s="13" t="n">
-        <v>0.01008527459861507</v>
+        <v>0.009929961648873801</v>
       </c>
     </row>
     <row r="5">
@@ -7225,7 +7225,7 @@
         <v>46267</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -7233,40 +7233,40 @@
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>48.18</v>
+        <v>48.209</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>48.37</v>
+        <v>48.399</v>
       </c>
       <c r="F5" s="8" t="n">
         <v>0.19</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>0.00394354503943545</v>
+        <v>0.003941172810056214</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>55.658</v>
+        <v>55.718</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>55.978</v>
+        <v>56.039</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.32</v>
+        <v>0.321</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>0.005749398109885372</v>
+        <v>0.00576115438457949</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>6600.17</v>
+        <v>6605.81</v>
       </c>
       <c r="M5" s="12" t="n">
-        <v>6770</v>
+        <v>6780</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>169.83</v>
+        <v>174.19</v>
       </c>
       <c r="O5" s="13" t="n">
-        <v>0.02573115540963338</v>
+        <v>0.02636921134576986</v>
       </c>
     </row>
     <row r="6">
@@ -7274,7 +7274,7 @@
         <v>46267</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
@@ -7282,40 +7282,40 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>47.4536</v>
+        <v>47.4531</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>48.7303</v>
+        <v>48.7296</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>1.2767</v>
+        <v>1.2765</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.02690417586863799</v>
+        <v>0.02690024466262478</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>55.0165</v>
+        <v>55.0428</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>56.3818</v>
+        <v>56.4077</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>1.3653</v>
+        <v>1.3649</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0.02481619150618451</v>
+        <v>0.02479706700967247</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>6595.52</v>
+        <v>6601.16</v>
       </c>
       <c r="M6" s="12" t="n">
-        <v>6746.54</v>
+        <v>6752.06</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>151.02</v>
+        <v>150.9</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>0.02289736063267188</v>
+        <v>0.02285961861248629</v>
       </c>
     </row>
     <row r="7">
@@ -7323,7 +7323,7 @@
         <v>46267</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
@@ -7334,37 +7334,37 @@
         <v>47.302</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>49.226</v>
+        <v>49.225</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>1.924</v>
+        <v>1.923</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>0.04067481290431695</v>
+        <v>0.04065367214916916</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>54.738</v>
+        <v>54.762</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>56.974</v>
+        <v>56.997</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>2.236</v>
+        <v>2.235</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>0.040849135883664</v>
+        <v>0.04081297249917826</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>6589.45</v>
+        <v>6597.34</v>
       </c>
       <c r="M7" s="12" t="n">
-        <v>6783.97</v>
+        <v>6791.54</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>194.52</v>
+        <v>194.2</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>0.02951991440863805</v>
+        <v>0.02943610606699064</v>
       </c>
     </row>
     <row r="8">
@@ -7372,7 +7372,7 @@
         <v>46267</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
@@ -7380,40 +7380,40 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>47.555</v>
+        <v>47.5549</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>48.9551</v>
+        <v>48.955</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>1.4001</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>0.02944169908526969</v>
+        <v>0.02944176099623803</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>55.0301</v>
+        <v>55.0586</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>56.6552</v>
+        <v>56.6845</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>1.6251</v>
+        <v>1.6259</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>0.02953111115553125</v>
+        <v>0.02953035493092814</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>6600.75</v>
+        <v>6612.89</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>6796.06</v>
+        <v>6808.62</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>195.31</v>
+        <v>195.73</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>0.02958906184903231</v>
+        <v>0.02959825431845986</v>
       </c>
     </row>
     <row r="9">
@@ -7421,7 +7421,7 @@
         <v>46267</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -7429,40 +7429,40 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>48.2245</v>
+        <v>48.2242</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>48.2821</v>
+        <v>48.2813</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.0576</v>
+        <v>0.0571</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.001194413627927713</v>
+        <v>0.001184052819953467</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>55.7996</v>
+        <v>55.8185</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>55.8827</v>
+        <v>55.9017</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.08309999999999999</v>
+        <v>0.0832</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>0.001489257987512455</v>
+        <v>0.001490545249334898</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6659.64</v>
+        <v>6667.12</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>6688.18</v>
+        <v>6695.98</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>28.54</v>
+        <v>28.86</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>0.004285516934849331</v>
+        <v>0.004328705648015935</v>
       </c>
     </row>
     <row r="10">
@@ -7470,7 +7470,7 @@
         <v>46267</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -7478,40 +7478,40 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>48.2381</v>
+        <v>48.238</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>48.2772</v>
+        <v>48.2765</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.0391</v>
+        <v>0.0385</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.0008105626050777289</v>
+        <v>0.0007981259587876778</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>55.7767</v>
+        <v>55.7958</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>55.8867</v>
+        <v>55.91</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.11</v>
+        <v>0.1142</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>0.001972149661059188</v>
+        <v>0.002046749038458092</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>6655.84</v>
+        <v>6664.2</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>6687.65</v>
+        <v>6695.84</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>31.81</v>
+        <v>31.64</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>0.004779261520709632</v>
+        <v>0.004747756669967888</v>
       </c>
     </row>
     <row r="11">
@@ -7519,7 +7519,7 @@
         <v>46267</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
@@ -7527,40 +7527,40 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>47.9241</v>
+        <v>47.9238</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>49.1615</v>
+        <v>49.1621</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1.2374</v>
+        <v>1.2383</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.02581999453302201</v>
+        <v>0.025838935977531</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>55.3594</v>
+        <v>55.3734</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>56.6321</v>
+        <v>56.6524</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>1.2727</v>
+        <v>1.279</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>0.02298977228799445</v>
+        <v>0.02309773284645696</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6601.47</v>
+        <v>6616.09</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>6709.49</v>
+        <v>6724.63</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>108.02</v>
+        <v>108.54</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>0.01636302217536397</v>
+        <v>0.01640546002246039</v>
       </c>
     </row>
     <row r="12">
@@ -7568,7 +7568,7 @@
         <v>46267</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
@@ -7588,28 +7588,28 @@
         <v>0.01776477349913789</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>55.2861</v>
+        <v>55.3099</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>56.447</v>
+        <v>56.4666</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>1.1609</v>
+        <v>1.1567</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>0.02099804471648389</v>
+        <v>0.0209130734280843</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>6606.01</v>
+        <v>6612.1</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>6760.81</v>
+        <v>6766.77</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>154.8</v>
+        <v>154.67</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>0.02343320703420067</v>
+        <v>0.02339196321894708</v>
       </c>
     </row>
     <row r="13">
@@ -7617,7 +7617,7 @@
         <v>46267</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
@@ -7625,40 +7625,40 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>47.9985</v>
+        <v>47.9982</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>48.606</v>
+        <v>48.6054</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.6075</v>
+        <v>0.6072</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.01265664552017251</v>
+        <v>0.01265047439278973</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>55.5613</v>
+        <v>55.5764</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>56.2222</v>
+        <v>56.237</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>0.6609</v>
+        <v>0.6606</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>0.01189497006009579</v>
+        <v>0.01188634024514002</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6670.14</v>
+        <v>6683.15</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>6724.29</v>
+        <v>6737.49</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>54.15</v>
+        <v>54.34</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>0.008118270381131431</v>
+        <v>0.008130896358752984</v>
       </c>
     </row>
     <row r="14">
@@ -7666,7 +7666,7 @@
         <v>46267</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
@@ -7674,40 +7674,40 @@
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>47.455</v>
+        <v>47.454</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>48.805</v>
+        <v>48.804</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>1.35</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>0.02844800337161522</v>
+        <v>0.02844860285750411</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>54.914</v>
+        <v>54.935</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>56.477</v>
+        <v>56.498</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>1.563</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>0.028462687110755</v>
+        <v>0.02845180668062255</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>6562.01</v>
+        <v>6580.71</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>6804.43</v>
+        <v>6823.81</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>242.42</v>
+        <v>243.1</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>0.03694294888304041</v>
+        <v>0.03694130268618432</v>
       </c>
     </row>
     <row r="15">
@@ -7715,7 +7715,7 @@
         <v>46267</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
@@ -7723,40 +7723,40 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>47.9988</v>
+        <v>47.9984</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>48.6058</v>
+        <v>48.6053</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.607</v>
+        <v>0.6069</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>0.01264614948707051</v>
+        <v>0.01264417147238241</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>55.5608</v>
+        <v>55.5861</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>56.2216</v>
+        <v>56.2467</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>0.6608000000000001</v>
+        <v>0.6606</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>0.01189327727462528</v>
+        <v>0.01188426603053641</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>6679.6</v>
+        <v>6685.19</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>6734.63</v>
+        <v>6739.53</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>55.03</v>
+        <v>54.34</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>0.008238517276483621</v>
+        <v>0.008128415198371325</v>
       </c>
     </row>
     <row r="16">
@@ -7764,7 +7764,7 @@
         <v>46267</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
@@ -7772,40 +7772,40 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>47.8675</v>
+        <v>47.8672</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>48.8475</v>
+        <v>48.8472</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>0.98</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>0.02047318117720792</v>
+        <v>0.02047330948958786</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>55.3947</v>
+        <v>55.4111</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>56.5288</v>
+        <v>56.5455</v>
       </c>
       <c r="J16" s="10" t="n">
-        <v>1.1341</v>
+        <v>1.1344</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>0.02047307774931537</v>
+        <v>0.0204724324187753</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>6596.25</v>
+        <v>6611.86</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>6798.84</v>
+        <v>6814.92</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>202.59</v>
+        <v>203.06</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>0.03071290505969301</v>
+        <v>0.03071147906942978</v>
       </c>
     </row>
     <row r="17">
@@ -7813,7 +7813,7 @@
         <v>46267</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
@@ -7821,40 +7821,40 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>48.24</v>
+        <v>48.25</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>48.309</v>
+        <v>48.31</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.001430348258706468</v>
+        <v>0.001243523316062176</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>55.682</v>
+        <v>55.718</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>55.86</v>
+        <v>55.887</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>0.178</v>
+        <v>0.169</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>0.003196724255594268</v>
+        <v>0.003033131124591694</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>6616.79</v>
+        <v>6628.13</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>6705.79</v>
+        <v>6713.71</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>89</v>
+        <v>85.58</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>0.01345063089504125</v>
+        <v>0.01291163571022294</v>
       </c>
     </row>
     <row r="18">
@@ -7862,7 +7862,7 @@
         <v>46267</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
@@ -7870,40 +7870,40 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>48.2187</v>
+        <v>48.218</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>48.3651</v>
+        <v>48.3648</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>0.1464</v>
+        <v>0.1468</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.003036166466536842</v>
+        <v>0.003044506201003774</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>55.7901</v>
+        <v>55.8086</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>55.9613</v>
+        <v>55.9803</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>0.1712</v>
+        <v>0.1717</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>0.003068644795402769</v>
+        <v>0.003076586762613647</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>6666</v>
+        <v>6673.84</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>6713.15</v>
+        <v>6721.1</v>
       </c>
       <c r="N18" s="12" t="n">
-        <v>47.15</v>
+        <v>47.26</v>
       </c>
       <c r="O18" s="13" t="n">
-        <v>0.007073207320732073</v>
+        <v>0.007081380434652315</v>
       </c>
     </row>
     <row r="19">
@@ -7911,7 +7911,7 @@
         <v>46267</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
@@ -7927,16 +7927,16 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="12" t="n">
-        <v>6669.35</v>
+        <v>6681.95</v>
       </c>
       <c r="M19" s="12" t="n">
-        <v>6864.8</v>
+        <v>6877.67</v>
       </c>
       <c r="N19" s="12" t="n">
-        <v>195.45</v>
+        <v>195.72</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>0.02930570445395728</v>
+        <v>0.02929085072471359</v>
       </c>
     </row>
     <row r="20">
@@ -7944,7 +7944,7 @@
         <v>46267</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C20" s="31" t="inlineStr">
         <is>
@@ -7952,40 +7952,40 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>47.8049</v>
+        <v>47.7933</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>48.6915</v>
+        <v>48.6799</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>0.8866000000000001</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>0.01854621597367634</v>
+        <v>0.01855071735996468</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>55.3246</v>
+        <v>55.3353</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>56.3839</v>
+        <v>56.3898</v>
       </c>
       <c r="J20" s="10" t="n">
-        <v>1.0593</v>
+        <v>1.0545</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>0.0191469978996685</v>
+        <v>0.01905655160449117</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>6610.81</v>
+        <v>6617.13</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>7056.88</v>
+        <v>7063.22</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>446.07</v>
+        <v>446.09</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>0.06747584637888548</v>
+        <v>0.06741442286912906</v>
       </c>
     </row>
     <row r="21">
@@ -7993,7 +7993,7 @@
         <v>46267</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
@@ -8001,40 +8001,40 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>47.7518</v>
+        <v>47.7514</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>48.7551</v>
+        <v>48.7549</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.0033</v>
+        <v>1.0035</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.02101072629722859</v>
+        <v>0.02101509065702786</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>55.3409</v>
+        <v>55.357</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>56.3476</v>
+        <v>56.367</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>1.0067</v>
+        <v>1.01</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>0.01819088594511473</v>
+        <v>0.01824520837473129</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>6571.18</v>
+        <v>6583.01</v>
       </c>
       <c r="M21" s="12" t="n">
-        <v>6823.01</v>
+        <v>6835.05</v>
       </c>
       <c r="N21" s="12" t="n">
-        <v>251.83</v>
+        <v>252.04</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>0.03832340614623249</v>
+        <v>0.03828643735920195</v>
       </c>
     </row>
     <row r="22">
@@ -8042,7 +8042,7 @@
         <v>46267</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -8050,40 +8050,40 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>47.6776</v>
+        <v>47.6786</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>48.8354</v>
+        <v>48.8336</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.1578</v>
+        <v>1.155</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>0.02428394046680202</v>
+        <v>0.02422470458444669</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>55.1678</v>
+        <v>55.1928</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>56.5123</v>
+        <v>56.5298</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>1.3445</v>
+        <v>1.337</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>0.0243711005332821</v>
+        <v>0.02422417416764506</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>6595.24</v>
+        <v>6604.6</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>6776.85</v>
+        <v>6785.71</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>181.61</v>
+        <v>181.11</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>0.02753652634324149</v>
+        <v>0.02742179692941283</v>
       </c>
     </row>
     <row r="23">
@@ -8091,7 +8091,7 @@
         <v>46267</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C23" s="34" t="inlineStr">
         <is>
@@ -8099,16 +8099,16 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>48.28</v>
+        <v>48.27</v>
       </c>
       <c r="E23" s="8" t="n">
         <v>48.29</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>0.0002071251035625518</v>
+        <v>0.0004143360265175057</v>
       </c>
       <c r="H23" s="10" t="n">
         <v>55.75</v>
@@ -8123,16 +8123,16 @@
         <v>0.0008968609865470851</v>
       </c>
       <c r="L23" s="12" t="n">
-        <v>6669.43</v>
+        <v>6682.61</v>
       </c>
       <c r="M23" s="12" t="n">
-        <v>6675.67</v>
+        <v>6690.23</v>
       </c>
       <c r="N23" s="12" t="n">
-        <v>6.24</v>
+        <v>7.62</v>
       </c>
       <c r="O23" s="13" t="n">
-        <v>0.0009356121887477641</v>
+        <v>0.001140273037031938</v>
       </c>
     </row>
     <row r="24">
@@ -8140,7 +8140,7 @@
         <v>46267</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
@@ -8148,40 +8148,40 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>47.6134</v>
+        <v>47.613</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>48.5996</v>
+        <v>48.5991</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>0.9862</v>
+        <v>0.9861</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.0207126565210634</v>
+        <v>0.02071073026274337</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>55.1015</v>
+        <v>55.1196</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>56.2432</v>
+        <v>56.2617</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>1.1417</v>
+        <v>1.1421</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>0.02071994410315509</v>
+        <v>0.02072039710012409</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>6557.78</v>
+        <v>6578.23</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>6731.8</v>
+        <v>6752.43</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>174.02</v>
+        <v>174.2</v>
       </c>
       <c r="O24" s="13" t="n">
-        <v>0.02653641933703174</v>
+        <v>0.02648128751959113</v>
       </c>
     </row>
     <row r="25">
@@ -8189,7 +8189,7 @@
         <v>46267</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
@@ -8230,7 +8230,7 @@
         <v>46267</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
@@ -8238,40 +8238,40 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>48.2274</v>
+        <v>48.227</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>48.2805</v>
+        <v>48.2804</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>0.0531</v>
+        <v>0.0534</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>0.001101033852125555</v>
+        <v>0.001107263566052211</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>55.798</v>
+        <v>55.8172</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>55.8776</v>
+        <v>55.8979</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>0.0796</v>
+        <v>0.08069999999999999</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>0.00142657442919101</v>
+        <v>0.001445790903162466</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>6658.48</v>
+        <v>6662.57</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>6686.88</v>
+        <v>6690.94</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>28.4</v>
+        <v>28.37</v>
       </c>
       <c r="O26" s="13" t="n">
-        <v>0.004265237711910226</v>
+        <v>0.004258116612658479</v>
       </c>
     </row>
     <row r="27">
@@ -8279,7 +8279,7 @@
         <v>46267</v>
       </c>
       <c r="B27" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C27" s="38" t="inlineStr">
         <is>
@@ -8287,40 +8287,40 @@
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>48.256</v>
+        <v>48.265</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>48.355</v>
+        <v>48.366</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.099</v>
+        <v>0.101</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>0.002051558355437666</v>
+        <v>0.002092613695224283</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>55.697</v>
+        <v>55.733</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>55.918</v>
+        <v>55.962</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>0.221</v>
+        <v>0.229</v>
       </c>
       <c r="K27" s="11" t="n">
-        <v>0.003967897732373377</v>
+        <v>0.004108876249259864</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>6636</v>
+        <v>6638</v>
       </c>
       <c r="M27" s="12" t="n">
-        <v>6687</v>
+        <v>6693</v>
       </c>
       <c r="N27" s="12" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>0.007685352622061483</v>
+        <v>0.008285628201265442</v>
       </c>
     </row>
     <row r="28">
@@ -8328,7 +8328,7 @@
         <v>46267</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -8336,40 +8336,40 @@
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>47.762</v>
+        <v>47.7615</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>48.762</v>
+        <v>48.7615</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>0.02093714668564968</v>
+        <v>0.02093736586999989</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>55.301</v>
+        <v>55.318</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>56.391</v>
+        <v>56.408</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>1.09</v>
       </c>
       <c r="K28" s="11" t="n">
-        <v>0.01971031265257409</v>
+        <v>0.01970425539607361</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>6644.9</v>
+        <v>6663.22</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>6744.9</v>
+        <v>6763.22</v>
       </c>
       <c r="N28" s="12" t="n">
         <v>100</v>
       </c>
       <c r="O28" s="13" t="n">
-        <v>0.01504913542716971</v>
+        <v>0.0150077590114089</v>
       </c>
     </row>
     <row r="29">
@@ -8377,7 +8377,7 @@
         <v>46267</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
@@ -8393,16 +8393,16 @@
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="12" t="n">
-        <v>6667.97</v>
+        <v>6681.95</v>
       </c>
       <c r="M29" s="12" t="n">
-        <v>6849.7</v>
+        <v>6863.94</v>
       </c>
       <c r="N29" s="12" t="n">
-        <v>181.73</v>
+        <v>181.99</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>0.02725417180941126</v>
+        <v>0.02723606132940234</v>
       </c>
     </row>
     <row r="30">
@@ -8410,7 +8410,7 @@
         <v>46267</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C30" s="41" t="inlineStr">
         <is>
@@ -8430,28 +8430,28 @@
         <v>0.02558322411533421</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>55.0681</v>
+        <v>55.0919</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>56.7244</v>
+        <v>56.7489</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>1.6563</v>
+        <v>1.657</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>0.03007730428324202</v>
+        <v>0.03007701676653011</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>6578.08</v>
+        <v>6586.13</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>6776.19</v>
+        <v>6784.36</v>
       </c>
       <c r="N30" s="12" t="n">
-        <v>198.11</v>
+        <v>198.23</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>0.03011669058448666</v>
+        <v>0.03009810009823675</v>
       </c>
     </row>
     <row r="31">
@@ -8459,7 +8459,7 @@
         <v>46267</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -8467,40 +8467,40 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>48.153</v>
+        <v>48.1413</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>48.3944</v>
+        <v>48.3827</v>
       </c>
       <c r="F31" s="8" t="n">
         <v>0.2414</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>0.005013187132681245</v>
+        <v>0.005014405510445293</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>55.6683</v>
+        <v>55.6806</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>56.0036</v>
+        <v>56.016</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>0.3353</v>
+        <v>0.3354</v>
       </c>
       <c r="K31" s="11" t="n">
-        <v>0.006023176565478019</v>
+        <v>0.006023641986616523</v>
       </c>
       <c r="L31" s="12" t="n">
-        <v>6593.08</v>
+        <v>6598.67</v>
       </c>
       <c r="M31" s="12" t="n">
-        <v>6726.61</v>
+        <v>6732.31</v>
       </c>
       <c r="N31" s="12" t="n">
-        <v>133.53</v>
+        <v>133.64</v>
       </c>
       <c r="O31" s="13" t="n">
-        <v>0.02025305320123524</v>
+        <v>0.02025256604740046</v>
       </c>
     </row>
     <row r="32">
@@ -8508,7 +8508,7 @@
         <v>46267</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C32" s="43" t="inlineStr">
         <is>
@@ -8516,40 +8516,40 @@
         </is>
       </c>
       <c r="D32" s="8" t="n">
-        <v>47.8522</v>
+        <v>47.8518</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>48.6544</v>
+        <v>48.6541</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.8022</v>
+        <v>0.8023</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>0.01676411951801589</v>
+        <v>0.01676634943722075</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>55.4133</v>
+        <v>55.4245</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>56.2636</v>
+        <v>56.2748</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>0.8502999999999999</v>
       </c>
       <c r="K32" s="11" t="n">
-        <v>0.0153446916173554</v>
+        <v>0.01534159081272722</v>
       </c>
       <c r="L32" s="12" t="n">
-        <v>6595.3</v>
+        <v>6611.43</v>
       </c>
       <c r="M32" s="12" t="n">
-        <v>6791.42</v>
+        <v>6807.72</v>
       </c>
       <c r="N32" s="12" t="n">
-        <v>196.12</v>
+        <v>196.29</v>
       </c>
       <c r="O32" s="13" t="n">
-        <v>0.02973632738465271</v>
+        <v>0.02968949228835517</v>
       </c>
     </row>
     <row r="33">
@@ -8557,7 +8557,7 @@
         <v>46267</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
@@ -8565,40 +8565,40 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>48.1543</v>
+        <v>48.1538</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>48.3575</v>
+        <v>48.357</v>
       </c>
       <c r="F33" s="8" t="n">
         <v>0.2032</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>0.004219768535727858</v>
+        <v>0.004219812351257845</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>55.7174</v>
+        <v>55.7353</v>
       </c>
       <c r="I33" s="10" t="n">
-        <v>55.942</v>
+        <v>55.9599</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>0.2246</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>0.004031056725547136</v>
+        <v>0.004029762107676822</v>
       </c>
       <c r="L33" s="12" t="n">
-        <v>6638.6</v>
+        <v>6650.43</v>
       </c>
       <c r="M33" s="12" t="n">
-        <v>6691.93</v>
+        <v>6703.85</v>
       </c>
       <c r="N33" s="12" t="n">
-        <v>53.33</v>
+        <v>53.42</v>
       </c>
       <c r="O33" s="13" t="n">
-        <v>0.008033320278371945</v>
+        <v>0.00803256330793648</v>
       </c>
     </row>
     <row r="34">
@@ -8606,7 +8606,7 @@
         <v>46267</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C34" s="45" t="inlineStr">
         <is>
@@ -8626,28 +8626,28 @@
         <v>0.02006489249309943</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>55.4497</v>
+        <v>55.4653</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>56.5517</v>
+        <v>56.5673</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>1.102</v>
       </c>
       <c r="K34" s="11" t="n">
-        <v>0.01987386766745357</v>
+        <v>0.01986827800444602</v>
       </c>
       <c r="L34" s="12" t="n">
-        <v>6594.99</v>
+        <v>6617.75</v>
       </c>
       <c r="M34" s="12" t="n">
-        <v>6739.59</v>
+        <v>6762.35</v>
       </c>
       <c r="N34" s="12" t="n">
         <v>144.6</v>
       </c>
       <c r="O34" s="13" t="n">
-        <v>0.02192573453485146</v>
+        <v>0.02185032677269465</v>
       </c>
     </row>
     <row r="35">
@@ -8655,7 +8655,7 @@
         <v>46267</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C35" s="46" t="inlineStr">
         <is>
@@ -8663,28 +8663,28 @@
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>48.255</v>
+        <v>48.271</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>48.3</v>
+        <v>48.31</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.045</v>
+        <v>0.039</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>0.0009325458501709667</v>
+        <v>0.000807938513807462</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>55.73</v>
+        <v>55.772</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>55.824</v>
+        <v>55.875</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>0.094</v>
+        <v>0.103</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>0.001686703750224296</v>
+        <v>0.00184680484831098</v>
       </c>
       <c r="L35" s="12" t="n"/>
       <c r="M35" s="12" t="n"/>
@@ -8696,7 +8696,7 @@
         <v>46267</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C36" s="47" t="inlineStr">
         <is>
@@ -8707,37 +8707,37 @@
         <v>47.65</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>48.66</v>
+        <v>48.65</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="G36" s="9" t="n">
-        <v>0.02119622245540399</v>
+        <v>0.02098635886673662</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>55.15</v>
+        <v>55.17</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>56.29</v>
+        <v>56.31</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>1.14</v>
       </c>
       <c r="K36" s="11" t="n">
-        <v>0.02067089755213055</v>
+        <v>0.02066340402392605</v>
       </c>
       <c r="L36" s="12" t="n">
-        <v>6569.54</v>
+        <v>6584.64</v>
       </c>
       <c r="M36" s="12" t="n">
-        <v>6771.48</v>
+        <v>6786.98</v>
       </c>
       <c r="N36" s="12" t="n">
-        <v>201.94</v>
+        <v>202.34</v>
       </c>
       <c r="O36" s="13" t="n">
-        <v>0.03073883407361855</v>
+        <v>0.03072909073237109</v>
       </c>
     </row>
     <row r="37">
@@ -8745,7 +8745,7 @@
         <v>46267</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C37" s="48" t="inlineStr">
         <is>
@@ -8753,40 +8753,40 @@
         </is>
       </c>
       <c r="D37" s="8" t="n">
-        <v>47.8908</v>
+        <v>47.8905</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>48.8596</v>
+        <v>48.8593</v>
       </c>
       <c r="F37" s="8" t="n">
         <v>0.9688</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>0.02022935511622274</v>
+        <v>0.02022948183877804</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>55.4124</v>
+        <v>55.4241</v>
       </c>
       <c r="I37" s="10" t="n">
-        <v>56.5334</v>
+        <v>56.5454</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1.121</v>
+        <v>1.1213</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>0.02023012899639792</v>
+        <v>0.02023127123399388</v>
       </c>
       <c r="L37" s="12" t="n">
-        <v>6629.01</v>
+        <v>6650.94</v>
       </c>
       <c r="M37" s="12" t="n">
-        <v>6762.86</v>
+        <v>6785.23</v>
       </c>
       <c r="N37" s="12" t="n">
-        <v>133.85</v>
+        <v>134.29</v>
       </c>
       <c r="O37" s="13" t="n">
-        <v>0.02019155198136675</v>
+        <v>0.02019113087774059</v>
       </c>
     </row>
     <row r="38">
@@ -8794,7 +8794,7 @@
         <v>46267</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
@@ -8802,40 +8802,40 @@
         </is>
       </c>
       <c r="D38" s="8" t="n">
-        <v>47.9387</v>
+        <v>47.9384</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>48.5909</v>
+        <v>48.5906</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>0.6522</v>
       </c>
       <c r="G38" s="9" t="n">
-        <v>0.01360487455855082</v>
+        <v>0.01360495969827946</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>55.4124</v>
+        <v>55.4326</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>56.2225</v>
+        <v>56.243</v>
       </c>
       <c r="J38" s="10" t="n">
-        <v>0.8101</v>
+        <v>0.8104</v>
       </c>
       <c r="K38" s="11" t="n">
-        <v>0.01461947145404278</v>
+        <v>0.01461955600134217</v>
       </c>
       <c r="L38" s="12" t="n">
-        <v>6607.06</v>
+        <v>6620.42</v>
       </c>
       <c r="M38" s="12" t="n">
-        <v>6740.46</v>
+        <v>6754.09</v>
       </c>
       <c r="N38" s="12" t="n">
-        <v>133.4</v>
+        <v>133.67</v>
       </c>
       <c r="O38" s="13" t="n">
-        <v>0.02019052347034838</v>
+        <v>0.02019056192809519</v>
       </c>
     </row>
     <row r="39">
@@ -8843,7 +8843,7 @@
         <v>46267</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="C39" s="50" t="inlineStr">
         <is>
@@ -8851,40 +8851,40 @@
         </is>
       </c>
       <c r="D39" s="8" t="n">
-        <v>47.769</v>
+        <v>47.7683</v>
       </c>
       <c r="E39" s="8" t="n">
         <v>48.766</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.997</v>
+        <v>0.9977</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>0.02087127635077142</v>
+        <v>0.02088623626966001</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>55.2408</v>
+        <v>55.2548</v>
       </c>
       <c r="I39" s="10" t="n">
-        <v>56.4494</v>
+        <v>56.4646</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1.2086</v>
+        <v>1.2098</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>0.02187875628158897</v>
+        <v>0.02189493039518739</v>
       </c>
       <c r="L39" s="12" t="n">
-        <v>6627.03</v>
+        <v>6640.01</v>
       </c>
       <c r="M39" s="12" t="n">
-        <v>6837.43</v>
+        <v>6850.92</v>
       </c>
       <c r="N39" s="12" t="n">
-        <v>210.4</v>
+        <v>210.91</v>
       </c>
       <c r="O39" s="13" t="n">
-        <v>0.03174876226605282</v>
+        <v>0.03176350638026148</v>
       </c>
     </row>
   </sheetData>
@@ -42186,7 +42186,7 @@
       </c>
       <c r="B5" s="62" t="n"/>
       <c r="C5" s="64" t="n">
-        <v>0.5944791666666667</v>
+        <v>0.6215046296296296</v>
       </c>
       <c r="D5" s="62" t="n"/>
       <c r="F5" s="62" t="inlineStr">
@@ -42217,7 +42217,7 @@
         <v>5</v>
       </c>
       <c r="N5" s="70" t="n">
-        <v>0.02022935511622274</v>
+        <v>0.02022948183877804</v>
       </c>
       <c r="O5" s="71" t="inlineStr">
         <is>
@@ -42225,10 +42225,10 @@
         </is>
       </c>
       <c r="P5" s="72" t="n">
-        <v>47.8908</v>
+        <v>47.8905</v>
       </c>
       <c r="Q5" s="72" t="n">
-        <v>48.8596</v>
+        <v>48.8593</v>
       </c>
     </row>
     <row r="6">
@@ -42270,7 +42270,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="70" t="n">
-        <v>0.02023012899639792</v>
+        <v>0.02023127123399388</v>
       </c>
       <c r="O6" s="71" t="inlineStr">
         <is>
@@ -42278,10 +42278,10 @@
         </is>
       </c>
       <c r="P6" s="72" t="n">
-        <v>55.4124</v>
+        <v>55.4241</v>
       </c>
       <c r="Q6" s="72" t="n">
-        <v>56.5334</v>
+        <v>56.5454</v>
       </c>
     </row>
     <row r="7">
@@ -42323,7 +42323,7 @@
         <v>5</v>
       </c>
       <c r="N7" s="70" t="n">
-        <v>0.02019155198136675</v>
+        <v>0.02019113087774059</v>
       </c>
       <c r="O7" s="71" t="inlineStr">
         <is>
@@ -42331,10 +42331,10 @@
         </is>
       </c>
       <c r="P7" s="72" t="n">
-        <v>6629.01</v>
+        <v>6650.94</v>
       </c>
       <c r="Q7" s="72" t="n">
-        <v>6762.86</v>
+        <v>6785.23</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Günlük kur verisi: 07.09.2026 15:27
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -7978,7 +7978,7 @@
         <v>46272</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
@@ -7998,28 +7998,28 @@
         <v>0.02833931607783866</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>55.373</v>
+        <v>55.3683</v>
       </c>
       <c r="I2" s="10" t="n">
-        <v>56.9472</v>
+        <v>56.9423</v>
       </c>
       <c r="J2" s="10" t="n">
-        <v>1.5742</v>
+        <v>1.574</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>0.02842901775233417</v>
+        <v>0.02842781880606773</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>6657.35</v>
+        <v>6660.62</v>
       </c>
       <c r="M2" s="12" t="n">
-        <v>6897.31</v>
+        <v>6900.64</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>239.96</v>
+        <v>240.02</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>0.03604437200988381</v>
+        <v>0.03603568436571971</v>
       </c>
     </row>
     <row r="3">
@@ -8027,7 +8027,7 @@
         <v>46272</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
@@ -8050,25 +8050,25 @@
         <v>55.833</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>56.747</v>
+        <v>56.752</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.914</v>
+        <v>0.919</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>0.01637024698654917</v>
+        <v>0.01645979975999857</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>6733.07</v>
+        <v>6736.66</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>6871.02</v>
+        <v>6875.37</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>137.95</v>
+        <v>138.71</v>
       </c>
       <c r="O3" s="13" t="n">
-        <v>0.02048842504236552</v>
+        <v>0.02059032220714716</v>
       </c>
     </row>
     <row r="4">
@@ -8076,7 +8076,7 @@
         <v>46272</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -8096,28 +8096,28 @@
         <v>0.00591028804877543</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>55.882</v>
+        <v>55.886</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>56.387</v>
+        <v>56.39</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.505</v>
+        <v>0.504</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>0.009036899180415876</v>
+        <v>0.009018358801846616</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>6795.61</v>
+        <v>6797.96</v>
       </c>
       <c r="M4" s="12" t="n">
-        <v>6862.87</v>
+        <v>6865.18</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>67.26000000000001</v>
+        <v>67.22</v>
       </c>
       <c r="O4" s="13" t="n">
-        <v>0.009897566222899784</v>
+        <v>0.009888260595825807</v>
       </c>
     </row>
     <row r="5">
@@ -8125,7 +8125,7 @@
         <v>46272</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -8133,40 +8133,40 @@
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>48.238</v>
+        <v>48.24</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>48.429</v>
+        <v>48.43</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.191</v>
+        <v>0.19</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>0.003959533977362245</v>
+        <v>0.003938640132669983</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>55.923</v>
+        <v>55.927</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>56.296</v>
+        <v>56.299</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.373</v>
+        <v>0.372</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>0.006669885378109186</v>
+        <v>0.006651527884563806</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>6726.76</v>
+        <v>6729.84</v>
       </c>
       <c r="M5" s="12" t="n">
-        <v>6880</v>
+        <v>6885</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>153.24</v>
+        <v>155.16</v>
       </c>
       <c r="O5" s="13" t="n">
-        <v>0.02278065517425923</v>
+        <v>0.023055525837167</v>
       </c>
     </row>
     <row r="6">
@@ -8174,7 +8174,7 @@
         <v>46272</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
@@ -8182,40 +8182,40 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>47.5888</v>
+        <v>47.589</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>48.8656</v>
+        <v>48.8657</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>1.2768</v>
+        <v>1.2767</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.02682984231583902</v>
+        <v>0.02682762823341529</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>55.4225</v>
+        <v>55.4271</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>56.7891</v>
+        <v>56.7918</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>1.3666</v>
+        <v>1.3647</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0.02465785556407596</v>
+        <v>0.02462152990143811</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>6719.65</v>
+        <v>6723.12</v>
       </c>
       <c r="M6" s="12" t="n">
-        <v>6870.84</v>
+        <v>6874.44</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>151.19</v>
+        <v>151.32</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>0.02249968376329124</v>
+        <v>0.02250740727519366</v>
       </c>
     </row>
     <row r="7">
@@ -8223,7 +8223,7 @@
         <v>46272</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
@@ -8243,28 +8243,28 @@
         <v>0.04062315540939371</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>55.138</v>
+        <v>55.139</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>57.383</v>
+        <v>57.39</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>2.245</v>
+        <v>2.251</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>0.04071602161848453</v>
+        <v>0.04082409909501442</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>6717.9</v>
+        <v>6720.22</v>
       </c>
       <c r="M7" s="12" t="n">
-        <v>6912.59</v>
+        <v>6915.18</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>194.69</v>
+        <v>194.96</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>0.02898078268506527</v>
+        <v>0.02901095499849707</v>
       </c>
     </row>
     <row r="8">
@@ -8272,7 +8272,7 @@
         <v>46272</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
@@ -8280,40 +8280,40 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>47.7164</v>
+        <v>47.7166</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>49.0645</v>
+        <v>49.0647</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>1.3481</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>0.02825234091423494</v>
+        <v>0.02825222249699266</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>55.463</v>
+        <v>55.4701</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>57.0349</v>
+        <v>57.0372</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>1.5719</v>
+        <v>1.5671</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>0.02834141680038945</v>
+        <v>0.02825125608210549</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>6736.74</v>
+        <v>6739.25</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>6928.2</v>
+        <v>6930.74</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>191.46</v>
+        <v>191.49</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>0.02842027449478531</v>
+        <v>0.02841414103943317</v>
       </c>
     </row>
     <row r="9">
@@ -8321,7 +8321,7 @@
         <v>46272</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -8329,40 +8329,40 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>48.3594</v>
+        <v>48.3605</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>48.4164</v>
+        <v>48.4173</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.057</v>
+        <v>0.0568</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.001178674673383044</v>
+        <v>0.001174512256903878</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>56.2018</v>
+        <v>56.2081</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>56.2851</v>
+        <v>56.2912</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.0833</v>
+        <v>0.08309999999999999</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>0.001482158934411353</v>
+        <v>0.001478434602841939</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6785.55</v>
+        <v>6789.5</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>6814.43</v>
+        <v>6818.36</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>28.88</v>
+        <v>28.86</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>0.004256103042494713</v>
+        <v>0.004250681198910082</v>
       </c>
     </row>
     <row r="10">
@@ -8370,7 +8370,7 @@
         <v>46272</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -8378,40 +8378,40 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>48.3723</v>
+        <v>48.3736</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>48.4116</v>
+        <v>48.4121</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.0393</v>
+        <v>0.0385</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.0008124484467350115</v>
+        <v>0.0007958886665453883</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>56.1827</v>
+        <v>56.1847</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>56.2939</v>
+        <v>56.2947</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.1112</v>
+        <v>0.11</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>0.001979256959882669</v>
+        <v>0.001957828376764493</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>6781.71</v>
+        <v>6785.65</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>6814.29</v>
+        <v>6818</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>32.58</v>
+        <v>32.35</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>0.004804098081457331</v>
+        <v>0.004767413586023447</v>
       </c>
     </row>
     <row r="11">
@@ -8419,7 +8419,7 @@
         <v>46272</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
@@ -8427,40 +8427,40 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>48.0637</v>
+        <v>48.0639</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>49.3044</v>
+        <v>49.3043</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1.2407</v>
+        <v>1.2404</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.02581365978898836</v>
+        <v>0.02580731068431817</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>55.7576</v>
+        <v>55.7531</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>57.0416</v>
+        <v>57.0317</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>1.284</v>
+        <v>1.2786</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>0.02302825085728223</v>
+        <v>0.0229332539356556</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6727.54</v>
+        <v>6735.41</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>6838.23</v>
+        <v>6845.39</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>110.69</v>
+        <v>109.98</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>0.01645326523513796</v>
+        <v>0.0163286273589878</v>
       </c>
     </row>
     <row r="12">
@@ -8468,7 +8468,7 @@
         <v>46272</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
@@ -8491,25 +8491,25 @@
         <v>55.6918</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>56.8535</v>
+        <v>56.8584</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>1.1617</v>
+        <v>1.1666</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>0.02085944429880162</v>
+        <v>0.02094742852628214</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>6731.19</v>
+        <v>6733.89</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>6887.46</v>
+        <v>6890.21</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>156.27</v>
+        <v>156.32</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>0.02321580582333882</v>
+        <v>0.02321392241334503</v>
       </c>
     </row>
     <row r="13">
@@ -8517,7 +8517,7 @@
         <v>46272</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
@@ -8525,40 +8525,40 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>48.134</v>
+        <v>48.1339</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>48.7414</v>
+        <v>48.7411</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.6074000000000001</v>
+        <v>0.6072</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.01261893879586155</v>
+        <v>0.01261480993644812</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>55.9673</v>
+        <v>55.9701</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>56.6287</v>
+        <v>56.6307</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>0.6614</v>
+        <v>0.6606</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>0.0118176149287173</v>
+        <v>0.01180273038640274</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6803.39</v>
+        <v>6805.56</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>6857.65</v>
+        <v>6859.83</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>54.26</v>
+        <v>54.27</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>0.007975435775400205</v>
+        <v>0.007974362139192073</v>
       </c>
     </row>
     <row r="14">
@@ -8566,7 +8566,7 @@
         <v>46272</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
@@ -8586,28 +8586,28 @@
         <v>0.02836730405547384</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>55.314</v>
+        <v>55.324</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>56.883</v>
+        <v>56.893</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>1.569</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>0.02836533246556026</v>
+        <v>0.02836020533583978</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>6692.96</v>
+        <v>6701.54</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>6940.09</v>
+        <v>6948.99</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>247.13</v>
+        <v>247.45</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>0.03692387224785446</v>
+        <v>0.03692434873178404</v>
       </c>
     </row>
     <row r="15">
@@ -8615,7 +8615,7 @@
         <v>46272</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
@@ -8623,40 +8623,40 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>48.1339</v>
+        <v>48.134</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>48.7412</v>
+        <v>48.7411</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.6073</v>
+        <v>0.6071</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>0.01261688747431644</v>
+        <v>0.01261270619520505</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>55.967</v>
+        <v>55.971</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>56.6282</v>
+        <v>56.6317</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>0.6612</v>
+        <v>0.6607</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>0.01181410474029339</v>
+        <v>0.0118043272408926</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>6805.6</v>
+        <v>6808.24</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>6859.86</v>
+        <v>6862.45</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>54.26</v>
+        <v>54.21</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>0.007972845891618667</v>
+        <v>0.007962410255807668</v>
       </c>
     </row>
     <row r="16">
@@ -8664,7 +8664,7 @@
         <v>46272</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
@@ -8696,16 +8696,16 @@
         <v>0.02041346632880179</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>6732.43</v>
+        <v>6736.14</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>6939.17</v>
+        <v>6942.6</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>206.74</v>
+        <v>206.46</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>0.03070808014342518</v>
+        <v>0.03064960051305347</v>
       </c>
     </row>
     <row r="17">
@@ -8713,7 +8713,7 @@
         <v>46272</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
@@ -8721,40 +8721,40 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>48.273</v>
+        <v>48.2839</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>48.338</v>
+        <v>48.3438</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.065</v>
+        <v>0.0599</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.001346508400140865</v>
+        <v>0.001240579157855931</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>55.959</v>
+        <v>55.975</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>56.119</v>
+        <v>56.129</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>0.16</v>
+        <v>0.154</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>0.00285923622652299</v>
+        <v>0.002751228226887003</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>6748.33</v>
+        <v>6750.36</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>6818.55</v>
+        <v>6822.33</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>70.22</v>
+        <v>71.97</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>0.01040553736998635</v>
+        <v>0.01066165360069685</v>
       </c>
     </row>
     <row r="18">
@@ -8762,7 +8762,7 @@
         <v>46272</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
@@ -8770,40 +8770,40 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>48.3527</v>
+        <v>48.3539</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>48.4995</v>
+        <v>48.5005</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>0.1468</v>
+        <v>0.1466</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.003036024875549866</v>
+        <v>0.003031813359418785</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>56.1941</v>
+        <v>56.1979</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>56.3665</v>
+        <v>56.3701</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>0.1724</v>
+        <v>0.1722</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>0.00306793773723576</v>
+        <v>0.003064171437010991</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>6791.9</v>
+        <v>6795.78</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>6839.98</v>
+        <v>6843.86</v>
       </c>
       <c r="N18" s="12" t="n">
         <v>48.08</v>
       </c>
       <c r="O18" s="13" t="n">
-        <v>0.007079020598065342</v>
+        <v>0.007074978883954454</v>
       </c>
     </row>
     <row r="19">
@@ -8811,7 +8811,7 @@
         <v>46272</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
@@ -8827,16 +8827,16 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="12" t="n">
-        <v>6791.45</v>
+        <v>6795.96</v>
       </c>
       <c r="M19" s="12" t="n">
-        <v>6989.72</v>
+        <v>6994.34</v>
       </c>
       <c r="N19" s="12" t="n">
-        <v>198.27</v>
+        <v>198.38</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>0.02919406017860693</v>
+        <v>0.02919087222408607</v>
       </c>
     </row>
     <row r="20">
@@ -8844,7 +8844,7 @@
         <v>46272</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C20" s="31" t="inlineStr">
         <is>
@@ -8852,40 +8852,40 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>47.8618</v>
+        <v>47.9414</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>48.8184</v>
+        <v>48.8254</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0.9566</v>
+        <v>0.884</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>0.0199867117408873</v>
+        <v>0.0184391778296003</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>55.6416</v>
+        <v>55.734</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>56.7777</v>
+        <v>56.7908</v>
       </c>
       <c r="J20" s="10" t="n">
-        <v>1.1361</v>
+        <v>1.0568</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>0.02041817632850242</v>
+        <v>0.01896149567588904</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>6735.46</v>
+        <v>6737.95</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>7181.18</v>
+        <v>7183.98</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>445.72</v>
+        <v>446.03</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>0.06617513874330781</v>
+        <v>0.06619669187215696</v>
       </c>
     </row>
     <row r="21">
@@ -8893,7 +8893,7 @@
         <v>46272</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
@@ -8904,37 +8904,37 @@
         <v>47.8873</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>48.8907</v>
+        <v>48.8906</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.0034</v>
+        <v>1.0033</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.02095336341785818</v>
+        <v>0.02095127518151994</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>55.7447</v>
+        <v>55.7467</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>56.7511</v>
+        <v>56.7565</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>1.0064</v>
+        <v>1.0098</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>0.01805373425635083</v>
+        <v>0.01811407670767956</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>6704.37</v>
+        <v>6704.68</v>
       </c>
       <c r="M21" s="12" t="n">
-        <v>6956.76</v>
+        <v>6956.73</v>
       </c>
       <c r="N21" s="12" t="n">
-        <v>252.39</v>
+        <v>252.05</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>0.03764559533557963</v>
+        <v>0.03759314389351916</v>
       </c>
     </row>
     <row r="22">
@@ -8942,7 +8942,7 @@
         <v>46272</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -8950,40 +8950,40 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>47.8124</v>
+        <v>47.8123</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>48.9701</v>
+        <v>48.972</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.1577</v>
+        <v>1.1597</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>0.02421338397570505</v>
+        <v>0.02425526485862425</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>55.5724</v>
+        <v>55.5723</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>56.9228</v>
+        <v>56.9301</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>1.3504</v>
+        <v>1.3578</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>0.02429983229084941</v>
+        <v>0.02443303588298487</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>6724.84</v>
+        <v>6725.79</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>6909.87</v>
+        <v>6910.79</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>185.03</v>
+        <v>185</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>0.02751440926475574</v>
+        <v>0.02750606248485308</v>
       </c>
     </row>
     <row r="23">
@@ -8991,7 +8991,7 @@
         <v>46272</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C23" s="34" t="inlineStr">
         <is>
@@ -9002,13 +9002,13 @@
         <v>48.3</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>48.32</v>
+        <v>48.31</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>0.0004140786749482402</v>
+        <v>0.0002070393374741201</v>
       </c>
       <c r="H23" s="10" t="n">
         <v>56</v>
@@ -9023,16 +9023,16 @@
         <v>0.0008928571428571428</v>
       </c>
       <c r="L23" s="12" t="n">
-        <v>6783.84</v>
+        <v>6788.7</v>
       </c>
       <c r="M23" s="12" t="n">
-        <v>6791.51</v>
+        <v>6794.96</v>
       </c>
       <c r="N23" s="12" t="n">
-        <v>7.67</v>
+        <v>6.26</v>
       </c>
       <c r="O23" s="13" t="n">
-        <v>0.001130628080850964</v>
+        <v>0.0009221205827330711</v>
       </c>
     </row>
     <row r="24">
@@ -9040,7 +9040,7 @@
         <v>46272</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
@@ -9048,40 +9048,40 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>47.7142</v>
+        <v>47.715</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>48.7524</v>
+        <v>48.7532</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>1.0382</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.02175872172225459</v>
+        <v>0.02175835691082469</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>55.4648</v>
+        <v>55.4686</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>56.6732</v>
+        <v>56.6772</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>1.2084</v>
+        <v>1.2086</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>0.02178679090161688</v>
+        <v>0.02178890399252911</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>6683.47</v>
+        <v>6684.26</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>6860.86</v>
+        <v>6861.49</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>177.39</v>
+        <v>177.23</v>
       </c>
       <c r="O24" s="13" t="n">
-        <v>0.02654160189243013</v>
+        <v>0.02651452816018527</v>
       </c>
     </row>
     <row r="25">
@@ -9089,7 +9089,7 @@
         <v>46272</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
@@ -9130,7 +9130,7 @@
         <v>46272</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
@@ -9141,37 +9141,37 @@
         <v>48.3628</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>48.4163</v>
+        <v>48.4161</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>0.0535</v>
+        <v>0.0533</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>0.001106222137676065</v>
+        <v>0.001102086727815594</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>56.201</v>
+        <v>56.2041</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>56.2826</v>
+        <v>56.2846</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>0.08160000000000001</v>
+        <v>0.0805</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>0.001451931460294301</v>
+        <v>0.001432279851469911</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>6779.62</v>
+        <v>6784.36</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>6810.25</v>
+        <v>6813.42</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>30.63</v>
+        <v>29.06</v>
       </c>
       <c r="O26" s="13" t="n">
-        <v>0.004517952333611619</v>
+        <v>0.004283381188498252</v>
       </c>
     </row>
     <row r="27">
@@ -9179,7 +9179,7 @@
         <v>46272</v>
       </c>
       <c r="B27" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C27" s="38" t="inlineStr">
         <is>
@@ -9190,37 +9190,37 @@
         <v>48.317</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>48.42</v>
+        <v>48.418</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.103</v>
+        <v>0.101</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>0.002131754868886727</v>
+        <v>0.002090361570461742</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>56.004</v>
+        <v>55.995</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>56.183</v>
+        <v>56.173</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>0.179</v>
+        <v>0.178</v>
       </c>
       <c r="K27" s="11" t="n">
-        <v>0.003196200271409185</v>
+        <v>0.003178855254933477</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>6772</v>
+        <v>6764</v>
       </c>
       <c r="M27" s="12" t="n">
-        <v>6808</v>
+        <v>6812</v>
       </c>
       <c r="N27" s="12" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>0.005316007088009451</v>
+        <v>0.007096392667060911</v>
       </c>
     </row>
     <row r="28">
@@ -9228,7 +9228,7 @@
         <v>46272</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -9236,16 +9236,16 @@
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>47.8725</v>
+        <v>47.873</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>48.8725</v>
+        <v>48.873</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>0.02088881925949136</v>
+        <v>0.02088860109038498</v>
       </c>
       <c r="H28" s="10" t="n">
         <v>55.681</v>
@@ -9260,16 +9260,16 @@
         <v>0.01957579784845818</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>6774.47</v>
+        <v>6781.07</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>6874.47</v>
+        <v>6881.07</v>
       </c>
       <c r="N28" s="12" t="n">
         <v>100</v>
       </c>
       <c r="O28" s="13" t="n">
-        <v>0.01476130236018463</v>
+        <v>0.01474693521818828</v>
       </c>
     </row>
     <row r="29">
@@ -9277,7 +9277,7 @@
         <v>46272</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
@@ -9293,16 +9293,16 @@
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="12" t="n">
-        <v>6789.9</v>
+        <v>6795.14</v>
       </c>
       <c r="M29" s="12" t="n">
-        <v>6974.19</v>
+        <v>6979.54</v>
       </c>
       <c r="N29" s="12" t="n">
-        <v>184.29</v>
+        <v>184.4</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>0.02714178412053197</v>
+        <v>0.0271370420624152</v>
       </c>
     </row>
     <row r="30">
@@ -9310,7 +9310,7 @@
         <v>46272</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C30" s="41" t="inlineStr">
         <is>
@@ -9333,25 +9333,25 @@
         <v>55.4727</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>57.1322</v>
+        <v>57.1371</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>1.6595</v>
+        <v>1.6644</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>0.029915616149926</v>
+        <v>0.03000394788787998</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>6702.92</v>
+        <v>6706.92</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>6904.1</v>
+        <v>6908.22</v>
       </c>
       <c r="N30" s="12" t="n">
-        <v>201.18</v>
+        <v>201.3</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>0.03001378503696896</v>
+        <v>0.03001377681558748</v>
       </c>
     </row>
     <row r="31">
@@ -9359,7 +9359,7 @@
         <v>46272</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -9367,40 +9367,40 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>48.2974</v>
+        <v>48.3122</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>48.5153</v>
+        <v>48.5302</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>0.2179</v>
+        <v>0.218</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>0.004511630025632849</v>
+        <v>0.00451231779964481</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>56.0589</v>
+        <v>56.0766</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>56.3966</v>
+        <v>56.4144</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>0.3377</v>
+        <v>0.3378</v>
       </c>
       <c r="K31" s="11" t="n">
-        <v>0.006024021163454866</v>
+        <v>0.006023903018371299</v>
       </c>
       <c r="L31" s="12" t="n">
-        <v>6769.12</v>
+        <v>6773.2</v>
       </c>
       <c r="M31" s="12" t="n">
-        <v>6871.17</v>
+        <v>6875.31</v>
       </c>
       <c r="N31" s="12" t="n">
-        <v>102.05</v>
+        <v>102.11</v>
       </c>
       <c r="O31" s="13" t="n">
-        <v>0.01507581487697071</v>
+        <v>0.01507559203921337</v>
       </c>
     </row>
     <row r="32">
@@ -9408,7 +9408,7 @@
         <v>46272</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C32" s="43" t="inlineStr">
         <is>
@@ -9416,40 +9416,40 @@
         </is>
       </c>
       <c r="D32" s="8" t="n">
-        <v>47.9875</v>
+        <v>47.9876</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>48.7898</v>
+        <v>48.79</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.8023</v>
+        <v>0.8024</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>0.01671893722323522</v>
+        <v>0.01672098625478249</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>55.8136</v>
+        <v>55.8099</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>56.6653</v>
+        <v>56.6616</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>0.8517</v>
       </c>
       <c r="K32" s="11" t="n">
-        <v>0.01525972164490375</v>
+        <v>0.01526073331075669</v>
       </c>
       <c r="L32" s="12" t="n">
-        <v>6733.81</v>
+        <v>6734.61</v>
       </c>
       <c r="M32" s="12" t="n">
-        <v>6930.31</v>
+        <v>6930.98</v>
       </c>
       <c r="N32" s="12" t="n">
-        <v>196.5</v>
+        <v>196.37</v>
       </c>
       <c r="O32" s="13" t="n">
-        <v>0.02918110252591029</v>
+        <v>0.02915833285075157</v>
       </c>
     </row>
     <row r="33">
@@ -9457,7 +9457,7 @@
         <v>46272</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
@@ -9465,40 +9465,40 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>48.2868</v>
+        <v>48.2869</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>48.4905</v>
+        <v>48.4906</v>
       </c>
       <c r="F33" s="8" t="n">
         <v>0.2037</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>0.004218544198414474</v>
+        <v>0.00421853546199901</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>56.1198</v>
+        <v>56.1223</v>
       </c>
       <c r="I33" s="10" t="n">
-        <v>56.3459</v>
+        <v>56.3484</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>0.2261</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>0.004028881072277521</v>
+        <v>0.004028701603462439</v>
       </c>
       <c r="L33" s="12" t="n">
-        <v>6769.39</v>
+        <v>6773.71</v>
       </c>
       <c r="M33" s="12" t="n">
-        <v>6823.76</v>
+        <v>6828.12</v>
       </c>
       <c r="N33" s="12" t="n">
-        <v>54.37</v>
+        <v>54.41</v>
       </c>
       <c r="O33" s="13" t="n">
-        <v>0.0080317428896843</v>
+        <v>0.00803252575029046</v>
       </c>
     </row>
     <row r="34">
@@ -9506,7 +9506,7 @@
         <v>46272</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C34" s="45" t="inlineStr">
         <is>
@@ -9517,37 +9517,37 @@
         <v>48.0254</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>48.991</v>
+        <v>48.9909</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>0.9656</v>
+        <v>0.9655</v>
       </c>
       <c r="G34" s="9" t="n">
-        <v>0.02010602722725891</v>
+        <v>0.02010394499577307</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>55.8036</v>
+        <v>55.8106</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>56.9201</v>
+        <v>56.927</v>
       </c>
       <c r="J34" s="10" t="n">
-        <v>1.1165</v>
+        <v>1.1164</v>
       </c>
       <c r="K34" s="11" t="n">
-        <v>0.02000766975607308</v>
+        <v>0.02000336853572619</v>
       </c>
       <c r="L34" s="12" t="n">
-        <v>6729.92</v>
+        <v>6739.74</v>
       </c>
       <c r="M34" s="12" t="n">
-        <v>6874.52</v>
+        <v>6884.34</v>
       </c>
       <c r="N34" s="12" t="n">
         <v>144.6</v>
       </c>
       <c r="O34" s="13" t="n">
-        <v>0.02148613950834482</v>
+        <v>0.02145483356924748</v>
       </c>
     </row>
     <row r="35">
@@ -9555,7 +9555,7 @@
         <v>46272</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C35" s="46" t="inlineStr">
         <is>
@@ -9563,28 +9563,28 @@
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>48.289</v>
+        <v>48.291</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>48.34</v>
+        <v>48.347</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.051</v>
+        <v>0.056</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>0.001056141150158421</v>
+        <v>0.00115963637116647</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>55.986</v>
+        <v>55.989</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>56.123</v>
+        <v>56.131</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>0.137</v>
+        <v>0.142</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>0.002447040331511449</v>
+        <v>0.002536212470306667</v>
       </c>
       <c r="L35" s="12" t="n"/>
       <c r="M35" s="12" t="n"/>
@@ -9596,7 +9596,7 @@
         <v>46272</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C36" s="47" t="inlineStr">
         <is>
@@ -9628,16 +9628,16 @@
         <v>0.02051835853131749</v>
       </c>
       <c r="L36" s="12" t="n">
-        <v>6710.49</v>
+        <v>6711.62</v>
       </c>
       <c r="M36" s="12" t="n">
-        <v>6913.64</v>
+        <v>6915.1</v>
       </c>
       <c r="N36" s="12" t="n">
-        <v>203.15</v>
+        <v>203.48</v>
       </c>
       <c r="O36" s="13" t="n">
-        <v>0.03027349716637682</v>
+        <v>0.03031756863469624</v>
       </c>
     </row>
     <row r="37">
@@ -9645,7 +9645,7 @@
         <v>46272</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C37" s="48" t="inlineStr">
         <is>
@@ -9665,28 +9665,28 @@
         <v>0.02023091899095272</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>55.816</v>
+        <v>55.8096</v>
       </c>
       <c r="I37" s="10" t="n">
-        <v>56.9451</v>
+        <v>56.9386</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1.1291</v>
+        <v>1.129</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>0.02022896660455783</v>
+        <v>0.02022949456724291</v>
       </c>
       <c r="L37" s="12" t="n">
-        <v>6766.18</v>
+        <v>6772.85</v>
       </c>
       <c r="M37" s="12" t="n">
-        <v>6902.8</v>
+        <v>6909.61</v>
       </c>
       <c r="N37" s="12" t="n">
-        <v>136.62</v>
+        <v>136.76</v>
       </c>
       <c r="O37" s="13" t="n">
-        <v>0.02019159998699414</v>
+        <v>0.02019238577555977</v>
       </c>
     </row>
     <row r="38">
@@ -9694,7 +9694,7 @@
         <v>46272</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
@@ -9702,40 +9702,40 @@
         </is>
       </c>
       <c r="D38" s="8" t="n">
-        <v>48.072</v>
+        <v>48.0735</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>48.7261</v>
+        <v>48.7276</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>0.6541</v>
       </c>
       <c r="G38" s="9" t="n">
-        <v>0.01360667332334831</v>
+        <v>0.01360624876491206</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>55.8151</v>
+        <v>55.8193</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>56.631</v>
+        <v>56.6353</v>
       </c>
       <c r="J38" s="10" t="n">
-        <v>0.8159</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="K38" s="11" t="n">
-        <v>0.01461790805713866</v>
+        <v>0.01461859965997424</v>
       </c>
       <c r="L38" s="12" t="n">
-        <v>6739.07</v>
+        <v>6742.04</v>
       </c>
       <c r="M38" s="12" t="n">
-        <v>6875.15</v>
+        <v>6878.17</v>
       </c>
       <c r="N38" s="12" t="n">
-        <v>136.08</v>
+        <v>136.13</v>
       </c>
       <c r="O38" s="13" t="n">
-        <v>0.02019269721192983</v>
+        <v>0.02019121808829375</v>
       </c>
     </row>
     <row r="39">
@@ -9743,7 +9743,7 @@
         <v>46272</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="C39" s="50" t="inlineStr">
         <is>
@@ -9751,40 +9751,40 @@
         </is>
       </c>
       <c r="D39" s="8" t="n">
-        <v>47.9028</v>
+        <v>47.9025</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>48.9025</v>
+        <v>48.9029</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.9997</v>
+        <v>1.0004</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>0.02086934375443607</v>
+        <v>0.02088408746933876</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>55.6435</v>
+        <v>55.6441</v>
       </c>
       <c r="I39" s="10" t="n">
-        <v>56.8608</v>
+        <v>56.8623</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1.2173</v>
+        <v>1.2182</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>0.02187676907455498</v>
+        <v>0.0218927074029412</v>
       </c>
       <c r="L39" s="12" t="n">
-        <v>6759.46</v>
+        <v>6760.38</v>
       </c>
       <c r="M39" s="12" t="n">
-        <v>6974.17</v>
+        <v>6975.08</v>
       </c>
       <c r="N39" s="12" t="n">
-        <v>214.71</v>
+        <v>214.7</v>
       </c>
       <c r="O39" s="13" t="n">
-        <v>0.0317643717101662</v>
+        <v>0.03175856978453874</v>
       </c>
     </row>
   </sheetData>
@@ -70626,7 +70626,7 @@
       </c>
       <c r="B5" s="62" t="n"/>
       <c r="C5" s="64" t="n">
-        <v>0.6182407407407408</v>
+        <v>0.6433101851851852</v>
       </c>
       <c r="D5" s="62" t="n"/>
       <c r="F5" s="62" t="inlineStr">
@@ -70710,7 +70710,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="70" t="n">
-        <v>0.02022896660455783</v>
+        <v>0.02022949456724291</v>
       </c>
       <c r="O6" s="71" t="inlineStr">
         <is>
@@ -70718,10 +70718,10 @@
         </is>
       </c>
       <c r="P6" s="72" t="n">
-        <v>55.816</v>
+        <v>55.8096</v>
       </c>
       <c r="Q6" s="72" t="n">
-        <v>56.9451</v>
+        <v>56.9386</v>
       </c>
     </row>
     <row r="7">
@@ -70763,7 +70763,7 @@
         <v>5</v>
       </c>
       <c r="N7" s="70" t="n">
-        <v>0.02019159998699414</v>
+        <v>0.02019238577555977</v>
       </c>
       <c r="O7" s="71" t="inlineStr">
         <is>
@@ -70771,10 +70771,10 @@
         </is>
       </c>
       <c r="P7" s="72" t="n">
-        <v>6766.18</v>
+        <v>6772.85</v>
       </c>
       <c r="Q7" s="72" t="n">
-        <v>6902.8</v>
+        <v>6909.61</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Günlük kur verisi: 07.09.2026 15:32
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -7978,7 +7978,7 @@
         <v>46272</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
@@ -7998,28 +7998,28 @@
         <v>0.02833931607783866</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>55.3683</v>
+        <v>55.3831</v>
       </c>
       <c r="I2" s="10" t="n">
-        <v>56.9423</v>
+        <v>56.9575</v>
       </c>
       <c r="J2" s="10" t="n">
-        <v>1.574</v>
+        <v>1.5744</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>0.02842781880606773</v>
+        <v>0.0284274444731335</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>6660.62</v>
+        <v>6662.14</v>
       </c>
       <c r="M2" s="12" t="n">
-        <v>6900.64</v>
+        <v>6902.2</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>240.02</v>
+        <v>240.06</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>0.03603568436571971</v>
+        <v>0.03603346672390553</v>
       </c>
     </row>
     <row r="3">
@@ -8027,7 +8027,7 @@
         <v>46272</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
@@ -8047,28 +8047,28 @@
         <v>0.01625965482064414</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>55.833</v>
+        <v>55.843</v>
       </c>
       <c r="I3" s="10" t="n">
-        <v>56.752</v>
+        <v>56.761</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.919</v>
+        <v>0.918</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>0.01645979975999857</v>
+        <v>0.0164389448990921</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>6736.66</v>
+        <v>6738.65</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>6875.37</v>
+        <v>6877.09</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>138.71</v>
+        <v>138.44</v>
       </c>
       <c r="O3" s="13" t="n">
-        <v>0.02059032220714716</v>
+        <v>0.0205441742782308</v>
       </c>
     </row>
     <row r="4">
@@ -8076,7 +8076,7 @@
         <v>46272</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -8084,40 +8084,40 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>48.221</v>
+        <v>48.217</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>48.506</v>
+        <v>48.509</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.285</v>
+        <v>0.292</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>0.00591028804877543</v>
+        <v>0.006055955368438517</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>55.886</v>
+        <v>55.881</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>56.39</v>
+        <v>56.396</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.504</v>
+        <v>0.515</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>0.009018358801846616</v>
+        <v>0.009216012598199746</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>6797.96</v>
+        <v>6800.12</v>
       </c>
       <c r="M4" s="12" t="n">
-        <v>6865.18</v>
+        <v>6868.53</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>67.22</v>
+        <v>68.41</v>
       </c>
       <c r="O4" s="13" t="n">
-        <v>0.009888260595825807</v>
+        <v>0.01006011658617789</v>
       </c>
     </row>
     <row r="5">
@@ -8125,7 +8125,7 @@
         <v>46272</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -8136,37 +8136,37 @@
         <v>48.24</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>48.43</v>
+        <v>48.431</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.19</v>
+        <v>0.191</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>0.003938640132669983</v>
+        <v>0.003959369817578773</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>55.927</v>
+        <v>55.936</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>56.299</v>
+        <v>56.309</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.372</v>
+        <v>0.373</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>0.006651527884563806</v>
+        <v>0.0066683352402746</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>6729.84</v>
+        <v>6733.16</v>
       </c>
       <c r="M5" s="12" t="n">
         <v>6885</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>155.16</v>
+        <v>151.84</v>
       </c>
       <c r="O5" s="13" t="n">
-        <v>0.023055525837167</v>
+        <v>0.02255107557224245</v>
       </c>
     </row>
     <row r="6">
@@ -8174,7 +8174,7 @@
         <v>46272</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
@@ -8182,40 +8182,40 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>47.589</v>
+        <v>47.5894</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>48.8657</v>
+        <v>48.8659</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>1.2767</v>
+        <v>1.2765</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.02682762823341529</v>
+        <v>0.02682320012439745</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>55.4271</v>
+        <v>55.4354</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>56.7918</v>
+        <v>56.8006</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>1.3647</v>
+        <v>1.3652</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0.02462152990143811</v>
+        <v>0.02462686297925153</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>6723.12</v>
+        <v>6725.62</v>
       </c>
       <c r="M6" s="12" t="n">
-        <v>6874.44</v>
+        <v>6876.92</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>151.32</v>
+        <v>151.3</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>0.02250740727519366</v>
+        <v>0.02249606727706888</v>
       </c>
     </row>
     <row r="7">
@@ -8223,7 +8223,7 @@
         <v>46272</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
@@ -8234,37 +8234,37 @@
         <v>47.436</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>49.363</v>
+        <v>49.364</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>1.927</v>
+        <v>1.928</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>0.04062315540939371</v>
+        <v>0.04064423644489417</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>55.139</v>
+        <v>55.149</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>57.39</v>
+        <v>57.395</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>2.251</v>
+        <v>2.246</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>0.04082409909501442</v>
+        <v>0.04072603311030118</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>6720.22</v>
+        <v>6722.13</v>
       </c>
       <c r="M7" s="12" t="n">
-        <v>6915.18</v>
+        <v>6916.8</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>194.96</v>
+        <v>194.67</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>0.02901095499849707</v>
+        <v>0.02895957085031084</v>
       </c>
     </row>
     <row r="8">
@@ -8272,7 +8272,7 @@
         <v>46272</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
@@ -8280,40 +8280,40 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>47.7166</v>
+        <v>47.7169</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>49.0647</v>
+        <v>49.065</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>1.3481</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>0.02825222249699266</v>
+        <v>0.02825204487299049</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>55.4701</v>
+        <v>55.48</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>57.0372</v>
+        <v>57.0474</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>1.5671</v>
+        <v>1.5674</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>0.02825125608210549</v>
+        <v>0.02825162220620043</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>6739.25</v>
+        <v>6740.86</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>6930.74</v>
+        <v>6932.3</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>191.49</v>
+        <v>191.44</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>0.02841414103943317</v>
+        <v>0.02839993710001394</v>
       </c>
     </row>
     <row r="9">
@@ -8321,7 +8321,7 @@
         <v>46272</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -8329,40 +8329,40 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>48.3605</v>
+        <v>48.361</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>48.4173</v>
+        <v>48.4178</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>0.0568</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.001174512256903878</v>
+        <v>0.001174500113728004</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>56.2081</v>
+        <v>56.2134</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>56.2912</v>
+        <v>56.2962</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.08309999999999999</v>
+        <v>0.0828</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>0.001478434602841939</v>
+        <v>0.001472958404935478</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6789.5</v>
+        <v>6792</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>6818.36</v>
+        <v>6820.85</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>28.86</v>
+        <v>28.85</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>0.004250681198910082</v>
+        <v>0.004247644287396938</v>
       </c>
     </row>
     <row r="10">
@@ -8370,7 +8370,7 @@
         <v>46272</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -8378,40 +8378,40 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>48.3736</v>
+        <v>48.3739</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>48.4121</v>
+        <v>48.4122</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.0385</v>
+        <v>0.0383</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.0007958886665453883</v>
+        <v>0.0007917492697508367</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>56.1847</v>
+        <v>56.1949</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>56.2947</v>
+        <v>56.3053</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.11</v>
+        <v>0.1104</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>0.001957828376764493</v>
+        <v>0.001964591092786</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>6785.65</v>
+        <v>6788.33</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>6818</v>
+        <v>6820.61</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>32.35</v>
+        <v>32.28</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>0.004767413586023447</v>
+        <v>0.004755219619552969</v>
       </c>
     </row>
     <row r="11">
@@ -8419,7 +8419,7 @@
         <v>46272</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
@@ -8439,28 +8439,28 @@
         <v>0.02580731068431817</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>55.7531</v>
+        <v>55.7729</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>57.0317</v>
+        <v>57.0519</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>1.2786</v>
+        <v>1.279</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>0.0229332539356556</v>
+        <v>0.02293228431729388</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6735.41</v>
+        <v>6738.01</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>6845.39</v>
+        <v>6848.13</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>109.98</v>
+        <v>110.12</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>0.0163286273589878</v>
+        <v>0.01634310426965825</v>
       </c>
     </row>
     <row r="12">
@@ -8468,7 +8468,7 @@
         <v>46272</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
@@ -8476,40 +8476,40 @@
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>47.983</v>
+        <v>47.9835</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>48.833</v>
+        <v>48.8335</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>0.85</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>0.01771460725673676</v>
+        <v>0.01771442266612482</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>55.6918</v>
+        <v>55.7019</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>56.8584</v>
+        <v>56.8688</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>1.1666</v>
+        <v>1.1669</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>0.02094742852628214</v>
+        <v>0.02094901610178468</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>6733.89</v>
+        <v>6736</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>6890.21</v>
+        <v>6892.68</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>156.32</v>
+        <v>156.68</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>0.02321392241334503</v>
+        <v>0.02326009501187648</v>
       </c>
     </row>
     <row r="13">
@@ -8517,7 +8517,7 @@
         <v>46272</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
@@ -8525,40 +8525,40 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>48.1339</v>
+        <v>48.1346</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>48.7411</v>
+        <v>48.7414</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.6072</v>
+        <v>0.6068</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.01261480993644812</v>
+        <v>0.01260631645427613</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>55.9701</v>
+        <v>55.9748</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>56.6307</v>
+        <v>56.635</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>0.6606</v>
+        <v>0.6602</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>0.01180273038640274</v>
+        <v>0.01179459328126228</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6805.56</v>
+        <v>6808.07</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>6859.83</v>
+        <v>6862.28</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>54.27</v>
+        <v>54.21</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>0.007974362139192073</v>
+        <v>0.007962609080106403</v>
       </c>
     </row>
     <row r="14">
@@ -8566,7 +8566,7 @@
         <v>46272</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
@@ -8574,40 +8574,40 @@
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>47.59</v>
+        <v>47.591</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>48.94</v>
+        <v>48.941</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>1.35</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>0.02836730405547384</v>
+        <v>0.0283667079910067</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>55.324</v>
+        <v>55.329</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>56.893</v>
+        <v>56.899</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>1.569</v>
+        <v>1.57</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>0.02836020533583978</v>
+        <v>0.02837571617054348</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>6701.54</v>
+        <v>6702.59</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>6948.99</v>
+        <v>6950.07</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>247.45</v>
+        <v>247.48</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>0.03692434873178404</v>
+        <v>0.03692304019789365</v>
       </c>
     </row>
     <row r="15">
@@ -8615,7 +8615,7 @@
         <v>46272</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
@@ -8623,40 +8623,40 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>48.134</v>
+        <v>48.1346</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>48.7411</v>
+        <v>48.7416</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.6071</v>
+        <v>0.607</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>0.01261270619520505</v>
+        <v>0.01261047146958737</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>55.971</v>
+        <v>55.9794</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>56.6317</v>
+        <v>56.6389</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>0.6607</v>
+        <v>0.6595</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>0.0118043272408926</v>
+        <v>0.01178111948323848</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>6808.24</v>
+        <v>6810.44</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>6862.45</v>
+        <v>6864.65</v>
       </c>
       <c r="N15" s="12" t="n">
         <v>54.21</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>0.007962410255807668</v>
+        <v>0.007959838130869666</v>
       </c>
     </row>
     <row r="16">
@@ -8664,7 +8664,7 @@
         <v>46272</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
@@ -8684,28 +8684,28 @@
         <v>0.02041317992721334</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>55.8014</v>
+        <v>55.8116</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>56.9405</v>
+        <v>56.951</v>
       </c>
       <c r="J16" s="10" t="n">
-        <v>1.1391</v>
+        <v>1.1394</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>0.02041346632880179</v>
+        <v>0.02041511083717364</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>6736.14</v>
+        <v>6736.31</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>6942.6</v>
+        <v>6943.23</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>206.46</v>
+        <v>206.92</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>0.03064960051305347</v>
+        <v>0.03071711367202519</v>
       </c>
     </row>
     <row r="17">
@@ -8713,7 +8713,7 @@
         <v>46272</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
@@ -8721,40 +8721,40 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>48.2839</v>
+        <v>48.2844</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>48.3438</v>
+        <v>48.3444</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.0599</v>
+        <v>0.06</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.001240579157855931</v>
+        <v>0.001242637373561647</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>55.975</v>
+        <v>55.982</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>56.129</v>
+        <v>56.138</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>0.154</v>
+        <v>0.156</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>0.002751228226887003</v>
+        <v>0.002786609981779858</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>6750.36</v>
+        <v>6753.6</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>6822.33</v>
+        <v>6825.59</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>71.97</v>
+        <v>71.98999999999999</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>0.01066165360069685</v>
+        <v>0.01065950011845534</v>
       </c>
     </row>
     <row r="18">
@@ -8762,7 +8762,7 @@
         <v>46272</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
@@ -8770,40 +8770,40 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>48.3539</v>
+        <v>48.3545</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>48.5005</v>
+        <v>48.501</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>0.1466</v>
+        <v>0.1465</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.003031813359418785</v>
+        <v>0.003029707679740251</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>56.1979</v>
+        <v>56.2056</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>56.3701</v>
+        <v>56.3778</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>0.1722</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>0.003064171437010991</v>
+        <v>0.003063751654639396</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>6795.78</v>
+        <v>6799.23</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>6843.86</v>
+        <v>6847.17</v>
       </c>
       <c r="N18" s="12" t="n">
-        <v>48.08</v>
+        <v>47.94</v>
       </c>
       <c r="O18" s="13" t="n">
-        <v>0.007074978883954454</v>
+        <v>0.007050798399230502</v>
       </c>
     </row>
     <row r="19">
@@ -8811,7 +8811,7 @@
         <v>46272</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
@@ -8827,16 +8827,16 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="12" t="n">
-        <v>6795.96</v>
+        <v>6798.67</v>
       </c>
       <c r="M19" s="12" t="n">
-        <v>6994.34</v>
+        <v>6997.09</v>
       </c>
       <c r="N19" s="12" t="n">
-        <v>198.38</v>
+        <v>198.42</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>0.02919087222408607</v>
+        <v>0.02918512003082956</v>
       </c>
     </row>
     <row r="20">
@@ -8844,7 +8844,7 @@
         <v>46272</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C20" s="31" t="inlineStr">
         <is>
@@ -8852,40 +8852,40 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>47.9414</v>
+        <v>47.8878</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>48.8254</v>
+        <v>48.8404</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0.884</v>
+        <v>0.9526</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>0.0184391778296003</v>
+        <v>0.01989233165858528</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>55.734</v>
+        <v>55.745</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>56.7908</v>
+        <v>56.7951</v>
       </c>
       <c r="J20" s="10" t="n">
-        <v>1.0568</v>
+        <v>1.0501</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>0.01896149567588904</v>
+        <v>0.01883756390707687</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>6737.95</v>
+        <v>6741.38</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>7183.98</v>
+        <v>7187.6</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>446.03</v>
+        <v>446.22</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>0.06619669187215696</v>
+        <v>0.06619119527455802</v>
       </c>
     </row>
     <row r="21">
@@ -8893,7 +8893,7 @@
         <v>46272</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
@@ -8901,40 +8901,40 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>47.8873</v>
+        <v>47.8878</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>48.8906</v>
+        <v>48.8909</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.0033</v>
+        <v>1.0031</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.02095127518151994</v>
+        <v>0.02094687999866354</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>55.7467</v>
+        <v>55.755</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>56.7565</v>
+        <v>56.7616</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>1.0098</v>
+        <v>1.0066</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>0.01811407670767956</v>
+        <v>0.01805398618957941</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>6704.68</v>
+        <v>6709.4</v>
       </c>
       <c r="M21" s="12" t="n">
-        <v>6956.73</v>
+        <v>6961.22</v>
       </c>
       <c r="N21" s="12" t="n">
-        <v>252.05</v>
+        <v>251.82</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>0.03759314389351916</v>
+        <v>0.03753241720571139</v>
       </c>
     </row>
     <row r="22">
@@ -8942,7 +8942,7 @@
         <v>46272</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -8950,40 +8950,40 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>47.8123</v>
+        <v>47.8126</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>48.972</v>
+        <v>48.9724</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.1597</v>
+        <v>1.1598</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>0.02425526485862425</v>
+        <v>0.02425720416793899</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>55.5723</v>
+        <v>55.5822</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>56.9301</v>
+        <v>56.9405</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>1.3578</v>
+        <v>1.3583</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>0.02443303588298487</v>
+        <v>0.02443767968882124</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>6725.79</v>
+        <v>6730.36</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>6910.79</v>
+        <v>6915.65</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>185</v>
+        <v>185.29</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>0.02750606248485308</v>
+        <v>0.02753047385281025</v>
       </c>
     </row>
     <row r="23">
@@ -8991,7 +8991,7 @@
         <v>46272</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C23" s="34" t="inlineStr">
         <is>
@@ -9023,16 +9023,16 @@
         <v>0.0008928571428571428</v>
       </c>
       <c r="L23" s="12" t="n">
-        <v>6788.7</v>
+        <v>6791.13</v>
       </c>
       <c r="M23" s="12" t="n">
-        <v>6794.96</v>
+        <v>6797.39</v>
       </c>
       <c r="N23" s="12" t="n">
         <v>6.26</v>
       </c>
       <c r="O23" s="13" t="n">
-        <v>0.0009221205827330711</v>
+        <v>0.0009217906298362717</v>
       </c>
     </row>
     <row r="24">
@@ -9040,7 +9040,7 @@
         <v>46272</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
@@ -9048,40 +9048,40 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>47.715</v>
+        <v>47.7155</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>48.7532</v>
+        <v>48.7538</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>1.0382</v>
+        <v>1.0383</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.02175835691082469</v>
+        <v>0.02176022466494116</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>55.4686</v>
+        <v>55.4735</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>56.6772</v>
+        <v>56.6866</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>1.2086</v>
+        <v>1.2131</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>0.02178890399252911</v>
+        <v>0.02186809918249254</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>6684.26</v>
+        <v>6687.59</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>6861.49</v>
+        <v>6865</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>177.23</v>
+        <v>177.41</v>
       </c>
       <c r="O24" s="13" t="n">
-        <v>0.02651452816018527</v>
+        <v>0.02652824111525976</v>
       </c>
     </row>
     <row r="25">
@@ -9089,7 +9089,7 @@
         <v>46272</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
@@ -9097,28 +9097,28 @@
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>48.2326</v>
+        <v>48.3465</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>48.3195</v>
+        <v>48.4336</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>0.08690000000000001</v>
+        <v>0.0871</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>0.001801685996608103</v>
+        <v>0.001801578190768722</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>56.0571</v>
+        <v>56.1851</v>
       </c>
       <c r="I25" s="10" t="n">
-        <v>56.1581</v>
+        <v>56.2864</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>0.101</v>
+        <v>0.1013</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>0.001801734303058845</v>
+        <v>0.001802969114587319</v>
       </c>
       <c r="L25" s="12" t="n"/>
       <c r="M25" s="12" t="n"/>
@@ -9130,7 +9130,7 @@
         <v>46272</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
@@ -9138,40 +9138,40 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>48.3628</v>
+        <v>48.3633</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>48.4161</v>
+        <v>48.4167</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>0.0533</v>
+        <v>0.0534</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>0.001102086727815594</v>
+        <v>0.001104143017536024</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>56.2041</v>
+        <v>56.2132</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>56.2846</v>
+        <v>56.2939</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>0.0805</v>
+        <v>0.08069999999999999</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>0.001432279851469911</v>
+        <v>0.001435605871930436</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>6784.36</v>
+        <v>6787.52</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>6813.42</v>
+        <v>6816.18</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>29.06</v>
+        <v>28.66</v>
       </c>
       <c r="O26" s="13" t="n">
-        <v>0.004283381188498252</v>
+        <v>0.004222455329781717</v>
       </c>
     </row>
     <row r="27">
@@ -9179,7 +9179,7 @@
         <v>46272</v>
       </c>
       <c r="B27" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C27" s="38" t="inlineStr">
         <is>
@@ -9190,37 +9190,37 @@
         <v>48.317</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>48.418</v>
+        <v>48.419</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.101</v>
+        <v>0.102</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>0.002090361570461742</v>
+        <v>0.002111058219674235</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>55.995</v>
+        <v>56.015</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>56.173</v>
+        <v>56.194</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>0.178</v>
+        <v>0.179</v>
       </c>
       <c r="K27" s="11" t="n">
-        <v>0.003178855254933477</v>
+        <v>0.003195572614478265</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>6764</v>
+        <v>6771</v>
       </c>
       <c r="M27" s="12" t="n">
-        <v>6812</v>
+        <v>6817</v>
       </c>
       <c r="N27" s="12" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>0.007096392667060911</v>
+        <v>0.006793678924826466</v>
       </c>
     </row>
     <row r="28">
@@ -9228,7 +9228,7 @@
         <v>46272</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -9236,40 +9236,40 @@
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>47.873</v>
+        <v>47.8735</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>48.873</v>
+        <v>48.8735</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>0.02088860109038498</v>
+        <v>0.02088838292583579</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>55.681</v>
+        <v>55.694</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>56.771</v>
+        <v>56.784</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>1.09</v>
       </c>
       <c r="K28" s="11" t="n">
-        <v>0.01957579784845818</v>
+        <v>0.01957122849858153</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>6781.07</v>
+        <v>6783.66</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>6881.07</v>
+        <v>6883.66</v>
       </c>
       <c r="N28" s="12" t="n">
         <v>100</v>
       </c>
       <c r="O28" s="13" t="n">
-        <v>0.01474693521818828</v>
+        <v>0.01474130484133934</v>
       </c>
     </row>
     <row r="29">
@@ -9277,7 +9277,7 @@
         <v>46272</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
@@ -9293,16 +9293,16 @@
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="12" t="n">
-        <v>6795.14</v>
+        <v>6798.2</v>
       </c>
       <c r="M29" s="12" t="n">
-        <v>6979.54</v>
+        <v>6982.65</v>
       </c>
       <c r="N29" s="12" t="n">
-        <v>184.4</v>
+        <v>184.45</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>0.0271370420624152</v>
+        <v>0.02713218204818922</v>
       </c>
     </row>
     <row r="30">
@@ -9310,7 +9310,7 @@
         <v>46272</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C30" s="41" t="inlineStr">
         <is>
@@ -9318,40 +9318,40 @@
         </is>
       </c>
       <c r="D30" s="8" t="n">
-        <v>47.823</v>
+        <v>47.8235</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>49.043</v>
+        <v>49.0435</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>1.22</v>
       </c>
       <c r="G30" s="9" t="n">
-        <v>0.02551073751123936</v>
+        <v>0.02551047079364747</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>55.4727</v>
+        <v>55.4876</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>57.1371</v>
+        <v>57.1476</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>1.6644</v>
+        <v>1.66</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>0.03000394788787998</v>
+        <v>0.02991659397775359</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>6706.92</v>
+        <v>6710.09</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>6908.22</v>
+        <v>6911.48</v>
       </c>
       <c r="N30" s="12" t="n">
-        <v>201.3</v>
+        <v>201.39</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>0.03001377681558748</v>
+        <v>0.03001301025768656</v>
       </c>
     </row>
     <row r="31">
@@ -9359,7 +9359,7 @@
         <v>46272</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -9367,40 +9367,40 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>48.3122</v>
+        <v>48.3107</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>48.5302</v>
+        <v>48.5286</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>0.218</v>
+        <v>0.2179</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>0.00451231779964481</v>
+        <v>0.004510387967882891</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>56.0766</v>
+        <v>56.084</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>56.4144</v>
+        <v>56.4218</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>0.3378</v>
       </c>
       <c r="K31" s="11" t="n">
-        <v>0.006023903018371299</v>
+        <v>0.006023108194850582</v>
       </c>
       <c r="L31" s="12" t="n">
-        <v>6773.2</v>
+        <v>6776.09</v>
       </c>
       <c r="M31" s="12" t="n">
-        <v>6875.31</v>
+        <v>6878.24</v>
       </c>
       <c r="N31" s="12" t="n">
-        <v>102.11</v>
+        <v>102.15</v>
       </c>
       <c r="O31" s="13" t="n">
-        <v>0.01507559203921337</v>
+        <v>0.0150750654138301</v>
       </c>
     </row>
     <row r="32">
@@ -9408,7 +9408,7 @@
         <v>46272</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C32" s="43" t="inlineStr">
         <is>
@@ -9416,40 +9416,40 @@
         </is>
       </c>
       <c r="D32" s="8" t="n">
-        <v>47.9876</v>
+        <v>47.9875</v>
       </c>
       <c r="E32" s="8" t="n">
         <v>48.79</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.8024</v>
+        <v>0.8025</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>0.01672098625478249</v>
+        <v>0.01672310497525397</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>55.8099</v>
+        <v>55.8229</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>56.6616</v>
+        <v>56.6747</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>0.8517</v>
+        <v>0.8518</v>
       </c>
       <c r="K32" s="11" t="n">
-        <v>0.01526073331075669</v>
+        <v>0.01525897078080859</v>
       </c>
       <c r="L32" s="12" t="n">
-        <v>6734.61</v>
+        <v>6738.33</v>
       </c>
       <c r="M32" s="12" t="n">
-        <v>6930.98</v>
+        <v>6934.84</v>
       </c>
       <c r="N32" s="12" t="n">
-        <v>196.37</v>
+        <v>196.51</v>
       </c>
       <c r="O32" s="13" t="n">
-        <v>0.02915833285075157</v>
+        <v>0.02916301220035231</v>
       </c>
     </row>
     <row r="33">
@@ -9457,7 +9457,7 @@
         <v>46272</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
@@ -9477,28 +9477,28 @@
         <v>0.00421853546199901</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>56.1223</v>
+        <v>56.13</v>
       </c>
       <c r="I33" s="10" t="n">
-        <v>56.3484</v>
+        <v>56.3561</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>0.2261</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>0.004028701603462439</v>
+        <v>0.004028148939960805</v>
       </c>
       <c r="L33" s="12" t="n">
-        <v>6773.71</v>
+        <v>6774.75</v>
       </c>
       <c r="M33" s="12" t="n">
-        <v>6828.12</v>
+        <v>6829.16</v>
       </c>
       <c r="N33" s="12" t="n">
         <v>54.41</v>
       </c>
       <c r="O33" s="13" t="n">
-        <v>0.00803252575029046</v>
+        <v>0.008031292667626111</v>
       </c>
     </row>
     <row r="34">
@@ -9506,7 +9506,7 @@
         <v>46272</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C34" s="45" t="inlineStr">
         <is>
@@ -9526,28 +9526,28 @@
         <v>0.02010394499577307</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>55.8106</v>
+        <v>55.816</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>56.927</v>
+        <v>56.9325</v>
       </c>
       <c r="J34" s="10" t="n">
-        <v>1.1164</v>
+        <v>1.1165</v>
       </c>
       <c r="K34" s="11" t="n">
-        <v>0.02000336853572619</v>
+        <v>0.02000322488175434</v>
       </c>
       <c r="L34" s="12" t="n">
-        <v>6739.74</v>
+        <v>6742.87</v>
       </c>
       <c r="M34" s="12" t="n">
-        <v>6884.34</v>
+        <v>6887.47</v>
       </c>
       <c r="N34" s="12" t="n">
         <v>144.6</v>
       </c>
       <c r="O34" s="13" t="n">
-        <v>0.02145483356924748</v>
+        <v>0.02144487436358702</v>
       </c>
     </row>
     <row r="35">
@@ -9555,7 +9555,7 @@
         <v>46272</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C35" s="46" t="inlineStr">
         <is>
@@ -9563,28 +9563,28 @@
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>48.291</v>
+        <v>48.292</v>
       </c>
       <c r="E35" s="8" t="n">
         <v>48.347</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.056</v>
+        <v>0.055</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>0.00115963637116647</v>
+        <v>0.001138904994616086</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>55.989</v>
+        <v>55.999</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>56.131</v>
+        <v>56.141</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>0.142</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>0.002536212470306667</v>
+        <v>0.002535759567135127</v>
       </c>
       <c r="L35" s="12" t="n"/>
       <c r="M35" s="12" t="n"/>
@@ -9596,7 +9596,7 @@
         <v>46272</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C36" s="47" t="inlineStr">
         <is>
@@ -9616,28 +9616,28 @@
         <v>0.02092487968194183</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>55.56</v>
+        <v>55.57</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>56.7</v>
+        <v>56.71</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>1.14</v>
       </c>
       <c r="K36" s="11" t="n">
-        <v>0.02051835853131749</v>
+        <v>0.02051466618679143</v>
       </c>
       <c r="L36" s="12" t="n">
-        <v>6711.62</v>
+        <v>6715.15</v>
       </c>
       <c r="M36" s="12" t="n">
-        <v>6915.1</v>
+        <v>6918.47</v>
       </c>
       <c r="N36" s="12" t="n">
-        <v>203.48</v>
+        <v>203.32</v>
       </c>
       <c r="O36" s="13" t="n">
-        <v>0.03031756863469624</v>
+        <v>0.03027780466556965</v>
       </c>
     </row>
     <row r="37">
@@ -9645,7 +9645,7 @@
         <v>46272</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C37" s="48" t="inlineStr">
         <is>
@@ -9665,28 +9665,28 @@
         <v>0.02023091899095272</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>55.8096</v>
+        <v>55.8217</v>
       </c>
       <c r="I37" s="10" t="n">
-        <v>56.9386</v>
+        <v>56.951</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1.129</v>
+        <v>1.1293</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>0.02022949456724291</v>
+        <v>0.02023048384409647</v>
       </c>
       <c r="L37" s="12" t="n">
-        <v>6772.85</v>
+        <v>6774.09</v>
       </c>
       <c r="M37" s="12" t="n">
-        <v>6909.61</v>
+        <v>6910.87</v>
       </c>
       <c r="N37" s="12" t="n">
-        <v>136.76</v>
+        <v>136.78</v>
       </c>
       <c r="O37" s="13" t="n">
-        <v>0.02019238577555977</v>
+        <v>0.02019164197700355</v>
       </c>
     </row>
     <row r="38">
@@ -9694,7 +9694,7 @@
         <v>46272</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
@@ -9702,40 +9702,40 @@
         </is>
       </c>
       <c r="D38" s="8" t="n">
-        <v>48.0735</v>
+        <v>48.074</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>48.7276</v>
+        <v>48.7281</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>0.6541</v>
       </c>
       <c r="G38" s="9" t="n">
-        <v>0.01360624876491206</v>
+        <v>0.01360610725132088</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>55.8193</v>
+        <v>55.8289</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>56.6353</v>
+        <v>56.645</v>
       </c>
       <c r="J38" s="10" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.8161</v>
       </c>
       <c r="K38" s="11" t="n">
-        <v>0.01461859965997424</v>
+        <v>0.01461787712098931</v>
       </c>
       <c r="L38" s="12" t="n">
-        <v>6742.04</v>
+        <v>6745.06</v>
       </c>
       <c r="M38" s="12" t="n">
-        <v>6878.17</v>
+        <v>6881.25</v>
       </c>
       <c r="N38" s="12" t="n">
-        <v>136.13</v>
+        <v>136.19</v>
       </c>
       <c r="O38" s="13" t="n">
-        <v>0.02019121808829375</v>
+        <v>0.02019107317058707</v>
       </c>
     </row>
     <row r="39">
@@ -9743,7 +9743,7 @@
         <v>46272</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="C39" s="50" t="inlineStr">
         <is>
@@ -9751,40 +9751,40 @@
         </is>
       </c>
       <c r="D39" s="8" t="n">
-        <v>47.9025</v>
+        <v>47.9032</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>48.9029</v>
+        <v>48.9031</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>1.0004</v>
+        <v>0.9999</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>0.02088408746933876</v>
+        <v>0.02087334457823277</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>55.6441</v>
+        <v>55.6543</v>
       </c>
       <c r="I39" s="10" t="n">
-        <v>56.8623</v>
+        <v>56.8712</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1.2182</v>
+        <v>1.2169</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>0.0218927074029412</v>
+        <v>0.02186533655081458</v>
       </c>
       <c r="L39" s="12" t="n">
-        <v>6760.38</v>
+        <v>6764.08</v>
       </c>
       <c r="M39" s="12" t="n">
-        <v>6975.08</v>
+        <v>6978.79</v>
       </c>
       <c r="N39" s="12" t="n">
-        <v>214.7</v>
+        <v>214.71</v>
       </c>
       <c r="O39" s="13" t="n">
-        <v>0.03175856978453874</v>
+        <v>0.03174267601802463</v>
       </c>
     </row>
   </sheetData>
@@ -70626,7 +70626,7 @@
       </c>
       <c r="B5" s="62" t="n"/>
       <c r="C5" s="64" t="n">
-        <v>0.6433101851851852</v>
+        <v>0.6471759259259259</v>
       </c>
       <c r="D5" s="62" t="n"/>
       <c r="F5" s="62" t="inlineStr">
@@ -70710,7 +70710,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="70" t="n">
-        <v>0.02022949456724291</v>
+        <v>0.02023048384409647</v>
       </c>
       <c r="O6" s="71" t="inlineStr">
         <is>
@@ -70718,10 +70718,10 @@
         </is>
       </c>
       <c r="P6" s="72" t="n">
-        <v>55.8096</v>
+        <v>55.8217</v>
       </c>
       <c r="Q6" s="72" t="n">
-        <v>56.9386</v>
+        <v>56.951</v>
       </c>
     </row>
     <row r="7">
@@ -70763,7 +70763,7 @@
         <v>5</v>
       </c>
       <c r="N7" s="70" t="n">
-        <v>0.02019238577555977</v>
+        <v>0.02019164197700355</v>
       </c>
       <c r="O7" s="71" t="inlineStr">
         <is>
@@ -70771,10 +70771,10 @@
         </is>
       </c>
       <c r="P7" s="72" t="n">
-        <v>6772.85</v>
+        <v>6774.09</v>
       </c>
       <c r="Q7" s="72" t="n">
-        <v>6909.61</v>
+        <v>6910.87</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Günlük kur verisi: 08.09.2026 14:19
</commit_message>
<xml_diff>
--- a/output/banka_kurlari.xlsx
+++ b/output/banka_kurlari.xlsx
@@ -8158,7 +8158,7 @@
         <v>46273</v>
       </c>
       <c r="B2" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
@@ -8178,28 +8178,28 @@
         <v>0.02832326283987915</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>55.3421</v>
+        <v>55.3423</v>
       </c>
       <c r="I2" s="10" t="n">
-        <v>56.9145</v>
+        <v>56.9097</v>
       </c>
       <c r="J2" s="10" t="n">
-        <v>1.5724</v>
+        <v>1.5674</v>
       </c>
       <c r="K2" s="11" t="n">
-        <v>0.02841236599261683</v>
+        <v>0.02832191650871033</v>
       </c>
       <c r="L2" s="12" t="n">
-        <v>6674.85</v>
+        <v>6670.62</v>
       </c>
       <c r="M2" s="12" t="n">
-        <v>6915.26</v>
+        <v>6910.88</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>240.41</v>
+        <v>240.26</v>
       </c>
       <c r="O2" s="13" t="n">
-        <v>0.03601728877802497</v>
+        <v>0.03601764153856763</v>
       </c>
     </row>
     <row r="3">
@@ -8207,7 +8207,7 @@
         <v>46273</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
@@ -8227,28 +8227,28 @@
         <v>0.01625085831998169</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>55.806</v>
+        <v>55.801</v>
       </c>
       <c r="I3" s="10" t="n">
         <v>56.718</v>
       </c>
       <c r="J3" s="10" t="n">
-        <v>0.912</v>
+        <v>0.917</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>0.01634232878185141</v>
+        <v>0.01643339725094532</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>6747.58</v>
+        <v>6750.13</v>
       </c>
       <c r="M3" s="12" t="n">
-        <v>6885.97</v>
+        <v>6889.21</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>138.39</v>
+        <v>139.08</v>
       </c>
       <c r="O3" s="13" t="n">
-        <v>0.02050957528476876</v>
+        <v>0.02060404762574943</v>
       </c>
     </row>
     <row r="4">
@@ -8256,7 +8256,7 @@
         <v>46273</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
@@ -8264,40 +8264,40 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>48.241</v>
+        <v>48.242</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>48.539</v>
+        <v>48.538</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.298</v>
+        <v>0.296</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>0.006177318048962501</v>
+        <v>0.006135732349405083</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>55.85</v>
+        <v>55.841</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>56.372</v>
+        <v>56.359</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.522</v>
+        <v>0.518</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>0.009346463742166517</v>
+        <v>0.009276338174459626</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>6808.62</v>
+        <v>6806.11</v>
       </c>
       <c r="M4" s="12" t="n">
-        <v>6877.88</v>
+        <v>6875.12</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>69.26000000000001</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="O4" s="13" t="n">
-        <v>0.01017239910583936</v>
+        <v>0.01013941884571363</v>
       </c>
     </row>
     <row r="5">
@@ -8305,7 +8305,7 @@
         <v>46273</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -8313,40 +8313,40 @@
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>48.27</v>
+        <v>48.29</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>48.48</v>
+        <v>48.5</v>
       </c>
       <c r="F5" s="8" t="n">
         <v>0.21</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>0.00435052827843381</v>
+        <v>0.004348726444398427</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>55.901</v>
+        <v>55.918</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>56.301</v>
+        <v>56.32</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.4</v>
+        <v>0.402</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>0.007155507057118835</v>
+        <v>0.007189098322543724</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>6736.92</v>
+        <v>6743.25</v>
       </c>
       <c r="M5" s="12" t="n">
-        <v>6900</v>
+        <v>6905</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>163.08</v>
+        <v>161.75</v>
       </c>
       <c r="O5" s="13" t="n">
-        <v>0.02420690760763079</v>
+        <v>0.02398694991287584</v>
       </c>
     </row>
     <row r="6">
@@ -8354,7 +8354,7 @@
         <v>46273</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
@@ -8362,40 +8362,40 @@
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>47.6153</v>
+        <v>47.6154</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>48.8923</v>
+        <v>48.8916</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>1.277</v>
+        <v>1.2762</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>0.02681911066400926</v>
+        <v>0.02680225305258383</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>55.3962</v>
+        <v>55.3953</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>56.7623</v>
+        <v>56.7603</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>1.3661</v>
+        <v>1.365</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0.02466053628227207</v>
+        <v>0.02464107965838257</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>6732.17</v>
+        <v>6737.63</v>
       </c>
       <c r="M6" s="12" t="n">
-        <v>6883.32</v>
+        <v>6888.74</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>151.15</v>
+        <v>151.11</v>
       </c>
       <c r="O6" s="13" t="n">
-        <v>0.02245189886767565</v>
+        <v>0.02242776762748919</v>
       </c>
     </row>
     <row r="7">
@@ -8403,7 +8403,7 @@
         <v>46273</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
@@ -8435,16 +8435,16 @@
         <v>0.04073523007693424</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>6730.24</v>
+        <v>6734.78</v>
       </c>
       <c r="M7" s="12" t="n">
-        <v>6924.7</v>
+        <v>6930.34</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>194.46</v>
+        <v>195.56</v>
       </c>
       <c r="O7" s="13" t="n">
-        <v>0.02889347185241537</v>
+        <v>0.02903732564389631</v>
       </c>
     </row>
     <row r="8">
@@ -8452,7 +8452,7 @@
         <v>46273</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
@@ -8460,40 +8460,40 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>47.7171</v>
+        <v>47.7172</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>49.1172</v>
+        <v>49.1173</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>1.4001</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>0.02934168254147884</v>
+        <v>0.02934162105069032</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>55.4086</v>
+        <v>55.4087</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>57.0393</v>
+        <v>57.0345</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>1.6307</v>
+        <v>1.6258</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>0.02943044942481853</v>
+        <v>0.02934196254378825</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>6744.87</v>
+        <v>6749.93</v>
       </c>
       <c r="M8" s="12" t="n">
-        <v>6943.88</v>
+        <v>6949.16</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>199.01</v>
+        <v>199.23</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>0.02950538705712638</v>
+        <v>0.02951586164597262</v>
       </c>
     </row>
     <row r="9">
@@ -8501,7 +8501,7 @@
         <v>46273</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
@@ -8509,40 +8509,40 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>48.3863</v>
+        <v>48.3865</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>48.4436</v>
+        <v>48.4438</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>0.0573</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.001184219500147769</v>
+        <v>0.001184214605313466</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>56.1755</v>
+        <v>56.1757</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>56.2589</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.0834</v>
+        <v>0.0832</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>0.001484632980569821</v>
+        <v>0.001481067436631853</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>6797.41</v>
+        <v>6802.62</v>
       </c>
       <c r="M9" s="12" t="n">
-        <v>6826.33</v>
+        <v>6831.56</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>28.92</v>
+        <v>28.94</v>
       </c>
       <c r="O9" s="13" t="n">
-        <v>0.004254561663927878</v>
+        <v>0.00425424321805422</v>
       </c>
     </row>
     <row r="10">
@@ -8550,7 +8550,7 @@
         <v>46273</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
@@ -8558,40 +8558,40 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>48.4001</v>
+        <v>48.4002</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>48.4388</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.0387</v>
+        <v>0.0386</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.0007995851248241223</v>
+        <v>0.0007975173656307206</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>56.1574</v>
+        <v>56.1527</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>56.2676</v>
       </c>
       <c r="J10" s="10" t="n">
-        <v>0.1102</v>
+        <v>0.1149</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>0.001962341561397073</v>
+        <v>0.002046206148591252</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>6793.89</v>
+        <v>6799.08</v>
       </c>
       <c r="M10" s="12" t="n">
-        <v>6826.27</v>
+        <v>6831.63</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>32.38</v>
+        <v>32.55</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>0.004766047139414974</v>
+        <v>0.004787412414620802</v>
       </c>
     </row>
     <row r="11">
@@ -8599,7 +8599,7 @@
         <v>46273</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
@@ -8607,40 +8607,40 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>48.0858</v>
+        <v>48.0863</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>49.3276</v>
+        <v>49.3275</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>1.2418</v>
+        <v>1.2412</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.02582467173261129</v>
+        <v>0.02581192564202278</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>55.7374</v>
+        <v>55.7428</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>57.0256</v>
+        <v>57.0255</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>1.2882</v>
+        <v>1.2827</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>0.02311194996537334</v>
+        <v>0.02301104357872227</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6752.44</v>
+        <v>6753.01</v>
       </c>
       <c r="M11" s="12" t="n">
-        <v>6863.45</v>
+        <v>6863.44</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>111.01</v>
+        <v>110.43</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>0.01643998317645177</v>
+        <v>0.0163527079035867</v>
       </c>
     </row>
     <row r="12">
@@ -8648,7 +8648,7 @@
         <v>46273</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
@@ -8671,25 +8671,25 @@
         <v>55.6656</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>56.8311</v>
+        <v>56.8262</v>
       </c>
       <c r="J12" s="10" t="n">
-        <v>1.1655</v>
+        <v>1.1606</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>0.02093752694662413</v>
+        <v>0.02084950130780949</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>6742.9</v>
+        <v>6747.47</v>
       </c>
       <c r="M12" s="12" t="n">
-        <v>6899.8</v>
+        <v>6904.46</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>156.9</v>
+        <v>156.99</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>0.02326891990093283</v>
+        <v>0.02326649840606924</v>
       </c>
     </row>
     <row r="13">
@@ -8697,7 +8697,7 @@
         <v>46273</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
@@ -8705,40 +8705,40 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>48.1605</v>
+        <v>48.1606</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>48.7673</v>
+        <v>48.7674</v>
       </c>
       <c r="F13" s="8" t="n">
         <v>0.6068</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.01259953696494015</v>
+        <v>0.01259951080343684</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>55.9366</v>
+        <v>55.9275</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>56.5968</v>
+        <v>56.5882</v>
       </c>
       <c r="J13" s="10" t="n">
-        <v>0.6602</v>
+        <v>0.6607</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>0.01180264799791192</v>
+        <v>0.01181350856018953</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6822.33</v>
+        <v>6811.49</v>
       </c>
       <c r="M13" s="12" t="n">
-        <v>6876.64</v>
+        <v>6865.81</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>54.31</v>
+        <v>54.32</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>0.007960623423375885</v>
+        <v>0.007974760294737275</v>
       </c>
     </row>
     <row r="14">
@@ -8746,7 +8746,7 @@
         <v>46273</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
@@ -8766,28 +8766,28 @@
         <v>0.0283512191024214</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>55.295</v>
+        <v>55.281</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>56.863</v>
+        <v>56.848</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>1.568</v>
+        <v>1.567</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>0.02835699430328239</v>
+        <v>0.02834608635878512</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>6716.99</v>
+        <v>6703.74</v>
       </c>
       <c r="M14" s="12" t="n">
-        <v>6964.98</v>
+        <v>6951.25</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>247.99</v>
+        <v>247.51</v>
       </c>
       <c r="O14" s="13" t="n">
-        <v>0.03691981080811495</v>
+        <v>0.03692118131073102</v>
       </c>
     </row>
     <row r="15">
@@ -8795,7 +8795,7 @@
         <v>46273</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
@@ -8803,40 +8803,40 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>48.1605</v>
+        <v>48.1606</v>
       </c>
       <c r="E15" s="8" t="n">
         <v>48.7674</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.6069</v>
+        <v>0.6068</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>0.01260161335534307</v>
+        <v>0.01259951080343684</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>55.94</v>
+        <v>55.9386</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>56.6003</v>
+        <v>56.5993</v>
       </c>
       <c r="J15" s="10" t="n">
-        <v>0.6603</v>
+        <v>0.6607</v>
       </c>
       <c r="K15" s="11" t="n">
-        <v>0.01180371826957454</v>
+        <v>0.01181116438380653</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>6817.56</v>
+        <v>6822.38</v>
       </c>
       <c r="M15" s="12" t="n">
-        <v>6871.91</v>
+        <v>6876.76</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>54.35</v>
+        <v>54.38</v>
       </c>
       <c r="O15" s="13" t="n">
-        <v>0.007972060385240468</v>
+        <v>0.007970825430421642</v>
       </c>
     </row>
     <row r="16">
@@ -8844,7 +8844,7 @@
         <v>46273</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
@@ -8864,28 +8864,28 @@
         <v>0.0204040416658859</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>55.7721</v>
+        <v>55.7697</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>56.9101</v>
+        <v>56.9076</v>
       </c>
       <c r="J16" s="10" t="n">
-        <v>1.138</v>
+        <v>1.1379</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>0.02040446746670826</v>
+        <v>0.020403552466662</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>6751.49</v>
+        <v>6745</v>
       </c>
       <c r="M16" s="12" t="n">
-        <v>6958.82</v>
+        <v>6952.78</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>207.33</v>
+        <v>207.78</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>0.0307087768774004</v>
+        <v>0.03080504077094144</v>
       </c>
     </row>
     <row r="17">
@@ -8893,7 +8893,7 @@
         <v>46273</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
@@ -8901,40 +8901,40 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>48.41</v>
+        <v>48.42</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>48.464</v>
+        <v>48.474</v>
       </c>
       <c r="F17" s="8" t="n">
         <v>0.054</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.001115472009915307</v>
+        <v>0.001115241635687732</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>56.064</v>
+        <v>56.07</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>56.211</v>
+        <v>56.218</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>0.147</v>
+        <v>0.148</v>
       </c>
       <c r="K17" s="11" t="n">
-        <v>0.002622003424657534</v>
+        <v>0.002639557695737471</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>6770.89</v>
+        <v>6777.87</v>
       </c>
       <c r="M17" s="12" t="n">
-        <v>6844.64</v>
+        <v>6851.75</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>73.75</v>
+        <v>73.88</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>0.01089221653283394</v>
+        <v>0.01090017955493392</v>
       </c>
     </row>
     <row r="18">
@@ -8942,7 +8942,7 @@
         <v>46273</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
@@ -8950,40 +8950,40 @@
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>48.3804</v>
+        <v>48.3806</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>48.5272</v>
+        <v>48.5271</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>0.1468</v>
+        <v>0.1465</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>0.003034286611933758</v>
+        <v>0.003028073235966483</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>56.1707</v>
+        <v>56.1637</v>
       </c>
       <c r="I18" s="10" t="n">
-        <v>56.343</v>
+        <v>56.3356</v>
       </c>
       <c r="J18" s="10" t="n">
-        <v>0.1723</v>
+        <v>0.1719</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>0.003067435513532856</v>
+        <v>0.003060695787492633</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>6806.82</v>
+        <v>6809.39</v>
       </c>
       <c r="M18" s="12" t="n">
-        <v>6854.94</v>
+        <v>6857.51</v>
       </c>
       <c r="N18" s="12" t="n">
         <v>48.12</v>
       </c>
       <c r="O18" s="13" t="n">
-        <v>0.00706938041552443</v>
+        <v>0.007066712289940802</v>
       </c>
     </row>
     <row r="19">
@@ -8991,7 +8991,7 @@
         <v>46273</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
@@ -9007,16 +9007,16 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="11" t="n"/>
       <c r="L19" s="12" t="n">
-        <v>6796.3</v>
+        <v>6798.49</v>
       </c>
       <c r="M19" s="12" t="n">
-        <v>6994.73</v>
+        <v>6996.94</v>
       </c>
       <c r="N19" s="12" t="n">
-        <v>198.43</v>
+        <v>198.45</v>
       </c>
       <c r="O19" s="13" t="n">
-        <v>0.02919676883009873</v>
+        <v>0.0291903054943083</v>
       </c>
     </row>
     <row r="20">
@@ -9024,7 +9024,7 @@
         <v>46273</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C20" s="31" t="inlineStr">
         <is>
@@ -9032,40 +9032,40 @@
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>47.9687</v>
+        <v>47.9671</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>48.8518</v>
+        <v>48.8538</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0.8831</v>
+        <v>0.8867</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>0.01840992146962498</v>
+        <v>0.0184855869960869</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>55.7075</v>
+        <v>55.7028</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>56.7631</v>
+        <v>56.7533</v>
       </c>
       <c r="J20" s="10" t="n">
-        <v>1.0556</v>
+        <v>1.0505</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>0.01894897455459319</v>
+        <v>0.01885901606382444</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>6749.33</v>
+        <v>6753.08</v>
       </c>
       <c r="M20" s="12" t="n">
-        <v>7195.37</v>
+        <v>7198.32</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>446.04</v>
+        <v>445.24</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>0.06608655970296311</v>
+        <v>0.06593139722911619</v>
       </c>
     </row>
     <row r="21">
@@ -9073,7 +9073,7 @@
         <v>46273</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C21" s="32" t="inlineStr">
         <is>
@@ -9081,40 +9081,40 @@
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>47.9137</v>
+        <v>47.9138</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>48.9178</v>
+        <v>48.9174</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>1.0041</v>
+        <v>1.0036</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>0.02095642791101501</v>
+        <v>0.02094594876632619</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>55.7174</v>
+        <v>55.7129</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>56.7241</v>
+        <v>56.7191</v>
       </c>
       <c r="J21" s="10" t="n">
-        <v>1.0067</v>
+        <v>1.0062</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>0.01806796440609217</v>
+        <v>0.01806044919578769</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>6718.27</v>
+        <v>6718.18</v>
       </c>
       <c r="M21" s="12" t="n">
-        <v>6969.78</v>
+        <v>6970.88</v>
       </c>
       <c r="N21" s="12" t="n">
-        <v>251.51</v>
+        <v>252.7</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>0.03743672106063019</v>
+        <v>0.0376143538875112</v>
       </c>
     </row>
     <row r="22">
@@ -9122,7 +9122,7 @@
         <v>46273</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
@@ -9130,40 +9130,40 @@
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>47.8397</v>
+        <v>47.8386</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>48.9974</v>
+        <v>48.9989</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>1.1577</v>
+        <v>1.1603</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>0.02419956646885327</v>
+        <v>0.02425447232987588</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>55.5467</v>
+        <v>55.5358</v>
       </c>
       <c r="I22" s="10" t="n">
-        <v>56.8958</v>
+        <v>56.8927</v>
       </c>
       <c r="J22" s="10" t="n">
-        <v>1.3491</v>
+        <v>1.3569</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>0.0242876714548299</v>
+        <v>0.02443288833509196</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>6738.82</v>
+        <v>6742.5</v>
       </c>
       <c r="M22" s="12" t="n">
-        <v>6923.63</v>
+        <v>6928.77</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>184.81</v>
+        <v>186.27</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>0.02742468265957541</v>
+        <v>0.02762625139043381</v>
       </c>
     </row>
     <row r="23">
@@ -9171,7 +9171,7 @@
         <v>46273</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C23" s="34" t="inlineStr">
         <is>
@@ -9179,16 +9179,16 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>48.43</v>
+        <v>48.45</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>48.45</v>
+        <v>48.46</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>0.0004129671691100557</v>
+        <v>0.0002063983488132095</v>
       </c>
       <c r="H23" s="10" t="n">
         <v>56.1</v>
@@ -9203,16 +9203,16 @@
         <v>0.00089126559714795</v>
       </c>
       <c r="L23" s="12" t="n">
-        <v>6824.01</v>
+        <v>6821.96</v>
       </c>
       <c r="M23" s="12" t="n">
-        <v>6831.69</v>
+        <v>6828.23</v>
       </c>
       <c r="N23" s="12" t="n">
-        <v>7.68</v>
+        <v>6.27</v>
       </c>
       <c r="O23" s="13" t="n">
-        <v>0.001125437975618441</v>
+        <v>0.000919090701206105</v>
       </c>
     </row>
     <row r="24">
@@ -9220,7 +9220,7 @@
         <v>46273</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
@@ -9228,40 +9228,40 @@
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>47.7407</v>
+        <v>47.7404</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>48.7802</v>
+        <v>48.7807</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>1.0395</v>
+        <v>1.0403</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.02177387428336828</v>
+        <v>0.02179076840579467</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>55.4418</v>
+        <v>55.4352</v>
       </c>
       <c r="I24" s="10" t="n">
-        <v>56.6495</v>
+        <v>56.6437</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>1.2077</v>
+        <v>1.2085</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>0.02178320328705056</v>
+        <v>0.02180022801396946</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>6708.67</v>
+        <v>6712.74</v>
       </c>
       <c r="M24" s="12" t="n">
-        <v>6886.12</v>
+        <v>6890.53</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>177.45</v>
+        <v>177.79</v>
       </c>
       <c r="O24" s="13" t="n">
-        <v>0.02645084644199223</v>
+        <v>0.02648545899290007</v>
       </c>
     </row>
     <row r="25">
@@ -9269,7 +9269,7 @@
         <v>46273</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C25" s="36" t="inlineStr">
         <is>
@@ -9310,7 +9310,7 @@
         <v>46273</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C26" s="37" t="inlineStr">
         <is>
@@ -9318,40 +9318,40 @@
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>48.3883</v>
+        <v>48.3885</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>48.443</v>
+        <v>48.4433</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>0.0547</v>
+        <v>0.0548</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>0.001130438556427897</v>
+        <v>0.0011325004908191</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>56.1778</v>
+        <v>56.1722</v>
       </c>
       <c r="I26" s="10" t="n">
-        <v>56.2605</v>
+        <v>56.2563</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>0.0827</v>
+        <v>0.08409999999999999</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>0.001472111759449462</v>
+        <v>0.0014971818800047</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>6795.62</v>
+        <v>6798.7</v>
       </c>
       <c r="M26" s="12" t="n">
-        <v>6823.88</v>
+        <v>6826.73</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>28.26</v>
+        <v>28.03</v>
       </c>
       <c r="O26" s="13" t="n">
-        <v>0.004158560955438944</v>
+        <v>0.00412284701487049</v>
       </c>
     </row>
     <row r="27">
@@ -9359,7 +9359,7 @@
         <v>46273</v>
       </c>
       <c r="B27" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C27" s="38" t="inlineStr">
         <is>
@@ -9367,40 +9367,40 @@
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>48.393</v>
+        <v>48.409</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>48.484</v>
+        <v>48.513</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.091</v>
+        <v>0.104</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>0.001880437253321761</v>
+        <v>0.002148360841992191</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>56.05</v>
+        <v>56.068</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>56.253</v>
+        <v>56.272</v>
       </c>
       <c r="J27" s="10" t="n">
-        <v>0.203</v>
+        <v>0.204</v>
       </c>
       <c r="K27" s="11" t="n">
-        <v>0.003621766280107047</v>
+        <v>0.003638439038310623</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>6788</v>
+        <v>6794</v>
       </c>
       <c r="M27" s="12" t="n">
-        <v>6834</v>
+        <v>6843</v>
       </c>
       <c r="N27" s="12" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>0.006776664702416029</v>
+        <v>0.007212246099499558</v>
       </c>
     </row>
     <row r="28">
@@ -9408,7 +9408,7 @@
         <v>46273</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -9416,40 +9416,40 @@
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>47.9215</v>
+        <v>47.9245</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>48.9215</v>
+        <v>48.9245</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>0.02086746032574105</v>
+        <v>0.02086615405481539</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>55.677</v>
+        <v>55.674</v>
       </c>
       <c r="I28" s="10" t="n">
-        <v>56.767</v>
+        <v>56.764</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>1.09</v>
       </c>
       <c r="K28" s="11" t="n">
-        <v>0.01957720423154983</v>
+        <v>0.01957825915148903</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>6803.33</v>
+        <v>6794.53</v>
       </c>
       <c r="M28" s="12" t="n">
-        <v>6903.33</v>
+        <v>6894.53</v>
       </c>
       <c r="N28" s="12" t="n">
         <v>100</v>
       </c>
       <c r="O28" s="13" t="n">
-        <v>0.01469868432076645</v>
+        <v>0.01471772146123426</v>
       </c>
     </row>
     <row r="29">
@@ -9457,7 +9457,7 @@
         <v>46273</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
@@ -9473,16 +9473,16 @@
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="11" t="n"/>
       <c r="L29" s="12" t="n">
-        <v>6797.08</v>
+        <v>6798.49</v>
       </c>
       <c r="M29" s="12" t="n">
-        <v>6981.56</v>
+        <v>6982.97</v>
       </c>
       <c r="N29" s="12" t="n">
         <v>184.48</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>0.02714106645794959</v>
+        <v>0.0271354374280171</v>
       </c>
     </row>
     <row r="30">
@@ -9490,7 +9490,7 @@
         <v>46273</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C30" s="41" t="inlineStr">
         <is>
@@ -9510,28 +9510,28 @@
         <v>0.02549634273772204</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>55.4468</v>
+        <v>55.442</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>57.1047</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>1.6579</v>
+        <v>1.6627</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>0.02990073367624462</v>
+        <v>0.02998989935428015</v>
       </c>
       <c r="L30" s="12" t="n">
-        <v>6717.76</v>
+        <v>6720.56</v>
       </c>
       <c r="M30" s="12" t="n">
-        <v>6919.37</v>
+        <v>6922.35</v>
       </c>
       <c r="N30" s="12" t="n">
-        <v>201.61</v>
+        <v>201.79</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>0.03001149192588005</v>
+        <v>0.03002577166188532</v>
       </c>
     </row>
     <row r="31">
@@ -9539,7 +9539,7 @@
         <v>46273</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C31" s="42" t="inlineStr">
         <is>
@@ -9547,40 +9547,40 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>48.3388</v>
+        <v>48.3389</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>48.5568</v>
+        <v>48.557</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>0.218</v>
+        <v>0.2181</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>0.004509834749724858</v>
+        <v>0.004511894147363717</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>56.0514</v>
+        <v>56.0462</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>56.389</v>
+        <v>56.3839</v>
       </c>
       <c r="J31" s="10" t="n">
-        <v>0.3376</v>
+        <v>0.3377</v>
       </c>
       <c r="K31" s="11" t="n">
-        <v>0.006023043135407857</v>
+        <v>0.006025386199242767</v>
       </c>
       <c r="L31" s="12" t="n">
-        <v>6782.97</v>
+        <v>6786.7</v>
       </c>
       <c r="M31" s="12" t="n">
-        <v>6885.23</v>
+        <v>6889.01</v>
       </c>
       <c r="N31" s="12" t="n">
-        <v>102.26</v>
+        <v>102.31</v>
       </c>
       <c r="O31" s="13" t="n">
-        <v>0.01507599178530939</v>
+        <v>0.01507507330514094</v>
       </c>
     </row>
     <row r="32">
@@ -9588,7 +9588,7 @@
         <v>46273</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C32" s="43" t="inlineStr">
         <is>
@@ -9599,37 +9599,37 @@
         <v>48.0142</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>48.8163</v>
+        <v>48.8166</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.8021</v>
+        <v>0.8024</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>0.01670547463042183</v>
+        <v>0.01671172278201032</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>55.79</v>
+        <v>55.7852</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>56.6404</v>
+        <v>56.6354</v>
       </c>
       <c r="J32" s="10" t="n">
-        <v>0.8504</v>
+        <v>0.8502</v>
       </c>
       <c r="K32" s="11" t="n">
-        <v>0.01524287506721635</v>
+        <v>0.01524060144984691</v>
       </c>
       <c r="L32" s="12" t="n">
-        <v>6744.81</v>
+        <v>6743.42</v>
       </c>
       <c r="M32" s="12" t="n">
-        <v>6940.94</v>
+        <v>6939.6</v>
       </c>
       <c r="N32" s="12" t="n">
-        <v>196.13</v>
+        <v>196.18</v>
       </c>
       <c r="O32" s="13" t="n">
-        <v>0.02907865455068416</v>
+        <v>0.02909206307778546</v>
       </c>
     </row>
     <row r="33">
@@ -9637,7 +9637,7 @@
         <v>46273</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C33" s="44" t="inlineStr">
         <is>
@@ -9645,40 +9645,40 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>48.3157</v>
+        <v>48.3158</v>
       </c>
       <c r="E33" s="8" t="n">
         <v>48.5196</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>0.2039</v>
+        <v>0.2038</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>0.004220160320558328</v>
+        <v>0.004218081869698939</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>56.0918</v>
+        <v>56.0882</v>
       </c>
       <c r="I33" s="10" t="n">
-        <v>56.3178</v>
+        <v>56.3142</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>0.226</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>0.00402910942419391</v>
+        <v>0.004029368031065358</v>
       </c>
       <c r="L33" s="12" t="n">
-        <v>6787.62</v>
+        <v>6787.5</v>
       </c>
       <c r="M33" s="12" t="n">
-        <v>6842.14</v>
+        <v>6842.02</v>
       </c>
       <c r="N33" s="12" t="n">
         <v>54.52</v>
       </c>
       <c r="O33" s="13" t="n">
-        <v>0.008032270516027709</v>
+        <v>0.008032412523020258</v>
       </c>
     </row>
     <row r="34">
@@ -9686,7 +9686,7 @@
         <v>46273</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C34" s="45" t="inlineStr">
         <is>
@@ -9706,28 +9706,28 @@
         <v>0.02014480116373686</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>55.783</v>
+        <v>55.7788</v>
       </c>
       <c r="I34" s="10" t="n">
-        <v>56.9021</v>
+        <v>56.8979</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>1.1191</v>
       </c>
       <c r="K34" s="11" t="n">
-        <v>0.02006166753311941</v>
+        <v>0.02006317812502241</v>
       </c>
       <c r="L34" s="12" t="n">
-        <v>6752.91</v>
+        <v>6753.13</v>
       </c>
       <c r="M34" s="12" t="n">
-        <v>6897.51</v>
+        <v>6897.73</v>
       </c>
       <c r="N34" s="12" t="n">
         <v>144.6</v>
       </c>
       <c r="O34" s="13" t="n">
-        <v>0.02141299084394728</v>
+        <v>0.0214122932625316</v>
       </c>
     </row>
     <row r="35">
@@ -9735,7 +9735,7 @@
         <v>46273</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C35" s="46" t="inlineStr">
         <is>
@@ -9743,28 +9743,28 @@
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>48.42</v>
+        <v>48.446</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>48.455</v>
+        <v>48.475</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.035</v>
+        <v>0.029</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>0.0007228418009087153</v>
+        <v>0.000598604631961359</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>56.08</v>
+        <v>56.102</v>
       </c>
       <c r="I35" s="10" t="n">
-        <v>56.198</v>
+        <v>56.216</v>
       </c>
       <c r="J35" s="10" t="n">
-        <v>0.118</v>
+        <v>0.114</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>0.00210413694721826</v>
+        <v>0.002032013118961891</v>
       </c>
       <c r="L35" s="12" t="n"/>
       <c r="M35" s="12" t="n"/>
@@ -9776,7 +9776,7 @@
         <v>46273</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C36" s="47" t="inlineStr">
         <is>
@@ -9796,28 +9796,28 @@
         <v>0.01880091915604763</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>55.59</v>
+        <v>55.58</v>
       </c>
       <c r="I36" s="10" t="n">
-        <v>56.61</v>
+        <v>56.6</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>1.02</v>
       </c>
       <c r="K36" s="11" t="n">
-        <v>0.01834862385321101</v>
+        <v>0.01835192515293271</v>
       </c>
       <c r="L36" s="12" t="n">
-        <v>6735.26</v>
+        <v>6735.94</v>
       </c>
       <c r="M36" s="12" t="n">
-        <v>6924.04</v>
+        <v>6925.57</v>
       </c>
       <c r="N36" s="12" t="n">
-        <v>188.78</v>
+        <v>189.63</v>
       </c>
       <c r="O36" s="13" t="n">
-        <v>0.02802861359472389</v>
+        <v>0.02815197285011446</v>
       </c>
     </row>
     <row r="37">
@@ -9825,7 +9825,7 @@
         <v>46273</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C37" s="48" t="inlineStr">
         <is>
@@ -9845,28 +9845,28 @@
         <v>0.02022821252942144</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>55.8018</v>
+        <v>55.7933</v>
       </c>
       <c r="I37" s="10" t="n">
-        <v>56.9306</v>
+        <v>56.9219</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1.1288</v>
+        <v>1.1286</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>0.02022873814106355</v>
+        <v>0.0202282352899004</v>
       </c>
       <c r="L37" s="12" t="n">
-        <v>6785.67</v>
+        <v>6782.05</v>
       </c>
       <c r="M37" s="12" t="n">
-        <v>6922.69</v>
+        <v>6918.98</v>
       </c>
       <c r="N37" s="12" t="n">
-        <v>137.02</v>
+        <v>136.93</v>
       </c>
       <c r="O37" s="13" t="n">
-        <v>0.02019255283560798</v>
+        <v>0.02019006052742165</v>
       </c>
     </row>
     <row r="38">
@@ -9874,7 +9874,7 @@
         <v>46273</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
@@ -9894,28 +9894,28 @@
         <v>0.01360296716410463</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>55.7907</v>
+        <v>55.786</v>
       </c>
       <c r="I38" s="10" t="n">
-        <v>56.6062</v>
+        <v>56.6016</v>
       </c>
       <c r="J38" s="10" t="n">
-        <v>0.8155</v>
+        <v>0.8156</v>
       </c>
       <c r="K38" s="11" t="n">
-        <v>0.01461713152908997</v>
+        <v>0.01462015559459363</v>
       </c>
       <c r="L38" s="12" t="n">
-        <v>6751.75</v>
+        <v>6755.68</v>
       </c>
       <c r="M38" s="12" t="n">
-        <v>6888.07</v>
+        <v>6892.09</v>
       </c>
       <c r="N38" s="12" t="n">
-        <v>136.32</v>
+        <v>136.41</v>
       </c>
       <c r="O38" s="13" t="n">
-        <v>0.02019032102788166</v>
+        <v>0.02019189778083035</v>
       </c>
     </row>
     <row r="39">
@@ -9923,7 +9923,7 @@
         <v>46273</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="C39" s="50" t="inlineStr">
         <is>
@@ -9931,40 +9931,40 @@
         </is>
       </c>
       <c r="D39" s="8" t="n">
-        <v>47.9291</v>
+        <v>47.9295</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>48.9295</v>
+        <v>48.9294</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>1.0004</v>
+        <v>0.9999</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>0.02087249708423484</v>
+        <v>0.0208618909022627</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>55.6136</v>
+        <v>55.6107</v>
       </c>
       <c r="I39" s="10" t="n">
-        <v>56.8305</v>
+        <v>56.8265</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1.2169</v>
+        <v>1.2158</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>0.02188133837766302</v>
+        <v>0.02186269908488834</v>
       </c>
       <c r="L39" s="12" t="n">
-        <v>6773.96</v>
+        <v>6777.13</v>
       </c>
       <c r="M39" s="12" t="n">
-        <v>6989.02</v>
+        <v>6992.17</v>
       </c>
       <c r="N39" s="12" t="n">
-        <v>215.06</v>
+        <v>215.04</v>
       </c>
       <c r="O39" s="13" t="n">
-        <v>0.03174804693266568</v>
+        <v>0.0317302456939737</v>
       </c>
     </row>
   </sheetData>
@@ -76314,7 +76314,7 @@
       </c>
       <c r="B5" s="62" t="n"/>
       <c r="C5" s="64" t="n">
-        <v>0.5463078703703703</v>
+        <v>0.5962037037037037</v>
       </c>
       <c r="D5" s="62" t="n"/>
       <c r="F5" s="62" t="inlineStr">
@@ -76398,7 +76398,7 @@
         <v>5</v>
       </c>
       <c r="N6" s="70" t="n">
-        <v>0.01834862385321101</v>
+        <v>0.01835192515293271</v>
       </c>
       <c r="O6" s="71" t="inlineStr">
         <is>
@@ -76406,10 +76406,10 @@
         </is>
       </c>
       <c r="P6" s="72" t="n">
-        <v>55.59</v>
+        <v>55.58</v>
       </c>
       <c r="Q6" s="72" t="n">
-        <v>56.61</v>
+        <v>56.6</v>
       </c>
     </row>
     <row r="7">
@@ -76451,7 +76451,7 @@
         <v>5</v>
       </c>
       <c r="N7" s="70" t="n">
-        <v>0.02019255283560798</v>
+        <v>0.02019006052742165</v>
       </c>
       <c r="O7" s="77" t="inlineStr">
         <is>
@@ -76459,10 +76459,10 @@
         </is>
       </c>
       <c r="P7" s="72" t="n">
-        <v>6785.67</v>
+        <v>6782.05</v>
       </c>
       <c r="Q7" s="72" t="n">
-        <v>6922.69</v>
+        <v>6918.98</v>
       </c>
     </row>
     <row r="8">

</xml_diff>